<commit_message>
update templated issued at
</commit_message>
<xml_diff>
--- a/public/assets/templates/template_kalibrasi_jangka_sorong_sertifikat.xlsx
+++ b/public/assets/templates/template_kalibrasi_jangka_sorong_sertifikat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2BB3758-9CA2-457F-82BA-1D2877218C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C2900C1-308F-4800-A6E7-7AB850E3A8F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{12CE2AE1-1EA9-4BA9-947C-BB59CA2A4E03}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="51">
   <si>
     <t>SERTIFIKAT KALIBRASI INTERNAL DIMENSI</t>
   </si>
@@ -167,9 +167,6 @@
   </si>
   <si>
     <t>Diterima oleh :</t>
-  </si>
-  <si>
-    <t>Diterbitkan tanggal : 17/03/2025</t>
   </si>
   <si>
     <r>
@@ -771,9 +768,141 @@
     <xf numFmtId="167" fontId="6" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -783,6 +912,69 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
@@ -792,18 +984,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -816,194 +999,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1907,214 +1904,214 @@
   <sheetData>
     <row r="1" spans="2:39" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:39" ht="19" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="102"/>
-      <c r="C2" s="103"/>
-      <c r="D2" s="103"/>
-      <c r="E2" s="103"/>
-      <c r="F2" s="103"/>
-      <c r="G2" s="104"/>
-      <c r="H2" s="109" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="110"/>
-      <c r="J2" s="110"/>
-      <c r="K2" s="110"/>
-      <c r="L2" s="110"/>
-      <c r="M2" s="110"/>
-      <c r="N2" s="110"/>
-      <c r="O2" s="110"/>
-      <c r="P2" s="110"/>
-      <c r="Q2" s="110"/>
-      <c r="R2" s="110"/>
-      <c r="S2" s="110"/>
-      <c r="T2" s="110"/>
-      <c r="U2" s="110"/>
-      <c r="V2" s="110"/>
-      <c r="W2" s="110"/>
-      <c r="X2" s="110"/>
-      <c r="Y2" s="110"/>
-      <c r="Z2" s="110"/>
-      <c r="AA2" s="110"/>
-      <c r="AB2" s="110"/>
-      <c r="AC2" s="110"/>
-      <c r="AD2" s="110"/>
-      <c r="AE2" s="110"/>
-      <c r="AF2" s="110"/>
-      <c r="AG2" s="110"/>
-      <c r="AH2" s="110"/>
-      <c r="AI2" s="110"/>
-      <c r="AJ2" s="111"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+      <c r="L2" s="52"/>
+      <c r="M2" s="52"/>
+      <c r="N2" s="52"/>
+      <c r="O2" s="52"/>
+      <c r="P2" s="52"/>
+      <c r="Q2" s="52"/>
+      <c r="R2" s="52"/>
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+      <c r="U2" s="52"/>
+      <c r="V2" s="52"/>
+      <c r="W2" s="52"/>
+      <c r="X2" s="52"/>
+      <c r="Y2" s="52"/>
+      <c r="Z2" s="52"/>
+      <c r="AA2" s="52"/>
+      <c r="AB2" s="52"/>
+      <c r="AC2" s="52"/>
+      <c r="AD2" s="52"/>
+      <c r="AE2" s="52"/>
+      <c r="AF2" s="52"/>
+      <c r="AG2" s="52"/>
+      <c r="AH2" s="52"/>
+      <c r="AI2" s="52"/>
+      <c r="AJ2" s="53"/>
     </row>
     <row r="3" spans="2:39" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="105"/>
+      <c r="B3" s="45"/>
       <c r="C3" s="46"/>
       <c r="D3" s="46"/>
       <c r="E3" s="46"/>
       <c r="F3" s="46"/>
       <c r="G3" s="47"/>
-      <c r="H3" s="112"/>
-      <c r="I3" s="112"/>
-      <c r="J3" s="112"/>
-      <c r="K3" s="112"/>
-      <c r="L3" s="112"/>
-      <c r="M3" s="112"/>
-      <c r="N3" s="112"/>
-      <c r="O3" s="112"/>
-      <c r="P3" s="112"/>
-      <c r="Q3" s="112"/>
-      <c r="R3" s="112"/>
-      <c r="S3" s="112"/>
-      <c r="T3" s="112"/>
-      <c r="U3" s="112"/>
-      <c r="V3" s="112"/>
-      <c r="W3" s="112"/>
-      <c r="X3" s="112"/>
-      <c r="Y3" s="112"/>
-      <c r="Z3" s="112"/>
-      <c r="AA3" s="112"/>
-      <c r="AB3" s="112"/>
-      <c r="AC3" s="112"/>
-      <c r="AD3" s="112"/>
-      <c r="AE3" s="112"/>
-      <c r="AF3" s="112"/>
-      <c r="AG3" s="112"/>
-      <c r="AH3" s="112"/>
-      <c r="AI3" s="112"/>
-      <c r="AJ3" s="113"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54"/>
+      <c r="M3" s="54"/>
+      <c r="N3" s="54"/>
+      <c r="O3" s="54"/>
+      <c r="P3" s="54"/>
+      <c r="Q3" s="54"/>
+      <c r="R3" s="54"/>
+      <c r="S3" s="54"/>
+      <c r="T3" s="54"/>
+      <c r="U3" s="54"/>
+      <c r="V3" s="54"/>
+      <c r="W3" s="54"/>
+      <c r="X3" s="54"/>
+      <c r="Y3" s="54"/>
+      <c r="Z3" s="54"/>
+      <c r="AA3" s="54"/>
+      <c r="AB3" s="54"/>
+      <c r="AC3" s="54"/>
+      <c r="AD3" s="54"/>
+      <c r="AE3" s="54"/>
+      <c r="AF3" s="54"/>
+      <c r="AG3" s="54"/>
+      <c r="AH3" s="54"/>
+      <c r="AI3" s="54"/>
+      <c r="AJ3" s="55"/>
     </row>
     <row r="4" spans="2:39" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="105"/>
+      <c r="B4" s="45"/>
       <c r="C4" s="46"/>
       <c r="D4" s="46"/>
       <c r="E4" s="46"/>
       <c r="F4" s="46"/>
       <c r="G4" s="47"/>
-      <c r="H4" s="112"/>
-      <c r="I4" s="112"/>
-      <c r="J4" s="112"/>
-      <c r="K4" s="112"/>
-      <c r="L4" s="112"/>
-      <c r="M4" s="112"/>
-      <c r="N4" s="112"/>
-      <c r="O4" s="112"/>
-      <c r="P4" s="112"/>
-      <c r="Q4" s="112"/>
-      <c r="R4" s="112"/>
-      <c r="S4" s="112"/>
-      <c r="T4" s="112"/>
-      <c r="U4" s="112"/>
-      <c r="V4" s="112"/>
-      <c r="W4" s="112"/>
-      <c r="X4" s="112"/>
-      <c r="Y4" s="112"/>
-      <c r="Z4" s="112"/>
-      <c r="AA4" s="112"/>
-      <c r="AB4" s="112"/>
-      <c r="AC4" s="112"/>
-      <c r="AD4" s="112"/>
-      <c r="AE4" s="112"/>
-      <c r="AF4" s="112"/>
-      <c r="AG4" s="112"/>
-      <c r="AH4" s="112"/>
-      <c r="AI4" s="112"/>
-      <c r="AJ4" s="113"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54"/>
+      <c r="K4" s="54"/>
+      <c r="L4" s="54"/>
+      <c r="M4" s="54"/>
+      <c r="N4" s="54"/>
+      <c r="O4" s="54"/>
+      <c r="P4" s="54"/>
+      <c r="Q4" s="54"/>
+      <c r="R4" s="54"/>
+      <c r="S4" s="54"/>
+      <c r="T4" s="54"/>
+      <c r="U4" s="54"/>
+      <c r="V4" s="54"/>
+      <c r="W4" s="54"/>
+      <c r="X4" s="54"/>
+      <c r="Y4" s="54"/>
+      <c r="Z4" s="54"/>
+      <c r="AA4" s="54"/>
+      <c r="AB4" s="54"/>
+      <c r="AC4" s="54"/>
+      <c r="AD4" s="54"/>
+      <c r="AE4" s="54"/>
+      <c r="AF4" s="54"/>
+      <c r="AG4" s="54"/>
+      <c r="AH4" s="54"/>
+      <c r="AI4" s="54"/>
+      <c r="AJ4" s="55"/>
     </row>
     <row r="5" spans="2:39" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="106"/>
-      <c r="C5" s="107"/>
-      <c r="D5" s="107"/>
-      <c r="E5" s="107"/>
-      <c r="F5" s="107"/>
-      <c r="G5" s="108"/>
-      <c r="H5" s="114"/>
-      <c r="I5" s="114"/>
-      <c r="J5" s="114"/>
-      <c r="K5" s="114"/>
-      <c r="L5" s="114"/>
-      <c r="M5" s="114"/>
-      <c r="N5" s="114"/>
-      <c r="O5" s="114"/>
-      <c r="P5" s="114"/>
-      <c r="Q5" s="114"/>
-      <c r="R5" s="114"/>
-      <c r="S5" s="114"/>
-      <c r="T5" s="114"/>
-      <c r="U5" s="114"/>
-      <c r="V5" s="114"/>
-      <c r="W5" s="114"/>
-      <c r="X5" s="114"/>
-      <c r="Y5" s="114"/>
-      <c r="Z5" s="114"/>
-      <c r="AA5" s="114"/>
-      <c r="AB5" s="114"/>
-      <c r="AC5" s="114"/>
-      <c r="AD5" s="114"/>
-      <c r="AE5" s="114"/>
-      <c r="AF5" s="114"/>
-      <c r="AG5" s="114"/>
-      <c r="AH5" s="114"/>
-      <c r="AI5" s="114"/>
-      <c r="AJ5" s="115"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="56"/>
+      <c r="K5" s="56"/>
+      <c r="L5" s="56"/>
+      <c r="M5" s="56"/>
+      <c r="N5" s="56"/>
+      <c r="O5" s="56"/>
+      <c r="P5" s="56"/>
+      <c r="Q5" s="56"/>
+      <c r="R5" s="56"/>
+      <c r="S5" s="56"/>
+      <c r="T5" s="56"/>
+      <c r="U5" s="56"/>
+      <c r="V5" s="56"/>
+      <c r="W5" s="56"/>
+      <c r="X5" s="56"/>
+      <c r="Y5" s="56"/>
+      <c r="Z5" s="56"/>
+      <c r="AA5" s="56"/>
+      <c r="AB5" s="56"/>
+      <c r="AC5" s="56"/>
+      <c r="AD5" s="56"/>
+      <c r="AE5" s="56"/>
+      <c r="AF5" s="56"/>
+      <c r="AG5" s="56"/>
+      <c r="AH5" s="56"/>
+      <c r="AI5" s="56"/>
+      <c r="AJ5" s="57"/>
     </row>
     <row r="6" spans="2:39" ht="3" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="106"/>
-      <c r="C6" s="107"/>
-      <c r="D6" s="107"/>
-      <c r="E6" s="107"/>
-      <c r="F6" s="107"/>
-      <c r="G6" s="107"/>
-      <c r="H6" s="107"/>
-      <c r="I6" s="107"/>
-      <c r="J6" s="107"/>
-      <c r="K6" s="107"/>
-      <c r="L6" s="107"/>
-      <c r="M6" s="107"/>
-      <c r="N6" s="107"/>
-      <c r="O6" s="107"/>
-      <c r="P6" s="107"/>
-      <c r="Q6" s="107"/>
-      <c r="R6" s="107"/>
-      <c r="S6" s="107"/>
-      <c r="T6" s="107"/>
-      <c r="U6" s="107"/>
-      <c r="V6" s="107"/>
-      <c r="W6" s="107"/>
-      <c r="X6" s="107"/>
-      <c r="Y6" s="107"/>
-      <c r="Z6" s="107"/>
-      <c r="AA6" s="107"/>
-      <c r="AB6" s="107"/>
-      <c r="AC6" s="107"/>
-      <c r="AD6" s="107"/>
-      <c r="AE6" s="107"/>
-      <c r="AF6" s="107"/>
-      <c r="AG6" s="107"/>
-      <c r="AH6" s="107"/>
-      <c r="AI6" s="107"/>
-      <c r="AJ6" s="116"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="49"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="49"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="49"/>
+      <c r="I6" s="49"/>
+      <c r="J6" s="49"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="49"/>
+      <c r="M6" s="49"/>
+      <c r="N6" s="49"/>
+      <c r="O6" s="49"/>
+      <c r="P6" s="49"/>
+      <c r="Q6" s="49"/>
+      <c r="R6" s="49"/>
+      <c r="S6" s="49"/>
+      <c r="T6" s="49"/>
+      <c r="U6" s="49"/>
+      <c r="V6" s="49"/>
+      <c r="W6" s="49"/>
+      <c r="X6" s="49"/>
+      <c r="Y6" s="49"/>
+      <c r="Z6" s="49"/>
+      <c r="AA6" s="49"/>
+      <c r="AB6" s="49"/>
+      <c r="AC6" s="49"/>
+      <c r="AD6" s="49"/>
+      <c r="AE6" s="49"/>
+      <c r="AF6" s="49"/>
+      <c r="AG6" s="49"/>
+      <c r="AH6" s="49"/>
+      <c r="AI6" s="49"/>
+      <c r="AJ6" s="58"/>
     </row>
     <row r="7" spans="2:39" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="96" t="s">
+      <c r="B7" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="97"/>
-      <c r="D7" s="97"/>
-      <c r="E7" s="97"/>
-      <c r="F7" s="97"/>
-      <c r="G7" s="97"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="40"/>
       <c r="H7" s="4" t="s">
         <v>2</v>
       </c>
       <c r="I7" s="5"/>
-      <c r="S7" s="98" t="s">
+      <c r="S7" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="T7" s="98"/>
-      <c r="U7" s="98"/>
-      <c r="V7" s="98"/>
-      <c r="W7" s="98"/>
-      <c r="X7" s="98"/>
-      <c r="Y7" s="98"/>
+      <c r="T7" s="41"/>
+      <c r="U7" s="41"/>
+      <c r="V7" s="41"/>
+      <c r="W7" s="41"/>
+      <c r="X7" s="41"/>
+      <c r="Y7" s="41"/>
       <c r="Z7" s="6" t="s">
         <v>2</v>
       </c>
@@ -2129,26 +2126,26 @@
       <c r="AJ7" s="8"/>
     </row>
     <row r="8" spans="2:39" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="96" t="s">
+      <c r="B8" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="97"/>
-      <c r="D8" s="97"/>
-      <c r="E8" s="97"/>
-      <c r="F8" s="97"/>
-      <c r="G8" s="97"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
       <c r="H8" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="S8" s="98" t="s">
+      <c r="S8" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="T8" s="98"/>
-      <c r="U8" s="98"/>
-      <c r="V8" s="98"/>
-      <c r="W8" s="98"/>
-      <c r="X8" s="98"/>
-      <c r="Y8" s="98"/>
+      <c r="T8" s="41"/>
+      <c r="U8" s="41"/>
+      <c r="V8" s="41"/>
+      <c r="W8" s="41"/>
+      <c r="X8" s="41"/>
+      <c r="Y8" s="41"/>
       <c r="Z8" s="6" t="s">
         <v>2</v>
       </c>
@@ -2163,26 +2160,26 @@
       <c r="AJ8" s="8"/>
     </row>
     <row r="9" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B9" s="96" t="s">
+      <c r="B9" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="97"/>
-      <c r="D9" s="97"/>
-      <c r="E9" s="97"/>
-      <c r="F9" s="97"/>
-      <c r="G9" s="97"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="40"/>
+      <c r="E9" s="40"/>
+      <c r="F9" s="40"/>
+      <c r="G9" s="40"/>
       <c r="H9" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="S9" s="97" t="s">
+      <c r="S9" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="T9" s="97"/>
-      <c r="U9" s="97"/>
-      <c r="V9" s="97"/>
-      <c r="W9" s="97"/>
-      <c r="X9" s="97"/>
-      <c r="Y9" s="97"/>
+      <c r="T9" s="40"/>
+      <c r="U9" s="40"/>
+      <c r="V9" s="40"/>
+      <c r="W9" s="40"/>
+      <c r="X9" s="40"/>
+      <c r="Y9" s="40"/>
       <c r="Z9" s="6" t="s">
         <v>2</v>
       </c>
@@ -2200,26 +2197,26 @@
       <c r="AM9" s="11"/>
     </row>
     <row r="10" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B10" s="100" t="s">
+      <c r="B10" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="101"/>
-      <c r="D10" s="101"/>
-      <c r="E10" s="101"/>
-      <c r="F10" s="101"/>
-      <c r="G10" s="101"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60"/>
       <c r="H10" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="S10" s="98" t="s">
+      <c r="S10" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="T10" s="98"/>
-      <c r="U10" s="98"/>
-      <c r="V10" s="98"/>
-      <c r="W10" s="98"/>
-      <c r="X10" s="98"/>
-      <c r="Y10" s="98"/>
+      <c r="T10" s="41"/>
+      <c r="U10" s="41"/>
+      <c r="V10" s="41"/>
+      <c r="W10" s="41"/>
+      <c r="X10" s="41"/>
+      <c r="Y10" s="41"/>
       <c r="Z10" s="6" t="s">
         <v>2</v>
       </c>
@@ -2238,26 +2235,26 @@
       <c r="AM10" s="11"/>
     </row>
     <row r="11" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B11" s="96" t="s">
+      <c r="B11" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="97"/>
-      <c r="D11" s="97"/>
-      <c r="E11" s="97"/>
-      <c r="F11" s="97"/>
-      <c r="G11" s="97"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
       <c r="H11" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="S11" s="98" t="s">
+      <c r="S11" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="T11" s="98"/>
-      <c r="U11" s="98"/>
-      <c r="V11" s="98"/>
-      <c r="W11" s="98"/>
-      <c r="X11" s="98"/>
-      <c r="Y11" s="98"/>
+      <c r="T11" s="41"/>
+      <c r="U11" s="41"/>
+      <c r="V11" s="41"/>
+      <c r="W11" s="41"/>
+      <c r="X11" s="41"/>
+      <c r="Y11" s="41"/>
       <c r="Z11" s="6" t="s">
         <v>2</v>
       </c>
@@ -2276,54 +2273,54 @@
       <c r="AM11" s="11"/>
     </row>
     <row r="12" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B12" s="96" t="s">
+      <c r="B12" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="97"/>
-      <c r="D12" s="97"/>
-      <c r="E12" s="97"/>
-      <c r="F12" s="97"/>
-      <c r="G12" s="97"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
       <c r="H12" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="S12" s="98" t="s">
+      <c r="S12" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="T12" s="98"/>
-      <c r="U12" s="98"/>
-      <c r="V12" s="98"/>
-      <c r="W12" s="98"/>
-      <c r="X12" s="98"/>
-      <c r="Y12" s="98"/>
+      <c r="T12" s="41"/>
+      <c r="U12" s="41"/>
+      <c r="V12" s="41"/>
+      <c r="W12" s="41"/>
+      <c r="X12" s="41"/>
+      <c r="Y12" s="41"/>
       <c r="Z12" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="AA12" s="99" t="s">
+      <c r="AA12" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="AB12" s="99"/>
-      <c r="AC12" s="99"/>
-      <c r="AD12" s="99"/>
-      <c r="AE12" s="99"/>
-      <c r="AF12" s="99"/>
-      <c r="AG12" s="99"/>
-      <c r="AH12" s="99"/>
-      <c r="AI12" s="99"/>
+      <c r="AB12" s="61"/>
+      <c r="AC12" s="61"/>
+      <c r="AD12" s="61"/>
+      <c r="AE12" s="61"/>
+      <c r="AF12" s="61"/>
+      <c r="AG12" s="61"/>
+      <c r="AH12" s="61"/>
+      <c r="AI12" s="61"/>
       <c r="AJ12" s="10"/>
       <c r="AK12" s="11"/>
       <c r="AL12" s="11"/>
       <c r="AM12" s="11"/>
     </row>
     <row r="13" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B13" s="96" t="s">
+      <c r="B13" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="97"/>
-      <c r="D13" s="97"/>
-      <c r="E13" s="97"/>
-      <c r="F13" s="97"/>
-      <c r="G13" s="97"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="40"/>
       <c r="H13" s="4" t="s">
         <v>2</v>
       </c>
@@ -2335,151 +2332,151 @@
       <c r="X13" s="7"/>
       <c r="Y13" s="7"/>
       <c r="Z13" s="14"/>
-      <c r="AA13" s="99"/>
-      <c r="AB13" s="99"/>
-      <c r="AC13" s="99"/>
-      <c r="AD13" s="99"/>
-      <c r="AE13" s="99"/>
-      <c r="AF13" s="99"/>
-      <c r="AG13" s="99"/>
-      <c r="AH13" s="99"/>
-      <c r="AI13" s="99"/>
+      <c r="AA13" s="61"/>
+      <c r="AB13" s="61"/>
+      <c r="AC13" s="61"/>
+      <c r="AD13" s="61"/>
+      <c r="AE13" s="61"/>
+      <c r="AF13" s="61"/>
+      <c r="AG13" s="61"/>
+      <c r="AH13" s="61"/>
+      <c r="AI13" s="61"/>
       <c r="AJ13" s="10"/>
       <c r="AK13" s="11"/>
       <c r="AL13" s="11"/>
       <c r="AM13" s="11"/>
     </row>
     <row r="14" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B14" s="96" t="s">
+      <c r="B14" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="97"/>
-      <c r="D14" s="97"/>
-      <c r="E14" s="97"/>
-      <c r="F14" s="97"/>
-      <c r="G14" s="97"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="40"/>
       <c r="H14" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="AA14" s="99"/>
-      <c r="AB14" s="99"/>
-      <c r="AC14" s="99"/>
-      <c r="AD14" s="99"/>
-      <c r="AE14" s="99"/>
-      <c r="AF14" s="99"/>
-      <c r="AG14" s="99"/>
-      <c r="AH14" s="99"/>
-      <c r="AI14" s="99"/>
+      <c r="AA14" s="61"/>
+      <c r="AB14" s="61"/>
+      <c r="AC14" s="61"/>
+      <c r="AD14" s="61"/>
+      <c r="AE14" s="61"/>
+      <c r="AF14" s="61"/>
+      <c r="AG14" s="61"/>
+      <c r="AH14" s="61"/>
+      <c r="AI14" s="61"/>
       <c r="AJ14" s="10"/>
       <c r="AK14" s="15"/>
       <c r="AL14" s="15"/>
       <c r="AM14" s="15"/>
     </row>
     <row r="15" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B15" s="96" t="s">
+      <c r="B15" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="97"/>
-      <c r="D15" s="97"/>
-      <c r="E15" s="97"/>
-      <c r="F15" s="97"/>
-      <c r="G15" s="97"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="40"/>
       <c r="H15" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="AA15" s="99"/>
-      <c r="AB15" s="99"/>
-      <c r="AC15" s="99"/>
-      <c r="AD15" s="99"/>
-      <c r="AE15" s="99"/>
-      <c r="AF15" s="99"/>
-      <c r="AG15" s="99"/>
-      <c r="AH15" s="99"/>
-      <c r="AI15" s="99"/>
+      <c r="AA15" s="61"/>
+      <c r="AB15" s="61"/>
+      <c r="AC15" s="61"/>
+      <c r="AD15" s="61"/>
+      <c r="AE15" s="61"/>
+      <c r="AF15" s="61"/>
+      <c r="AG15" s="61"/>
+      <c r="AH15" s="61"/>
+      <c r="AI15" s="61"/>
       <c r="AJ15" s="8"/>
     </row>
     <row r="16" spans="2:39" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="96" t="s">
+      <c r="B16" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="97"/>
-      <c r="D16" s="97"/>
-      <c r="E16" s="97"/>
-      <c r="F16" s="97"/>
-      <c r="G16" s="97"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="40"/>
       <c r="H16" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="AA16" s="99"/>
-      <c r="AB16" s="99"/>
-      <c r="AC16" s="99"/>
-      <c r="AD16" s="99"/>
-      <c r="AE16" s="99"/>
-      <c r="AF16" s="99"/>
-      <c r="AG16" s="99"/>
-      <c r="AH16" s="99"/>
-      <c r="AI16" s="99"/>
+      <c r="AA16" s="61"/>
+      <c r="AB16" s="61"/>
+      <c r="AC16" s="61"/>
+      <c r="AD16" s="61"/>
+      <c r="AE16" s="61"/>
+      <c r="AF16" s="61"/>
+      <c r="AG16" s="61"/>
+      <c r="AH16" s="61"/>
+      <c r="AI16" s="61"/>
       <c r="AJ16" s="8"/>
     </row>
     <row r="17" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B17" s="96" t="s">
+      <c r="B17" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="97"/>
-      <c r="D17" s="97"/>
-      <c r="E17" s="97"/>
-      <c r="F17" s="97"/>
-      <c r="G17" s="97"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="40"/>
       <c r="H17" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="AA17" s="99"/>
-      <c r="AB17" s="99"/>
-      <c r="AC17" s="99"/>
-      <c r="AD17" s="99"/>
-      <c r="AE17" s="99"/>
-      <c r="AF17" s="99"/>
-      <c r="AG17" s="99"/>
-      <c r="AH17" s="99"/>
-      <c r="AI17" s="99"/>
+      <c r="AA17" s="61"/>
+      <c r="AB17" s="61"/>
+      <c r="AC17" s="61"/>
+      <c r="AD17" s="61"/>
+      <c r="AE17" s="61"/>
+      <c r="AF17" s="61"/>
+      <c r="AG17" s="61"/>
+      <c r="AH17" s="61"/>
+      <c r="AI17" s="61"/>
       <c r="AJ17" s="8"/>
     </row>
     <row r="18" spans="2:36" ht="3" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="79"/>
-      <c r="C18" s="80"/>
-      <c r="D18" s="80"/>
-      <c r="E18" s="80"/>
-      <c r="F18" s="80"/>
-      <c r="G18" s="80"/>
-      <c r="H18" s="80"/>
-      <c r="I18" s="80"/>
-      <c r="J18" s="80"/>
-      <c r="K18" s="80"/>
-      <c r="L18" s="80"/>
-      <c r="M18" s="80"/>
-      <c r="N18" s="80"/>
-      <c r="O18" s="80"/>
-      <c r="P18" s="80"/>
-      <c r="Q18" s="80"/>
-      <c r="R18" s="80"/>
-      <c r="S18" s="80"/>
-      <c r="T18" s="80"/>
-      <c r="U18" s="80"/>
-      <c r="V18" s="80"/>
-      <c r="W18" s="80"/>
-      <c r="X18" s="80"/>
-      <c r="Y18" s="80"/>
-      <c r="Z18" s="80"/>
-      <c r="AA18" s="80"/>
-      <c r="AB18" s="80"/>
-      <c r="AC18" s="80"/>
-      <c r="AD18" s="80"/>
-      <c r="AE18" s="80"/>
-      <c r="AF18" s="80"/>
-      <c r="AG18" s="80"/>
-      <c r="AH18" s="80"/>
-      <c r="AI18" s="80"/>
-      <c r="AJ18" s="81"/>
+      <c r="B18" s="62"/>
+      <c r="C18" s="63"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="63"/>
+      <c r="I18" s="63"/>
+      <c r="J18" s="63"/>
+      <c r="K18" s="63"/>
+      <c r="L18" s="63"/>
+      <c r="M18" s="63"/>
+      <c r="N18" s="63"/>
+      <c r="O18" s="63"/>
+      <c r="P18" s="63"/>
+      <c r="Q18" s="63"/>
+      <c r="R18" s="63"/>
+      <c r="S18" s="63"/>
+      <c r="T18" s="63"/>
+      <c r="U18" s="63"/>
+      <c r="V18" s="63"/>
+      <c r="W18" s="63"/>
+      <c r="X18" s="63"/>
+      <c r="Y18" s="63"/>
+      <c r="Z18" s="63"/>
+      <c r="AA18" s="63"/>
+      <c r="AB18" s="63"/>
+      <c r="AC18" s="63"/>
+      <c r="AD18" s="63"/>
+      <c r="AE18" s="63"/>
+      <c r="AF18" s="63"/>
+      <c r="AG18" s="63"/>
+      <c r="AH18" s="63"/>
+      <c r="AI18" s="63"/>
+      <c r="AJ18" s="64"/>
     </row>
     <row r="19" spans="2:36" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B19" s="2"/>
@@ -2497,14 +2494,14 @@
       <c r="N19" s="3"/>
       <c r="O19" s="3"/>
       <c r="P19" s="16"/>
-      <c r="Q19" s="82" t="s">
+      <c r="Q19" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="R19" s="83"/>
-      <c r="S19" s="83"/>
-      <c r="T19" s="83"/>
-      <c r="U19" s="83"/>
-      <c r="V19" s="83"/>
+      <c r="R19" s="66"/>
+      <c r="S19" s="66"/>
+      <c r="T19" s="66"/>
+      <c r="U19" s="66"/>
+      <c r="V19" s="66"/>
       <c r="W19" s="16"/>
       <c r="X19" s="3"/>
       <c r="Y19" s="3"/>
@@ -2526,209 +2523,209 @@
     </row>
     <row r="21" spans="2:36" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="18"/>
-      <c r="C21" s="84" t="s">
+      <c r="C21" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="D21" s="85" t="s">
+      <c r="D21" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="E21" s="86"/>
-      <c r="F21" s="86"/>
-      <c r="G21" s="86"/>
-      <c r="H21" s="86"/>
-      <c r="I21" s="86"/>
-      <c r="J21" s="86"/>
-      <c r="K21" s="87"/>
-      <c r="L21" s="94" t="s">
+      <c r="E21" s="71"/>
+      <c r="F21" s="71"/>
+      <c r="G21" s="71"/>
+      <c r="H21" s="71"/>
+      <c r="I21" s="71"/>
+      <c r="J21" s="71"/>
+      <c r="K21" s="72"/>
+      <c r="L21" s="79" t="s">
         <v>24</v>
       </c>
-      <c r="M21" s="94"/>
-      <c r="N21" s="94"/>
-      <c r="O21" s="94"/>
-      <c r="P21" s="94"/>
-      <c r="Q21" s="94"/>
-      <c r="R21" s="94" t="s">
+      <c r="M21" s="79"/>
+      <c r="N21" s="79"/>
+      <c r="O21" s="79"/>
+      <c r="P21" s="79"/>
+      <c r="Q21" s="79"/>
+      <c r="R21" s="79" t="s">
         <v>25</v>
       </c>
-      <c r="S21" s="94"/>
-      <c r="T21" s="94"/>
-      <c r="U21" s="94"/>
-      <c r="V21" s="94"/>
-      <c r="W21" s="94"/>
-      <c r="X21" s="95" t="s">
+      <c r="S21" s="79"/>
+      <c r="T21" s="79"/>
+      <c r="U21" s="79"/>
+      <c r="V21" s="79"/>
+      <c r="W21" s="79"/>
+      <c r="X21" s="80" t="s">
         <v>26</v>
       </c>
-      <c r="Y21" s="95"/>
-      <c r="Z21" s="95"/>
-      <c r="AA21" s="95"/>
-      <c r="AB21" s="95"/>
-      <c r="AC21" s="95"/>
-      <c r="AD21" s="85" t="s">
+      <c r="Y21" s="80"/>
+      <c r="Z21" s="80"/>
+      <c r="AA21" s="80"/>
+      <c r="AB21" s="80"/>
+      <c r="AC21" s="80"/>
+      <c r="AD21" s="70" t="s">
         <v>27</v>
       </c>
-      <c r="AE21" s="86"/>
-      <c r="AF21" s="86"/>
-      <c r="AG21" s="86"/>
-      <c r="AH21" s="86"/>
-      <c r="AI21" s="87"/>
+      <c r="AE21" s="71"/>
+      <c r="AF21" s="71"/>
+      <c r="AG21" s="71"/>
+      <c r="AH21" s="71"/>
+      <c r="AI21" s="72"/>
       <c r="AJ21" s="8"/>
     </row>
     <row r="22" spans="2:36" ht="3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="18"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="88"/>
-      <c r="E22" s="89"/>
-      <c r="F22" s="89"/>
-      <c r="G22" s="89"/>
-      <c r="H22" s="89"/>
-      <c r="I22" s="89"/>
-      <c r="J22" s="89"/>
-      <c r="K22" s="90"/>
-      <c r="L22" s="94"/>
-      <c r="M22" s="94"/>
-      <c r="N22" s="94"/>
-      <c r="O22" s="94"/>
-      <c r="P22" s="94"/>
-      <c r="Q22" s="94"/>
-      <c r="R22" s="94"/>
-      <c r="S22" s="94"/>
-      <c r="T22" s="94"/>
-      <c r="U22" s="94"/>
-      <c r="V22" s="94"/>
-      <c r="W22" s="94"/>
-      <c r="X22" s="95"/>
-      <c r="Y22" s="95"/>
-      <c r="Z22" s="95"/>
-      <c r="AA22" s="95"/>
-      <c r="AB22" s="95"/>
-      <c r="AC22" s="95"/>
-      <c r="AD22" s="88"/>
-      <c r="AE22" s="89"/>
-      <c r="AF22" s="89"/>
-      <c r="AG22" s="89"/>
-      <c r="AH22" s="89"/>
-      <c r="AI22" s="90"/>
+      <c r="C22" s="68"/>
+      <c r="D22" s="73"/>
+      <c r="E22" s="74"/>
+      <c r="F22" s="74"/>
+      <c r="G22" s="74"/>
+      <c r="H22" s="74"/>
+      <c r="I22" s="74"/>
+      <c r="J22" s="74"/>
+      <c r="K22" s="75"/>
+      <c r="L22" s="79"/>
+      <c r="M22" s="79"/>
+      <c r="N22" s="79"/>
+      <c r="O22" s="79"/>
+      <c r="P22" s="79"/>
+      <c r="Q22" s="79"/>
+      <c r="R22" s="79"/>
+      <c r="S22" s="79"/>
+      <c r="T22" s="79"/>
+      <c r="U22" s="79"/>
+      <c r="V22" s="79"/>
+      <c r="W22" s="79"/>
+      <c r="X22" s="80"/>
+      <c r="Y22" s="80"/>
+      <c r="Z22" s="80"/>
+      <c r="AA22" s="80"/>
+      <c r="AB22" s="80"/>
+      <c r="AC22" s="80"/>
+      <c r="AD22" s="73"/>
+      <c r="AE22" s="74"/>
+      <c r="AF22" s="74"/>
+      <c r="AG22" s="74"/>
+      <c r="AH22" s="74"/>
+      <c r="AI22" s="75"/>
       <c r="AJ22" s="8"/>
     </row>
     <row r="23" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="18"/>
-      <c r="C23" s="54"/>
-      <c r="D23" s="91"/>
-      <c r="E23" s="92"/>
-      <c r="F23" s="92"/>
-      <c r="G23" s="92"/>
-      <c r="H23" s="92"/>
-      <c r="I23" s="92"/>
-      <c r="J23" s="92"/>
-      <c r="K23" s="93"/>
-      <c r="L23" s="94"/>
-      <c r="M23" s="94"/>
-      <c r="N23" s="94"/>
-      <c r="O23" s="94"/>
-      <c r="P23" s="94"/>
-      <c r="Q23" s="94"/>
-      <c r="R23" s="94"/>
-      <c r="S23" s="94"/>
-      <c r="T23" s="94"/>
-      <c r="U23" s="94"/>
-      <c r="V23" s="94"/>
-      <c r="W23" s="94"/>
-      <c r="X23" s="95"/>
-      <c r="Y23" s="95"/>
-      <c r="Z23" s="95"/>
-      <c r="AA23" s="95"/>
-      <c r="AB23" s="95"/>
-      <c r="AC23" s="95"/>
-      <c r="AD23" s="88"/>
-      <c r="AE23" s="89"/>
-      <c r="AF23" s="89"/>
-      <c r="AG23" s="89"/>
-      <c r="AH23" s="89"/>
-      <c r="AI23" s="90"/>
+      <c r="C23" s="68"/>
+      <c r="D23" s="76"/>
+      <c r="E23" s="77"/>
+      <c r="F23" s="77"/>
+      <c r="G23" s="77"/>
+      <c r="H23" s="77"/>
+      <c r="I23" s="77"/>
+      <c r="J23" s="77"/>
+      <c r="K23" s="78"/>
+      <c r="L23" s="79"/>
+      <c r="M23" s="79"/>
+      <c r="N23" s="79"/>
+      <c r="O23" s="79"/>
+      <c r="P23" s="79"/>
+      <c r="Q23" s="79"/>
+      <c r="R23" s="79"/>
+      <c r="S23" s="79"/>
+      <c r="T23" s="79"/>
+      <c r="U23" s="79"/>
+      <c r="V23" s="79"/>
+      <c r="W23" s="79"/>
+      <c r="X23" s="80"/>
+      <c r="Y23" s="80"/>
+      <c r="Z23" s="80"/>
+      <c r="AA23" s="80"/>
+      <c r="AB23" s="80"/>
+      <c r="AC23" s="80"/>
+      <c r="AD23" s="73"/>
+      <c r="AE23" s="74"/>
+      <c r="AF23" s="74"/>
+      <c r="AG23" s="74"/>
+      <c r="AH23" s="74"/>
+      <c r="AI23" s="75"/>
       <c r="AJ23" s="8"/>
     </row>
     <row r="24" spans="2:36" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="18"/>
-      <c r="C24" s="54"/>
-      <c r="D24" s="67" t="s">
+      <c r="C24" s="68"/>
+      <c r="D24" s="81" t="s">
         <v>28</v>
       </c>
-      <c r="E24" s="68"/>
-      <c r="F24" s="68"/>
-      <c r="G24" s="68"/>
-      <c r="H24" s="68"/>
-      <c r="I24" s="68"/>
-      <c r="J24" s="68"/>
-      <c r="K24" s="69"/>
-      <c r="L24" s="67" t="s">
+      <c r="E24" s="82"/>
+      <c r="F24" s="82"/>
+      <c r="G24" s="82"/>
+      <c r="H24" s="82"/>
+      <c r="I24" s="82"/>
+      <c r="J24" s="82"/>
+      <c r="K24" s="83"/>
+      <c r="L24" s="81" t="s">
         <v>28</v>
       </c>
-      <c r="M24" s="68"/>
-      <c r="N24" s="68"/>
-      <c r="O24" s="68"/>
-      <c r="P24" s="68"/>
-      <c r="Q24" s="69"/>
-      <c r="R24" s="67" t="s">
+      <c r="M24" s="82"/>
+      <c r="N24" s="82"/>
+      <c r="O24" s="82"/>
+      <c r="P24" s="82"/>
+      <c r="Q24" s="83"/>
+      <c r="R24" s="81" t="s">
         <v>28</v>
       </c>
-      <c r="S24" s="68"/>
-      <c r="T24" s="68"/>
-      <c r="U24" s="68"/>
-      <c r="V24" s="68"/>
-      <c r="W24" s="69"/>
-      <c r="X24" s="67" t="s">
+      <c r="S24" s="82"/>
+      <c r="T24" s="82"/>
+      <c r="U24" s="82"/>
+      <c r="V24" s="82"/>
+      <c r="W24" s="83"/>
+      <c r="X24" s="81" t="s">
         <v>28</v>
       </c>
-      <c r="Y24" s="68"/>
-      <c r="Z24" s="68"/>
-      <c r="AA24" s="68"/>
-      <c r="AB24" s="68"/>
-      <c r="AC24" s="69"/>
-      <c r="AD24" s="88"/>
-      <c r="AE24" s="89"/>
-      <c r="AF24" s="89"/>
-      <c r="AG24" s="89"/>
-      <c r="AH24" s="89"/>
-      <c r="AI24" s="90"/>
+      <c r="Y24" s="82"/>
+      <c r="Z24" s="82"/>
+      <c r="AA24" s="82"/>
+      <c r="AB24" s="82"/>
+      <c r="AC24" s="83"/>
+      <c r="AD24" s="73"/>
+      <c r="AE24" s="74"/>
+      <c r="AF24" s="74"/>
+      <c r="AG24" s="74"/>
+      <c r="AH24" s="74"/>
+      <c r="AI24" s="75"/>
       <c r="AJ24" s="8"/>
     </row>
     <row r="25" spans="2:36" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="18"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="40"/>
-      <c r="E25" s="41"/>
-      <c r="F25" s="41"/>
-      <c r="G25" s="41"/>
-      <c r="H25" s="41"/>
-      <c r="I25" s="41"/>
-      <c r="J25" s="41"/>
-      <c r="K25" s="42"/>
-      <c r="L25" s="40"/>
-      <c r="M25" s="41"/>
-      <c r="N25" s="41"/>
-      <c r="O25" s="41"/>
-      <c r="P25" s="41"/>
-      <c r="Q25" s="42"/>
-      <c r="R25" s="40"/>
-      <c r="S25" s="41"/>
-      <c r="T25" s="41"/>
-      <c r="U25" s="41"/>
-      <c r="V25" s="41"/>
-      <c r="W25" s="42"/>
-      <c r="X25" s="40"/>
-      <c r="Y25" s="41"/>
-      <c r="Z25" s="41"/>
-      <c r="AA25" s="41"/>
-      <c r="AB25" s="41"/>
-      <c r="AC25" s="42"/>
-      <c r="AD25" s="40" t="s">
+      <c r="C25" s="69"/>
+      <c r="D25" s="84"/>
+      <c r="E25" s="85"/>
+      <c r="F25" s="85"/>
+      <c r="G25" s="85"/>
+      <c r="H25" s="85"/>
+      <c r="I25" s="85"/>
+      <c r="J25" s="85"/>
+      <c r="K25" s="86"/>
+      <c r="L25" s="84"/>
+      <c r="M25" s="85"/>
+      <c r="N25" s="85"/>
+      <c r="O25" s="85"/>
+      <c r="P25" s="85"/>
+      <c r="Q25" s="86"/>
+      <c r="R25" s="84"/>
+      <c r="S25" s="85"/>
+      <c r="T25" s="85"/>
+      <c r="U25" s="85"/>
+      <c r="V25" s="85"/>
+      <c r="W25" s="86"/>
+      <c r="X25" s="84"/>
+      <c r="Y25" s="85"/>
+      <c r="Z25" s="85"/>
+      <c r="AA25" s="85"/>
+      <c r="AB25" s="85"/>
+      <c r="AC25" s="86"/>
+      <c r="AD25" s="84" t="s">
         <v>28</v>
       </c>
-      <c r="AE25" s="41"/>
-      <c r="AF25" s="41"/>
-      <c r="AG25" s="41"/>
-      <c r="AH25" s="41"/>
-      <c r="AI25" s="42"/>
+      <c r="AE25" s="85"/>
+      <c r="AF25" s="85"/>
+      <c r="AG25" s="85"/>
+      <c r="AH25" s="85"/>
+      <c r="AI25" s="86"/>
       <c r="AJ25" s="8"/>
     </row>
     <row r="26" spans="2:36" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2736,32 +2733,32 @@
       <c r="C26" s="19">
         <v>1</v>
       </c>
-      <c r="D26" s="73"/>
-      <c r="E26" s="74"/>
-      <c r="F26" s="74"/>
-      <c r="G26" s="74"/>
-      <c r="H26" s="74"/>
-      <c r="I26" s="74"/>
-      <c r="J26" s="74"/>
-      <c r="K26" s="75"/>
-      <c r="L26" s="73"/>
-      <c r="M26" s="74"/>
-      <c r="N26" s="74"/>
-      <c r="O26" s="74"/>
-      <c r="P26" s="74"/>
-      <c r="Q26" s="75"/>
-      <c r="R26" s="73"/>
-      <c r="S26" s="74"/>
-      <c r="T26" s="74"/>
-      <c r="U26" s="74"/>
-      <c r="V26" s="74"/>
-      <c r="W26" s="75"/>
-      <c r="X26" s="76"/>
-      <c r="Y26" s="77"/>
-      <c r="Z26" s="77"/>
-      <c r="AA26" s="77"/>
-      <c r="AB26" s="77"/>
-      <c r="AC26" s="78"/>
+      <c r="D26" s="87"/>
+      <c r="E26" s="88"/>
+      <c r="F26" s="88"/>
+      <c r="G26" s="88"/>
+      <c r="H26" s="88"/>
+      <c r="I26" s="88"/>
+      <c r="J26" s="88"/>
+      <c r="K26" s="89"/>
+      <c r="L26" s="87"/>
+      <c r="M26" s="88"/>
+      <c r="N26" s="88"/>
+      <c r="O26" s="88"/>
+      <c r="P26" s="88"/>
+      <c r="Q26" s="89"/>
+      <c r="R26" s="87"/>
+      <c r="S26" s="88"/>
+      <c r="T26" s="88"/>
+      <c r="U26" s="88"/>
+      <c r="V26" s="88"/>
+      <c r="W26" s="89"/>
+      <c r="X26" s="90"/>
+      <c r="Y26" s="91"/>
+      <c r="Z26" s="91"/>
+      <c r="AA26" s="91"/>
+      <c r="AB26" s="91"/>
+      <c r="AC26" s="92"/>
       <c r="AD26" s="30"/>
       <c r="AE26" s="31"/>
       <c r="AF26" s="31"/>
@@ -2775,32 +2772,32 @@
       <c r="C27" s="19">
         <v>2</v>
       </c>
-      <c r="D27" s="73"/>
-      <c r="E27" s="74"/>
-      <c r="F27" s="74"/>
-      <c r="G27" s="74"/>
-      <c r="H27" s="74"/>
-      <c r="I27" s="74"/>
-      <c r="J27" s="74"/>
-      <c r="K27" s="75"/>
-      <c r="L27" s="73"/>
-      <c r="M27" s="74"/>
-      <c r="N27" s="74"/>
-      <c r="O27" s="74"/>
-      <c r="P27" s="74"/>
-      <c r="Q27" s="75"/>
-      <c r="R27" s="73"/>
-      <c r="S27" s="74"/>
-      <c r="T27" s="74"/>
-      <c r="U27" s="74"/>
-      <c r="V27" s="74"/>
-      <c r="W27" s="75"/>
-      <c r="X27" s="76"/>
-      <c r="Y27" s="77"/>
-      <c r="Z27" s="77"/>
-      <c r="AA27" s="77"/>
-      <c r="AB27" s="77"/>
-      <c r="AC27" s="78"/>
+      <c r="D27" s="87"/>
+      <c r="E27" s="88"/>
+      <c r="F27" s="88"/>
+      <c r="G27" s="88"/>
+      <c r="H27" s="88"/>
+      <c r="I27" s="88"/>
+      <c r="J27" s="88"/>
+      <c r="K27" s="89"/>
+      <c r="L27" s="87"/>
+      <c r="M27" s="88"/>
+      <c r="N27" s="88"/>
+      <c r="O27" s="88"/>
+      <c r="P27" s="88"/>
+      <c r="Q27" s="89"/>
+      <c r="R27" s="87"/>
+      <c r="S27" s="88"/>
+      <c r="T27" s="88"/>
+      <c r="U27" s="88"/>
+      <c r="V27" s="88"/>
+      <c r="W27" s="89"/>
+      <c r="X27" s="90"/>
+      <c r="Y27" s="91"/>
+      <c r="Z27" s="91"/>
+      <c r="AA27" s="91"/>
+      <c r="AB27" s="91"/>
+      <c r="AC27" s="92"/>
       <c r="AD27" s="30"/>
       <c r="AE27" s="31"/>
       <c r="AF27" s="31"/>
@@ -2814,32 +2811,32 @@
       <c r="C28" s="19">
         <v>3</v>
       </c>
-      <c r="D28" s="73"/>
-      <c r="E28" s="74"/>
-      <c r="F28" s="74"/>
-      <c r="G28" s="74"/>
-      <c r="H28" s="74"/>
-      <c r="I28" s="74"/>
-      <c r="J28" s="74"/>
-      <c r="K28" s="75"/>
-      <c r="L28" s="73"/>
-      <c r="M28" s="74"/>
-      <c r="N28" s="74"/>
-      <c r="O28" s="74"/>
-      <c r="P28" s="74"/>
-      <c r="Q28" s="75"/>
-      <c r="R28" s="73"/>
-      <c r="S28" s="74"/>
-      <c r="T28" s="74"/>
-      <c r="U28" s="74"/>
-      <c r="V28" s="74"/>
-      <c r="W28" s="75"/>
-      <c r="X28" s="76"/>
-      <c r="Y28" s="77"/>
-      <c r="Z28" s="77"/>
-      <c r="AA28" s="77"/>
-      <c r="AB28" s="77"/>
-      <c r="AC28" s="78"/>
+      <c r="D28" s="87"/>
+      <c r="E28" s="88"/>
+      <c r="F28" s="88"/>
+      <c r="G28" s="88"/>
+      <c r="H28" s="88"/>
+      <c r="I28" s="88"/>
+      <c r="J28" s="88"/>
+      <c r="K28" s="89"/>
+      <c r="L28" s="87"/>
+      <c r="M28" s="88"/>
+      <c r="N28" s="88"/>
+      <c r="O28" s="88"/>
+      <c r="P28" s="88"/>
+      <c r="Q28" s="89"/>
+      <c r="R28" s="87"/>
+      <c r="S28" s="88"/>
+      <c r="T28" s="88"/>
+      <c r="U28" s="88"/>
+      <c r="V28" s="88"/>
+      <c r="W28" s="89"/>
+      <c r="X28" s="90"/>
+      <c r="Y28" s="91"/>
+      <c r="Z28" s="91"/>
+      <c r="AA28" s="91"/>
+      <c r="AB28" s="91"/>
+      <c r="AC28" s="92"/>
       <c r="AD28" s="30"/>
       <c r="AE28" s="31"/>
       <c r="AF28" s="31"/>
@@ -2853,32 +2850,32 @@
       <c r="C29" s="19">
         <v>4</v>
       </c>
-      <c r="D29" s="73"/>
-      <c r="E29" s="74"/>
-      <c r="F29" s="74"/>
-      <c r="G29" s="74"/>
-      <c r="H29" s="74"/>
-      <c r="I29" s="74"/>
-      <c r="J29" s="74"/>
-      <c r="K29" s="75"/>
-      <c r="L29" s="73"/>
-      <c r="M29" s="74"/>
-      <c r="N29" s="74"/>
-      <c r="O29" s="74"/>
-      <c r="P29" s="74"/>
-      <c r="Q29" s="75"/>
-      <c r="R29" s="73"/>
-      <c r="S29" s="74"/>
-      <c r="T29" s="74"/>
-      <c r="U29" s="74"/>
-      <c r="V29" s="74"/>
-      <c r="W29" s="75"/>
-      <c r="X29" s="76"/>
-      <c r="Y29" s="77"/>
-      <c r="Z29" s="77"/>
-      <c r="AA29" s="77"/>
-      <c r="AB29" s="77"/>
-      <c r="AC29" s="78"/>
+      <c r="D29" s="87"/>
+      <c r="E29" s="88"/>
+      <c r="F29" s="88"/>
+      <c r="G29" s="88"/>
+      <c r="H29" s="88"/>
+      <c r="I29" s="88"/>
+      <c r="J29" s="88"/>
+      <c r="K29" s="89"/>
+      <c r="L29" s="87"/>
+      <c r="M29" s="88"/>
+      <c r="N29" s="88"/>
+      <c r="O29" s="88"/>
+      <c r="P29" s="88"/>
+      <c r="Q29" s="89"/>
+      <c r="R29" s="87"/>
+      <c r="S29" s="88"/>
+      <c r="T29" s="88"/>
+      <c r="U29" s="88"/>
+      <c r="V29" s="88"/>
+      <c r="W29" s="89"/>
+      <c r="X29" s="90"/>
+      <c r="Y29" s="91"/>
+      <c r="Z29" s="91"/>
+      <c r="AA29" s="91"/>
+      <c r="AB29" s="91"/>
+      <c r="AC29" s="92"/>
       <c r="AD29" s="30"/>
       <c r="AE29" s="31"/>
       <c r="AF29" s="31"/>
@@ -2892,32 +2889,32 @@
       <c r="C30" s="19">
         <v>5</v>
       </c>
-      <c r="D30" s="73"/>
-      <c r="E30" s="74"/>
-      <c r="F30" s="74"/>
-      <c r="G30" s="74"/>
-      <c r="H30" s="74"/>
-      <c r="I30" s="74"/>
-      <c r="J30" s="74"/>
-      <c r="K30" s="75"/>
-      <c r="L30" s="73"/>
-      <c r="M30" s="74"/>
-      <c r="N30" s="74"/>
-      <c r="O30" s="74"/>
-      <c r="P30" s="74"/>
-      <c r="Q30" s="75"/>
-      <c r="R30" s="73"/>
-      <c r="S30" s="74"/>
-      <c r="T30" s="74"/>
-      <c r="U30" s="74"/>
-      <c r="V30" s="74"/>
-      <c r="W30" s="75"/>
-      <c r="X30" s="76"/>
-      <c r="Y30" s="77"/>
-      <c r="Z30" s="77"/>
-      <c r="AA30" s="77"/>
-      <c r="AB30" s="77"/>
-      <c r="AC30" s="78"/>
+      <c r="D30" s="87"/>
+      <c r="E30" s="88"/>
+      <c r="F30" s="88"/>
+      <c r="G30" s="88"/>
+      <c r="H30" s="88"/>
+      <c r="I30" s="88"/>
+      <c r="J30" s="88"/>
+      <c r="K30" s="89"/>
+      <c r="L30" s="87"/>
+      <c r="M30" s="88"/>
+      <c r="N30" s="88"/>
+      <c r="O30" s="88"/>
+      <c r="P30" s="88"/>
+      <c r="Q30" s="89"/>
+      <c r="R30" s="87"/>
+      <c r="S30" s="88"/>
+      <c r="T30" s="88"/>
+      <c r="U30" s="88"/>
+      <c r="V30" s="88"/>
+      <c r="W30" s="89"/>
+      <c r="X30" s="90"/>
+      <c r="Y30" s="91"/>
+      <c r="Z30" s="91"/>
+      <c r="AA30" s="91"/>
+      <c r="AB30" s="91"/>
+      <c r="AC30" s="92"/>
       <c r="AD30" s="27"/>
       <c r="AE30" s="28"/>
       <c r="AF30" s="28"/>
@@ -2931,32 +2928,32 @@
       <c r="C31" s="19">
         <v>6</v>
       </c>
-      <c r="D31" s="67"/>
-      <c r="E31" s="68"/>
-      <c r="F31" s="68"/>
-      <c r="G31" s="68"/>
-      <c r="H31" s="68"/>
-      <c r="I31" s="68"/>
-      <c r="J31" s="68"/>
-      <c r="K31" s="69"/>
-      <c r="L31" s="70"/>
-      <c r="M31" s="71"/>
-      <c r="N31" s="71"/>
-      <c r="O31" s="71"/>
-      <c r="P31" s="71"/>
-      <c r="Q31" s="72"/>
-      <c r="R31" s="70"/>
-      <c r="S31" s="71"/>
-      <c r="T31" s="71"/>
-      <c r="U31" s="71"/>
-      <c r="V31" s="71"/>
-      <c r="W31" s="72"/>
-      <c r="X31" s="70"/>
-      <c r="Y31" s="71"/>
-      <c r="Z31" s="71"/>
-      <c r="AA31" s="71"/>
-      <c r="AB31" s="71"/>
-      <c r="AC31" s="72"/>
+      <c r="D31" s="81"/>
+      <c r="E31" s="82"/>
+      <c r="F31" s="82"/>
+      <c r="G31" s="82"/>
+      <c r="H31" s="82"/>
+      <c r="I31" s="82"/>
+      <c r="J31" s="82"/>
+      <c r="K31" s="83"/>
+      <c r="L31" s="93"/>
+      <c r="M31" s="94"/>
+      <c r="N31" s="94"/>
+      <c r="O31" s="94"/>
+      <c r="P31" s="94"/>
+      <c r="Q31" s="95"/>
+      <c r="R31" s="93"/>
+      <c r="S31" s="94"/>
+      <c r="T31" s="94"/>
+      <c r="U31" s="94"/>
+      <c r="V31" s="94"/>
+      <c r="W31" s="95"/>
+      <c r="X31" s="93"/>
+      <c r="Y31" s="94"/>
+      <c r="Z31" s="94"/>
+      <c r="AA31" s="94"/>
+      <c r="AB31" s="94"/>
+      <c r="AC31" s="95"/>
       <c r="AD31" s="33"/>
       <c r="AE31" s="34"/>
       <c r="AF31" s="34"/>
@@ -2970,32 +2967,32 @@
       <c r="C32" s="19">
         <v>7</v>
       </c>
-      <c r="D32" s="67"/>
-      <c r="E32" s="68"/>
-      <c r="F32" s="68"/>
-      <c r="G32" s="68"/>
-      <c r="H32" s="68"/>
-      <c r="I32" s="68"/>
-      <c r="J32" s="68"/>
-      <c r="K32" s="69"/>
-      <c r="L32" s="70"/>
-      <c r="M32" s="71"/>
-      <c r="N32" s="71"/>
-      <c r="O32" s="71"/>
-      <c r="P32" s="71"/>
-      <c r="Q32" s="72"/>
-      <c r="R32" s="70"/>
-      <c r="S32" s="71"/>
-      <c r="T32" s="71"/>
-      <c r="U32" s="71"/>
-      <c r="V32" s="71"/>
-      <c r="W32" s="72"/>
-      <c r="X32" s="70"/>
-      <c r="Y32" s="71"/>
-      <c r="Z32" s="71"/>
-      <c r="AA32" s="71"/>
-      <c r="AB32" s="71"/>
-      <c r="AC32" s="72"/>
+      <c r="D32" s="81"/>
+      <c r="E32" s="82"/>
+      <c r="F32" s="82"/>
+      <c r="G32" s="82"/>
+      <c r="H32" s="82"/>
+      <c r="I32" s="82"/>
+      <c r="J32" s="82"/>
+      <c r="K32" s="83"/>
+      <c r="L32" s="93"/>
+      <c r="M32" s="94"/>
+      <c r="N32" s="94"/>
+      <c r="O32" s="94"/>
+      <c r="P32" s="94"/>
+      <c r="Q32" s="95"/>
+      <c r="R32" s="93"/>
+      <c r="S32" s="94"/>
+      <c r="T32" s="94"/>
+      <c r="U32" s="94"/>
+      <c r="V32" s="94"/>
+      <c r="W32" s="95"/>
+      <c r="X32" s="93"/>
+      <c r="Y32" s="94"/>
+      <c r="Z32" s="94"/>
+      <c r="AA32" s="94"/>
+      <c r="AB32" s="94"/>
+      <c r="AC32" s="95"/>
       <c r="AD32" s="36"/>
       <c r="AE32" s="37"/>
       <c r="AF32" s="37"/>
@@ -3006,337 +3003,337 @@
     </row>
     <row r="33" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="18"/>
-      <c r="C33" s="56" t="s">
+      <c r="C33" s="96" t="s">
         <v>29</v>
       </c>
-      <c r="D33" s="56"/>
-      <c r="E33" s="56"/>
-      <c r="F33" s="56"/>
-      <c r="G33" s="56"/>
-      <c r="H33" s="56"/>
-      <c r="I33" s="56"/>
-      <c r="J33" s="56"/>
-      <c r="K33" s="56"/>
-      <c r="L33" s="56"/>
-      <c r="M33" s="56"/>
-      <c r="N33" s="56"/>
-      <c r="O33" s="56"/>
-      <c r="P33" s="56"/>
-      <c r="Q33" s="56"/>
-      <c r="R33" s="56"/>
-      <c r="S33" s="56"/>
-      <c r="T33" s="56"/>
-      <c r="U33" s="56"/>
-      <c r="V33" s="56"/>
-      <c r="W33" s="56"/>
-      <c r="X33" s="56"/>
-      <c r="Y33" s="56"/>
-      <c r="Z33" s="56"/>
-      <c r="AA33" s="56"/>
-      <c r="AB33" s="56"/>
-      <c r="AC33" s="56"/>
-      <c r="AD33" s="56"/>
-      <c r="AE33" s="56"/>
-      <c r="AF33" s="56"/>
-      <c r="AG33" s="56"/>
-      <c r="AH33" s="56"/>
-      <c r="AI33" s="56"/>
+      <c r="D33" s="96"/>
+      <c r="E33" s="96"/>
+      <c r="F33" s="96"/>
+      <c r="G33" s="96"/>
+      <c r="H33" s="96"/>
+      <c r="I33" s="96"/>
+      <c r="J33" s="96"/>
+      <c r="K33" s="96"/>
+      <c r="L33" s="96"/>
+      <c r="M33" s="96"/>
+      <c r="N33" s="96"/>
+      <c r="O33" s="96"/>
+      <c r="P33" s="96"/>
+      <c r="Q33" s="96"/>
+      <c r="R33" s="96"/>
+      <c r="S33" s="96"/>
+      <c r="T33" s="96"/>
+      <c r="U33" s="96"/>
+      <c r="V33" s="96"/>
+      <c r="W33" s="96"/>
+      <c r="X33" s="96"/>
+      <c r="Y33" s="96"/>
+      <c r="Z33" s="96"/>
+      <c r="AA33" s="96"/>
+      <c r="AB33" s="96"/>
+      <c r="AC33" s="96"/>
+      <c r="AD33" s="96"/>
+      <c r="AE33" s="96"/>
+      <c r="AF33" s="96"/>
+      <c r="AG33" s="96"/>
+      <c r="AH33" s="96"/>
+      <c r="AI33" s="96"/>
       <c r="AJ33" s="8"/>
     </row>
     <row r="34" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="18"/>
-      <c r="C34" s="56"/>
-      <c r="D34" s="56"/>
-      <c r="E34" s="56"/>
-      <c r="F34" s="56"/>
-      <c r="G34" s="56"/>
-      <c r="H34" s="56"/>
-      <c r="I34" s="56"/>
-      <c r="J34" s="56"/>
-      <c r="K34" s="56"/>
-      <c r="L34" s="56"/>
-      <c r="M34" s="56"/>
-      <c r="N34" s="56"/>
-      <c r="O34" s="56"/>
-      <c r="P34" s="56"/>
-      <c r="Q34" s="56"/>
-      <c r="R34" s="56"/>
-      <c r="S34" s="56"/>
-      <c r="T34" s="56"/>
-      <c r="U34" s="56"/>
-      <c r="V34" s="56"/>
-      <c r="W34" s="56"/>
-      <c r="X34" s="56"/>
-      <c r="Y34" s="56"/>
-      <c r="Z34" s="56"/>
-      <c r="AA34" s="56"/>
-      <c r="AB34" s="56"/>
-      <c r="AC34" s="56"/>
-      <c r="AD34" s="56"/>
-      <c r="AE34" s="56"/>
-      <c r="AF34" s="56"/>
-      <c r="AG34" s="56"/>
-      <c r="AH34" s="56"/>
-      <c r="AI34" s="56"/>
+      <c r="C34" s="96"/>
+      <c r="D34" s="96"/>
+      <c r="E34" s="96"/>
+      <c r="F34" s="96"/>
+      <c r="G34" s="96"/>
+      <c r="H34" s="96"/>
+      <c r="I34" s="96"/>
+      <c r="J34" s="96"/>
+      <c r="K34" s="96"/>
+      <c r="L34" s="96"/>
+      <c r="M34" s="96"/>
+      <c r="N34" s="96"/>
+      <c r="O34" s="96"/>
+      <c r="P34" s="96"/>
+      <c r="Q34" s="96"/>
+      <c r="R34" s="96"/>
+      <c r="S34" s="96"/>
+      <c r="T34" s="96"/>
+      <c r="U34" s="96"/>
+      <c r="V34" s="96"/>
+      <c r="W34" s="96"/>
+      <c r="X34" s="96"/>
+      <c r="Y34" s="96"/>
+      <c r="Z34" s="96"/>
+      <c r="AA34" s="96"/>
+      <c r="AB34" s="96"/>
+      <c r="AC34" s="96"/>
+      <c r="AD34" s="96"/>
+      <c r="AE34" s="96"/>
+      <c r="AF34" s="96"/>
+      <c r="AG34" s="96"/>
+      <c r="AH34" s="96"/>
+      <c r="AI34" s="96"/>
       <c r="AJ34" s="8"/>
     </row>
     <row r="35" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="18"/>
-      <c r="C35" s="56"/>
-      <c r="D35" s="56"/>
-      <c r="E35" s="56"/>
-      <c r="F35" s="56"/>
-      <c r="G35" s="56"/>
-      <c r="H35" s="56"/>
-      <c r="I35" s="56"/>
-      <c r="J35" s="56"/>
-      <c r="K35" s="56"/>
-      <c r="L35" s="56"/>
-      <c r="M35" s="56"/>
-      <c r="N35" s="56"/>
-      <c r="O35" s="56"/>
-      <c r="P35" s="56"/>
-      <c r="Q35" s="56"/>
-      <c r="R35" s="56"/>
-      <c r="S35" s="56"/>
-      <c r="T35" s="56"/>
-      <c r="U35" s="56"/>
-      <c r="V35" s="56"/>
-      <c r="W35" s="56"/>
-      <c r="X35" s="56"/>
-      <c r="Y35" s="56"/>
-      <c r="Z35" s="56"/>
-      <c r="AA35" s="56"/>
-      <c r="AB35" s="56"/>
-      <c r="AC35" s="56"/>
-      <c r="AD35" s="56"/>
-      <c r="AE35" s="56"/>
-      <c r="AF35" s="56"/>
-      <c r="AG35" s="56"/>
-      <c r="AH35" s="56"/>
-      <c r="AI35" s="56"/>
+      <c r="C35" s="96"/>
+      <c r="D35" s="96"/>
+      <c r="E35" s="96"/>
+      <c r="F35" s="96"/>
+      <c r="G35" s="96"/>
+      <c r="H35" s="96"/>
+      <c r="I35" s="96"/>
+      <c r="J35" s="96"/>
+      <c r="K35" s="96"/>
+      <c r="L35" s="96"/>
+      <c r="M35" s="96"/>
+      <c r="N35" s="96"/>
+      <c r="O35" s="96"/>
+      <c r="P35" s="96"/>
+      <c r="Q35" s="96"/>
+      <c r="R35" s="96"/>
+      <c r="S35" s="96"/>
+      <c r="T35" s="96"/>
+      <c r="U35" s="96"/>
+      <c r="V35" s="96"/>
+      <c r="W35" s="96"/>
+      <c r="X35" s="96"/>
+      <c r="Y35" s="96"/>
+      <c r="Z35" s="96"/>
+      <c r="AA35" s="96"/>
+      <c r="AB35" s="96"/>
+      <c r="AC35" s="96"/>
+      <c r="AD35" s="96"/>
+      <c r="AE35" s="96"/>
+      <c r="AF35" s="96"/>
+      <c r="AG35" s="96"/>
+      <c r="AH35" s="96"/>
+      <c r="AI35" s="96"/>
       <c r="AJ35" s="8"/>
     </row>
     <row r="36" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="18"/>
-      <c r="C36" s="56"/>
-      <c r="D36" s="56"/>
-      <c r="E36" s="56"/>
-      <c r="F36" s="56"/>
-      <c r="G36" s="56"/>
-      <c r="H36" s="56"/>
-      <c r="I36" s="56"/>
-      <c r="J36" s="56"/>
-      <c r="K36" s="56"/>
-      <c r="L36" s="56"/>
-      <c r="M36" s="56"/>
-      <c r="N36" s="56"/>
-      <c r="O36" s="56"/>
-      <c r="P36" s="56"/>
-      <c r="Q36" s="56"/>
-      <c r="R36" s="56"/>
-      <c r="S36" s="56"/>
-      <c r="T36" s="56"/>
-      <c r="U36" s="56"/>
-      <c r="V36" s="56"/>
-      <c r="W36" s="56"/>
-      <c r="X36" s="56"/>
-      <c r="Y36" s="56"/>
-      <c r="Z36" s="56"/>
-      <c r="AA36" s="56"/>
-      <c r="AB36" s="56"/>
-      <c r="AC36" s="56"/>
-      <c r="AD36" s="56"/>
-      <c r="AE36" s="56"/>
-      <c r="AF36" s="56"/>
-      <c r="AG36" s="56"/>
-      <c r="AH36" s="56"/>
-      <c r="AI36" s="56"/>
+      <c r="C36" s="96"/>
+      <c r="D36" s="96"/>
+      <c r="E36" s="96"/>
+      <c r="F36" s="96"/>
+      <c r="G36" s="96"/>
+      <c r="H36" s="96"/>
+      <c r="I36" s="96"/>
+      <c r="J36" s="96"/>
+      <c r="K36" s="96"/>
+      <c r="L36" s="96"/>
+      <c r="M36" s="96"/>
+      <c r="N36" s="96"/>
+      <c r="O36" s="96"/>
+      <c r="P36" s="96"/>
+      <c r="Q36" s="96"/>
+      <c r="R36" s="96"/>
+      <c r="S36" s="96"/>
+      <c r="T36" s="96"/>
+      <c r="U36" s="96"/>
+      <c r="V36" s="96"/>
+      <c r="W36" s="96"/>
+      <c r="X36" s="96"/>
+      <c r="Y36" s="96"/>
+      <c r="Z36" s="96"/>
+      <c r="AA36" s="96"/>
+      <c r="AB36" s="96"/>
+      <c r="AC36" s="96"/>
+      <c r="AD36" s="96"/>
+      <c r="AE36" s="96"/>
+      <c r="AF36" s="96"/>
+      <c r="AG36" s="96"/>
+      <c r="AH36" s="96"/>
+      <c r="AI36" s="96"/>
       <c r="AJ36" s="8"/>
     </row>
     <row r="37" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="18"/>
-      <c r="C37" s="56"/>
-      <c r="D37" s="56"/>
-      <c r="E37" s="56"/>
-      <c r="F37" s="56"/>
-      <c r="G37" s="56"/>
-      <c r="H37" s="56"/>
-      <c r="I37" s="56"/>
-      <c r="J37" s="56"/>
-      <c r="K37" s="56"/>
-      <c r="L37" s="56"/>
-      <c r="M37" s="56"/>
-      <c r="N37" s="56"/>
-      <c r="O37" s="56"/>
-      <c r="P37" s="56"/>
-      <c r="Q37" s="56"/>
-      <c r="R37" s="56"/>
-      <c r="S37" s="56"/>
-      <c r="T37" s="56"/>
-      <c r="U37" s="56"/>
-      <c r="V37" s="56"/>
-      <c r="W37" s="56"/>
-      <c r="X37" s="56"/>
-      <c r="Y37" s="56"/>
-      <c r="Z37" s="56"/>
-      <c r="AA37" s="56"/>
-      <c r="AB37" s="56"/>
-      <c r="AC37" s="56"/>
-      <c r="AD37" s="56"/>
-      <c r="AE37" s="56"/>
-      <c r="AF37" s="56"/>
-      <c r="AG37" s="56"/>
-      <c r="AH37" s="56"/>
-      <c r="AI37" s="56"/>
+      <c r="C37" s="96"/>
+      <c r="D37" s="96"/>
+      <c r="E37" s="96"/>
+      <c r="F37" s="96"/>
+      <c r="G37" s="96"/>
+      <c r="H37" s="96"/>
+      <c r="I37" s="96"/>
+      <c r="J37" s="96"/>
+      <c r="K37" s="96"/>
+      <c r="L37" s="96"/>
+      <c r="M37" s="96"/>
+      <c r="N37" s="96"/>
+      <c r="O37" s="96"/>
+      <c r="P37" s="96"/>
+      <c r="Q37" s="96"/>
+      <c r="R37" s="96"/>
+      <c r="S37" s="96"/>
+      <c r="T37" s="96"/>
+      <c r="U37" s="96"/>
+      <c r="V37" s="96"/>
+      <c r="W37" s="96"/>
+      <c r="X37" s="96"/>
+      <c r="Y37" s="96"/>
+      <c r="Z37" s="96"/>
+      <c r="AA37" s="96"/>
+      <c r="AB37" s="96"/>
+      <c r="AC37" s="96"/>
+      <c r="AD37" s="96"/>
+      <c r="AE37" s="96"/>
+      <c r="AF37" s="96"/>
+      <c r="AG37" s="96"/>
+      <c r="AH37" s="96"/>
+      <c r="AI37" s="96"/>
       <c r="AJ37" s="8"/>
     </row>
     <row r="38" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="18"/>
-      <c r="C38" s="56"/>
-      <c r="D38" s="56"/>
-      <c r="E38" s="56"/>
-      <c r="F38" s="56"/>
-      <c r="G38" s="56"/>
-      <c r="H38" s="56"/>
-      <c r="I38" s="56"/>
-      <c r="J38" s="56"/>
-      <c r="K38" s="56"/>
-      <c r="L38" s="56"/>
-      <c r="M38" s="56"/>
-      <c r="N38" s="56"/>
-      <c r="O38" s="56"/>
-      <c r="P38" s="56"/>
-      <c r="Q38" s="56"/>
-      <c r="R38" s="56"/>
-      <c r="S38" s="56"/>
-      <c r="T38" s="56"/>
-      <c r="U38" s="56"/>
-      <c r="V38" s="56"/>
-      <c r="W38" s="56"/>
-      <c r="X38" s="56"/>
-      <c r="Y38" s="56"/>
-      <c r="Z38" s="56"/>
-      <c r="AA38" s="56"/>
-      <c r="AB38" s="56"/>
-      <c r="AC38" s="56"/>
-      <c r="AD38" s="56"/>
-      <c r="AE38" s="56"/>
-      <c r="AF38" s="56"/>
-      <c r="AG38" s="56"/>
-      <c r="AH38" s="56"/>
-      <c r="AI38" s="56"/>
+      <c r="C38" s="96"/>
+      <c r="D38" s="96"/>
+      <c r="E38" s="96"/>
+      <c r="F38" s="96"/>
+      <c r="G38" s="96"/>
+      <c r="H38" s="96"/>
+      <c r="I38" s="96"/>
+      <c r="J38" s="96"/>
+      <c r="K38" s="96"/>
+      <c r="L38" s="96"/>
+      <c r="M38" s="96"/>
+      <c r="N38" s="96"/>
+      <c r="O38" s="96"/>
+      <c r="P38" s="96"/>
+      <c r="Q38" s="96"/>
+      <c r="R38" s="96"/>
+      <c r="S38" s="96"/>
+      <c r="T38" s="96"/>
+      <c r="U38" s="96"/>
+      <c r="V38" s="96"/>
+      <c r="W38" s="96"/>
+      <c r="X38" s="96"/>
+      <c r="Y38" s="96"/>
+      <c r="Z38" s="96"/>
+      <c r="AA38" s="96"/>
+      <c r="AB38" s="96"/>
+      <c r="AC38" s="96"/>
+      <c r="AD38" s="96"/>
+      <c r="AE38" s="96"/>
+      <c r="AF38" s="96"/>
+      <c r="AG38" s="96"/>
+      <c r="AH38" s="96"/>
+      <c r="AI38" s="96"/>
       <c r="AJ38" s="8"/>
     </row>
     <row r="39" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="18"/>
-      <c r="C39" s="56"/>
-      <c r="D39" s="56"/>
-      <c r="E39" s="56"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="56"/>
-      <c r="H39" s="56"/>
-      <c r="I39" s="56"/>
-      <c r="J39" s="56"/>
-      <c r="K39" s="56"/>
-      <c r="L39" s="56"/>
-      <c r="M39" s="56"/>
-      <c r="N39" s="56"/>
-      <c r="O39" s="56"/>
-      <c r="P39" s="56"/>
-      <c r="Q39" s="56"/>
-      <c r="R39" s="56"/>
-      <c r="S39" s="56"/>
-      <c r="T39" s="56"/>
-      <c r="U39" s="56"/>
-      <c r="V39" s="56"/>
-      <c r="W39" s="56"/>
-      <c r="X39" s="56"/>
-      <c r="Y39" s="56"/>
-      <c r="Z39" s="56"/>
-      <c r="AA39" s="56"/>
-      <c r="AB39" s="56"/>
-      <c r="AC39" s="56"/>
-      <c r="AD39" s="56"/>
-      <c r="AE39" s="56"/>
-      <c r="AF39" s="56"/>
-      <c r="AG39" s="56"/>
-      <c r="AH39" s="56"/>
-      <c r="AI39" s="56"/>
+      <c r="C39" s="96"/>
+      <c r="D39" s="96"/>
+      <c r="E39" s="96"/>
+      <c r="F39" s="96"/>
+      <c r="G39" s="96"/>
+      <c r="H39" s="96"/>
+      <c r="I39" s="96"/>
+      <c r="J39" s="96"/>
+      <c r="K39" s="96"/>
+      <c r="L39" s="96"/>
+      <c r="M39" s="96"/>
+      <c r="N39" s="96"/>
+      <c r="O39" s="96"/>
+      <c r="P39" s="96"/>
+      <c r="Q39" s="96"/>
+      <c r="R39" s="96"/>
+      <c r="S39" s="96"/>
+      <c r="T39" s="96"/>
+      <c r="U39" s="96"/>
+      <c r="V39" s="96"/>
+      <c r="W39" s="96"/>
+      <c r="X39" s="96"/>
+      <c r="Y39" s="96"/>
+      <c r="Z39" s="96"/>
+      <c r="AA39" s="96"/>
+      <c r="AB39" s="96"/>
+      <c r="AC39" s="96"/>
+      <c r="AD39" s="96"/>
+      <c r="AE39" s="96"/>
+      <c r="AF39" s="96"/>
+      <c r="AG39" s="96"/>
+      <c r="AH39" s="96"/>
+      <c r="AI39" s="96"/>
       <c r="AJ39" s="8"/>
     </row>
     <row r="40" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="18"/>
-      <c r="C40" s="56"/>
-      <c r="D40" s="56"/>
-      <c r="E40" s="56"/>
-      <c r="F40" s="56"/>
-      <c r="G40" s="56"/>
-      <c r="H40" s="56"/>
-      <c r="I40" s="56"/>
-      <c r="J40" s="56"/>
-      <c r="K40" s="56"/>
-      <c r="L40" s="56"/>
-      <c r="M40" s="56"/>
-      <c r="N40" s="56"/>
-      <c r="O40" s="56"/>
-      <c r="P40" s="56"/>
-      <c r="Q40" s="56"/>
-      <c r="R40" s="56"/>
-      <c r="S40" s="56"/>
-      <c r="T40" s="56"/>
-      <c r="U40" s="56"/>
-      <c r="V40" s="56"/>
-      <c r="W40" s="56"/>
-      <c r="X40" s="56"/>
-      <c r="Y40" s="56"/>
-      <c r="Z40" s="56"/>
-      <c r="AA40" s="56"/>
-      <c r="AB40" s="56"/>
-      <c r="AC40" s="56"/>
-      <c r="AD40" s="56"/>
-      <c r="AE40" s="56"/>
-      <c r="AF40" s="56"/>
-      <c r="AG40" s="56"/>
-      <c r="AH40" s="56"/>
-      <c r="AI40" s="56"/>
+      <c r="C40" s="96"/>
+      <c r="D40" s="96"/>
+      <c r="E40" s="96"/>
+      <c r="F40" s="96"/>
+      <c r="G40" s="96"/>
+      <c r="H40" s="96"/>
+      <c r="I40" s="96"/>
+      <c r="J40" s="96"/>
+      <c r="K40" s="96"/>
+      <c r="L40" s="96"/>
+      <c r="M40" s="96"/>
+      <c r="N40" s="96"/>
+      <c r="O40" s="96"/>
+      <c r="P40" s="96"/>
+      <c r="Q40" s="96"/>
+      <c r="R40" s="96"/>
+      <c r="S40" s="96"/>
+      <c r="T40" s="96"/>
+      <c r="U40" s="96"/>
+      <c r="V40" s="96"/>
+      <c r="W40" s="96"/>
+      <c r="X40" s="96"/>
+      <c r="Y40" s="96"/>
+      <c r="Z40" s="96"/>
+      <c r="AA40" s="96"/>
+      <c r="AB40" s="96"/>
+      <c r="AC40" s="96"/>
+      <c r="AD40" s="96"/>
+      <c r="AE40" s="96"/>
+      <c r="AF40" s="96"/>
+      <c r="AG40" s="96"/>
+      <c r="AH40" s="96"/>
+      <c r="AI40" s="96"/>
       <c r="AJ40" s="8"/>
     </row>
     <row r="41" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="18"/>
-      <c r="C41" s="56"/>
-      <c r="D41" s="56"/>
-      <c r="E41" s="56"/>
-      <c r="F41" s="56"/>
-      <c r="G41" s="56"/>
-      <c r="H41" s="56"/>
-      <c r="I41" s="56"/>
-      <c r="J41" s="56"/>
-      <c r="K41" s="56"/>
-      <c r="L41" s="56"/>
-      <c r="M41" s="56"/>
-      <c r="N41" s="56"/>
-      <c r="O41" s="56"/>
-      <c r="P41" s="56"/>
-      <c r="Q41" s="56"/>
-      <c r="R41" s="56"/>
-      <c r="S41" s="56"/>
-      <c r="T41" s="56"/>
-      <c r="U41" s="56"/>
-      <c r="V41" s="56"/>
-      <c r="W41" s="56"/>
-      <c r="X41" s="56"/>
-      <c r="Y41" s="56"/>
-      <c r="Z41" s="56"/>
-      <c r="AA41" s="56"/>
-      <c r="AB41" s="56"/>
-      <c r="AC41" s="56"/>
-      <c r="AD41" s="56"/>
-      <c r="AE41" s="56"/>
-      <c r="AF41" s="56"/>
-      <c r="AG41" s="56"/>
-      <c r="AH41" s="56"/>
-      <c r="AI41" s="56"/>
+      <c r="C41" s="96"/>
+      <c r="D41" s="96"/>
+      <c r="E41" s="96"/>
+      <c r="F41" s="96"/>
+      <c r="G41" s="96"/>
+      <c r="H41" s="96"/>
+      <c r="I41" s="96"/>
+      <c r="J41" s="96"/>
+      <c r="K41" s="96"/>
+      <c r="L41" s="96"/>
+      <c r="M41" s="96"/>
+      <c r="N41" s="96"/>
+      <c r="O41" s="96"/>
+      <c r="P41" s="96"/>
+      <c r="Q41" s="96"/>
+      <c r="R41" s="96"/>
+      <c r="S41" s="96"/>
+      <c r="T41" s="96"/>
+      <c r="U41" s="96"/>
+      <c r="V41" s="96"/>
+      <c r="W41" s="96"/>
+      <c r="X41" s="96"/>
+      <c r="Y41" s="96"/>
+      <c r="Z41" s="96"/>
+      <c r="AA41" s="96"/>
+      <c r="AB41" s="96"/>
+      <c r="AC41" s="96"/>
+      <c r="AD41" s="96"/>
+      <c r="AE41" s="96"/>
+      <c r="AF41" s="96"/>
+      <c r="AG41" s="96"/>
+      <c r="AH41" s="96"/>
+      <c r="AI41" s="96"/>
       <c r="AJ41" s="8"/>
     </row>
     <row r="42" spans="2:36" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -3376,13 +3373,13 @@
     </row>
     <row r="43" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B43" s="18"/>
-      <c r="C43" s="57" t="s">
+      <c r="C43" s="97" t="s">
         <v>30</v>
       </c>
-      <c r="D43" s="57"/>
-      <c r="E43" s="57"/>
-      <c r="F43" s="57"/>
-      <c r="G43" s="57"/>
+      <c r="D43" s="97"/>
+      <c r="E43" s="97"/>
+      <c r="F43" s="97"/>
+      <c r="G43" s="97"/>
       <c r="AJ43" s="8"/>
     </row>
     <row r="44" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
@@ -3445,347 +3442,345 @@
     </row>
     <row r="52" spans="2:36" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B52" s="18"/>
-      <c r="H52" s="58" t="s">
+      <c r="H52" s="98" t="s">
         <v>36</v>
       </c>
-      <c r="I52" s="59"/>
-      <c r="J52" s="59"/>
-      <c r="K52" s="59"/>
-      <c r="L52" s="59"/>
-      <c r="M52" s="59"/>
-      <c r="N52" s="59"/>
-      <c r="O52" s="59"/>
-      <c r="P52" s="59"/>
-      <c r="Q52" s="59"/>
-      <c r="R52" s="59"/>
-      <c r="S52" s="59"/>
-      <c r="T52" s="59"/>
-      <c r="U52" s="59"/>
-      <c r="V52" s="59"/>
-      <c r="W52" s="59"/>
-      <c r="X52" s="59"/>
-      <c r="Y52" s="59"/>
-      <c r="Z52" s="59"/>
-      <c r="AA52" s="59"/>
-      <c r="AB52" s="59"/>
-      <c r="AC52" s="59"/>
-      <c r="AD52" s="59"/>
+      <c r="I52" s="99"/>
+      <c r="J52" s="99"/>
+      <c r="K52" s="99"/>
+      <c r="L52" s="99"/>
+      <c r="M52" s="99"/>
+      <c r="N52" s="99"/>
+      <c r="O52" s="99"/>
+      <c r="P52" s="99"/>
+      <c r="Q52" s="99"/>
+      <c r="R52" s="99"/>
+      <c r="S52" s="99"/>
+      <c r="T52" s="99"/>
+      <c r="U52" s="99"/>
+      <c r="V52" s="99"/>
+      <c r="W52" s="99"/>
+      <c r="X52" s="99"/>
+      <c r="Y52" s="99"/>
+      <c r="Z52" s="99"/>
+      <c r="AA52" s="99"/>
+      <c r="AB52" s="99"/>
+      <c r="AC52" s="99"/>
+      <c r="AD52" s="99"/>
       <c r="AJ52" s="8"/>
     </row>
     <row r="53" spans="2:36" x14ac:dyDescent="0.35">
       <c r="B53" s="18"/>
-      <c r="H53" s="60" t="s">
+      <c r="H53" s="100" t="s">
         <v>37</v>
       </c>
-      <c r="I53" s="60"/>
-      <c r="J53" s="60"/>
-      <c r="K53" s="60"/>
-      <c r="L53" s="60"/>
-      <c r="M53" s="60"/>
-      <c r="N53" s="60"/>
-      <c r="O53" s="60"/>
-      <c r="P53" s="60"/>
-      <c r="Q53" s="60"/>
-      <c r="R53" s="60"/>
-      <c r="S53" s="60"/>
-      <c r="T53" s="60"/>
-      <c r="U53" s="60"/>
-      <c r="V53" s="60"/>
-      <c r="W53" s="60"/>
-      <c r="X53" s="60"/>
-      <c r="Y53" s="60"/>
-      <c r="Z53" s="60"/>
-      <c r="AA53" s="60"/>
-      <c r="AB53" s="60"/>
-      <c r="AC53" s="60"/>
-      <c r="AD53" s="60"/>
+      <c r="I53" s="100"/>
+      <c r="J53" s="100"/>
+      <c r="K53" s="100"/>
+      <c r="L53" s="100"/>
+      <c r="M53" s="100"/>
+      <c r="N53" s="100"/>
+      <c r="O53" s="100"/>
+      <c r="P53" s="100"/>
+      <c r="Q53" s="100"/>
+      <c r="R53" s="100"/>
+      <c r="S53" s="100"/>
+      <c r="T53" s="100"/>
+      <c r="U53" s="100"/>
+      <c r="V53" s="100"/>
+      <c r="W53" s="100"/>
+      <c r="X53" s="100"/>
+      <c r="Y53" s="100"/>
+      <c r="Z53" s="100"/>
+      <c r="AA53" s="100"/>
+      <c r="AB53" s="100"/>
+      <c r="AC53" s="100"/>
+      <c r="AD53" s="100"/>
       <c r="AJ53" s="8"/>
     </row>
     <row r="54" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B54" s="18"/>
-      <c r="C54" s="61" t="s">
+      <c r="C54" s="101" t="s">
         <v>38</v>
       </c>
-      <c r="D54" s="61"/>
-      <c r="E54" s="61"/>
-      <c r="F54" s="61"/>
-      <c r="G54" s="61"/>
-      <c r="H54" s="62" t="s">
+      <c r="D54" s="101"/>
+      <c r="E54" s="101"/>
+      <c r="F54" s="101"/>
+      <c r="G54" s="101"/>
+      <c r="H54" s="102" t="s">
         <v>39</v>
       </c>
-      <c r="I54" s="62"/>
-      <c r="J54" s="62"/>
-      <c r="K54" s="62"/>
-      <c r="L54" s="62"/>
-      <c r="M54" s="63" t="s">
+      <c r="I54" s="102"/>
+      <c r="J54" s="102"/>
+      <c r="K54" s="102"/>
+      <c r="L54" s="102"/>
+      <c r="M54" s="103" t="s">
         <v>40</v>
       </c>
-      <c r="N54" s="64"/>
-      <c r="O54" s="64"/>
-      <c r="P54" s="64"/>
-      <c r="Q54" s="64"/>
-      <c r="R54" s="65"/>
-      <c r="S54" s="62" t="s">
+      <c r="N54" s="104"/>
+      <c r="O54" s="104"/>
+      <c r="P54" s="104"/>
+      <c r="Q54" s="104"/>
+      <c r="R54" s="105"/>
+      <c r="S54" s="102" t="s">
         <v>41</v>
       </c>
-      <c r="T54" s="62"/>
-      <c r="U54" s="62"/>
-      <c r="V54" s="62"/>
-      <c r="W54" s="62"/>
-      <c r="X54" s="66" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y54" s="49"/>
-      <c r="Z54" s="49"/>
-      <c r="AA54" s="49"/>
-      <c r="AB54" s="49"/>
-      <c r="AC54" s="49"/>
-      <c r="AD54" s="49"/>
-      <c r="AE54" s="49"/>
-      <c r="AF54" s="49"/>
-      <c r="AG54" s="49"/>
-      <c r="AH54" s="49"/>
-      <c r="AI54" s="49"/>
+      <c r="T54" s="102"/>
+      <c r="U54" s="102"/>
+      <c r="V54" s="102"/>
+      <c r="W54" s="102"/>
+      <c r="X54" s="106"/>
+      <c r="Y54" s="107"/>
+      <c r="Z54" s="107"/>
+      <c r="AA54" s="107"/>
+      <c r="AB54" s="107"/>
+      <c r="AC54" s="107"/>
+      <c r="AD54" s="107"/>
+      <c r="AE54" s="107"/>
+      <c r="AF54" s="107"/>
+      <c r="AG54" s="107"/>
+      <c r="AH54" s="107"/>
+      <c r="AI54" s="107"/>
       <c r="AJ54" s="8"/>
     </row>
     <row r="55" spans="2:36" x14ac:dyDescent="0.35">
       <c r="B55" s="18"/>
-      <c r="C55" s="44"/>
-      <c r="D55" s="44"/>
-      <c r="E55" s="44"/>
-      <c r="F55" s="44"/>
-      <c r="G55" s="44"/>
-      <c r="H55" s="44"/>
-      <c r="I55" s="44"/>
-      <c r="J55" s="44"/>
-      <c r="K55" s="44"/>
-      <c r="L55" s="44"/>
-      <c r="M55" s="45"/>
+      <c r="C55" s="109"/>
+      <c r="D55" s="109"/>
+      <c r="E55" s="109"/>
+      <c r="F55" s="109"/>
+      <c r="G55" s="109"/>
+      <c r="H55" s="109"/>
+      <c r="I55" s="109"/>
+      <c r="J55" s="109"/>
+      <c r="K55" s="109"/>
+      <c r="L55" s="109"/>
+      <c r="M55" s="110"/>
       <c r="N55" s="46"/>
       <c r="O55" s="46"/>
       <c r="P55" s="46"/>
       <c r="Q55" s="46"/>
       <c r="R55" s="47"/>
-      <c r="S55" s="44"/>
-      <c r="T55" s="44"/>
-      <c r="U55" s="44"/>
-      <c r="V55" s="44"/>
-      <c r="W55" s="45"/>
-      <c r="X55" s="48" t="s">
-        <v>43</v>
-      </c>
-      <c r="Y55" s="49"/>
-      <c r="Z55" s="49"/>
-      <c r="AA55" s="49"/>
-      <c r="AB55" s="49"/>
-      <c r="AC55" s="49"/>
-      <c r="AD55" s="49"/>
-      <c r="AE55" s="49"/>
-      <c r="AF55" s="49"/>
-      <c r="AG55" s="49"/>
-      <c r="AH55" s="49"/>
-      <c r="AI55" s="49"/>
+      <c r="S55" s="109"/>
+      <c r="T55" s="109"/>
+      <c r="U55" s="109"/>
+      <c r="V55" s="109"/>
+      <c r="W55" s="110"/>
+      <c r="X55" s="111" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y55" s="107"/>
+      <c r="Z55" s="107"/>
+      <c r="AA55" s="107"/>
+      <c r="AB55" s="107"/>
+      <c r="AC55" s="107"/>
+      <c r="AD55" s="107"/>
+      <c r="AE55" s="107"/>
+      <c r="AF55" s="107"/>
+      <c r="AG55" s="107"/>
+      <c r="AH55" s="107"/>
+      <c r="AI55" s="107"/>
       <c r="AJ55" s="8"/>
     </row>
     <row r="56" spans="2:36" x14ac:dyDescent="0.35">
       <c r="B56" s="18"/>
-      <c r="C56" s="44"/>
-      <c r="D56" s="44"/>
-      <c r="E56" s="44"/>
-      <c r="F56" s="44"/>
-      <c r="G56" s="44"/>
-      <c r="H56" s="44"/>
-      <c r="I56" s="44"/>
-      <c r="J56" s="44"/>
-      <c r="K56" s="44"/>
-      <c r="L56" s="44"/>
-      <c r="M56" s="45"/>
+      <c r="C56" s="109"/>
+      <c r="D56" s="109"/>
+      <c r="E56" s="109"/>
+      <c r="F56" s="109"/>
+      <c r="G56" s="109"/>
+      <c r="H56" s="109"/>
+      <c r="I56" s="109"/>
+      <c r="J56" s="109"/>
+      <c r="K56" s="109"/>
+      <c r="L56" s="109"/>
+      <c r="M56" s="110"/>
       <c r="N56" s="46"/>
       <c r="O56" s="46"/>
       <c r="P56" s="46"/>
       <c r="Q56" s="46"/>
       <c r="R56" s="47"/>
-      <c r="S56" s="44"/>
-      <c r="T56" s="44"/>
-      <c r="U56" s="44"/>
-      <c r="V56" s="44"/>
-      <c r="W56" s="45"/>
-      <c r="X56" s="49"/>
-      <c r="Y56" s="49"/>
-      <c r="Z56" s="49"/>
-      <c r="AA56" s="49"/>
-      <c r="AB56" s="49"/>
-      <c r="AC56" s="49"/>
-      <c r="AD56" s="49"/>
-      <c r="AE56" s="49"/>
-      <c r="AF56" s="49"/>
-      <c r="AG56" s="49"/>
-      <c r="AH56" s="49"/>
-      <c r="AI56" s="49"/>
+      <c r="S56" s="109"/>
+      <c r="T56" s="109"/>
+      <c r="U56" s="109"/>
+      <c r="V56" s="109"/>
+      <c r="W56" s="110"/>
+      <c r="X56" s="107"/>
+      <c r="Y56" s="107"/>
+      <c r="Z56" s="107"/>
+      <c r="AA56" s="107"/>
+      <c r="AB56" s="107"/>
+      <c r="AC56" s="107"/>
+      <c r="AD56" s="107"/>
+      <c r="AE56" s="107"/>
+      <c r="AF56" s="107"/>
+      <c r="AG56" s="107"/>
+      <c r="AH56" s="107"/>
+      <c r="AI56" s="107"/>
       <c r="AJ56" s="8"/>
     </row>
     <row r="57" spans="2:36" x14ac:dyDescent="0.35">
       <c r="B57" s="18"/>
-      <c r="C57" s="44"/>
-      <c r="D57" s="44"/>
-      <c r="E57" s="44"/>
-      <c r="F57" s="44"/>
-      <c r="G57" s="44"/>
-      <c r="H57" s="44"/>
-      <c r="I57" s="44"/>
-      <c r="J57" s="44"/>
-      <c r="K57" s="44"/>
-      <c r="L57" s="44"/>
-      <c r="M57" s="45"/>
+      <c r="C57" s="109"/>
+      <c r="D57" s="109"/>
+      <c r="E57" s="109"/>
+      <c r="F57" s="109"/>
+      <c r="G57" s="109"/>
+      <c r="H57" s="109"/>
+      <c r="I57" s="109"/>
+      <c r="J57" s="109"/>
+      <c r="K57" s="109"/>
+      <c r="L57" s="109"/>
+      <c r="M57" s="110"/>
       <c r="N57" s="46"/>
       <c r="O57" s="46"/>
       <c r="P57" s="46"/>
       <c r="Q57" s="46"/>
       <c r="R57" s="47"/>
-      <c r="S57" s="44"/>
-      <c r="T57" s="44"/>
-      <c r="U57" s="44"/>
-      <c r="V57" s="44"/>
-      <c r="W57" s="45"/>
-      <c r="X57" s="49"/>
-      <c r="Y57" s="49"/>
-      <c r="Z57" s="49"/>
-      <c r="AA57" s="49"/>
-      <c r="AB57" s="49"/>
-      <c r="AC57" s="49"/>
-      <c r="AD57" s="49"/>
-      <c r="AE57" s="49"/>
-      <c r="AF57" s="49"/>
-      <c r="AG57" s="49"/>
-      <c r="AH57" s="49"/>
-      <c r="AI57" s="49"/>
+      <c r="S57" s="109"/>
+      <c r="T57" s="109"/>
+      <c r="U57" s="109"/>
+      <c r="V57" s="109"/>
+      <c r="W57" s="110"/>
+      <c r="X57" s="107"/>
+      <c r="Y57" s="107"/>
+      <c r="Z57" s="107"/>
+      <c r="AA57" s="107"/>
+      <c r="AB57" s="107"/>
+      <c r="AC57" s="107"/>
+      <c r="AD57" s="107"/>
+      <c r="AE57" s="107"/>
+      <c r="AF57" s="107"/>
+      <c r="AG57" s="107"/>
+      <c r="AH57" s="107"/>
+      <c r="AI57" s="107"/>
       <c r="AJ57" s="8"/>
     </row>
     <row r="58" spans="2:36" x14ac:dyDescent="0.35">
       <c r="B58" s="18"/>
-      <c r="C58" s="44"/>
-      <c r="D58" s="44"/>
-      <c r="E58" s="44"/>
-      <c r="F58" s="44"/>
-      <c r="G58" s="44"/>
-      <c r="H58" s="44"/>
-      <c r="I58" s="44"/>
-      <c r="J58" s="44"/>
-      <c r="K58" s="44"/>
-      <c r="L58" s="44"/>
-      <c r="M58" s="45"/>
+      <c r="C58" s="109"/>
+      <c r="D58" s="109"/>
+      <c r="E58" s="109"/>
+      <c r="F58" s="109"/>
+      <c r="G58" s="109"/>
+      <c r="H58" s="109"/>
+      <c r="I58" s="109"/>
+      <c r="J58" s="109"/>
+      <c r="K58" s="109"/>
+      <c r="L58" s="109"/>
+      <c r="M58" s="110"/>
       <c r="N58" s="46"/>
       <c r="O58" s="46"/>
       <c r="P58" s="46"/>
       <c r="Q58" s="46"/>
       <c r="R58" s="47"/>
-      <c r="S58" s="44"/>
-      <c r="T58" s="44"/>
-      <c r="U58" s="44"/>
-      <c r="V58" s="44"/>
-      <c r="W58" s="45"/>
-      <c r="X58" s="49"/>
-      <c r="Y58" s="49"/>
-      <c r="Z58" s="49"/>
-      <c r="AA58" s="49"/>
-      <c r="AB58" s="49"/>
-      <c r="AC58" s="49"/>
-      <c r="AD58" s="49"/>
-      <c r="AE58" s="49"/>
-      <c r="AF58" s="49"/>
-      <c r="AG58" s="49"/>
-      <c r="AH58" s="49"/>
-      <c r="AI58" s="49"/>
+      <c r="S58" s="109"/>
+      <c r="T58" s="109"/>
+      <c r="U58" s="109"/>
+      <c r="V58" s="109"/>
+      <c r="W58" s="110"/>
+      <c r="X58" s="107"/>
+      <c r="Y58" s="107"/>
+      <c r="Z58" s="107"/>
+      <c r="AA58" s="107"/>
+      <c r="AB58" s="107"/>
+      <c r="AC58" s="107"/>
+      <c r="AD58" s="107"/>
+      <c r="AE58" s="107"/>
+      <c r="AF58" s="107"/>
+      <c r="AG58" s="107"/>
+      <c r="AH58" s="107"/>
+      <c r="AI58" s="107"/>
       <c r="AJ58" s="8"/>
     </row>
     <row r="59" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B59" s="18"/>
-      <c r="C59" s="50" t="s">
+      <c r="C59" s="112" t="s">
+        <v>43</v>
+      </c>
+      <c r="D59" s="112"/>
+      <c r="E59" s="112"/>
+      <c r="F59" s="112"/>
+      <c r="G59" s="112"/>
+      <c r="H59" s="112" t="s">
         <v>44</v>
       </c>
-      <c r="D59" s="50"/>
-      <c r="E59" s="50"/>
-      <c r="F59" s="50"/>
-      <c r="G59" s="50"/>
-      <c r="H59" s="50" t="s">
+      <c r="I59" s="112"/>
+      <c r="J59" s="112"/>
+      <c r="K59" s="112"/>
+      <c r="L59" s="112"/>
+      <c r="M59" s="113" t="s">
         <v>45</v>
       </c>
-      <c r="I59" s="50"/>
-      <c r="J59" s="50"/>
-      <c r="K59" s="50"/>
-      <c r="L59" s="50"/>
-      <c r="M59" s="51" t="s">
-        <v>46</v>
-      </c>
-      <c r="N59" s="52"/>
-      <c r="O59" s="52"/>
-      <c r="P59" s="52"/>
-      <c r="Q59" s="52"/>
-      <c r="R59" s="53"/>
-      <c r="S59" s="54" t="s">
-        <v>44</v>
-      </c>
-      <c r="T59" s="54"/>
-      <c r="U59" s="54"/>
-      <c r="V59" s="54"/>
-      <c r="W59" s="55"/>
-      <c r="X59" s="49"/>
-      <c r="Y59" s="49"/>
-      <c r="Z59" s="49"/>
-      <c r="AA59" s="49"/>
-      <c r="AB59" s="49"/>
-      <c r="AC59" s="49"/>
-      <c r="AD59" s="49"/>
-      <c r="AE59" s="49"/>
-      <c r="AF59" s="49"/>
-      <c r="AG59" s="49"/>
-      <c r="AH59" s="49"/>
-      <c r="AI59" s="49"/>
+      <c r="N59" s="114"/>
+      <c r="O59" s="114"/>
+      <c r="P59" s="114"/>
+      <c r="Q59" s="114"/>
+      <c r="R59" s="115"/>
+      <c r="S59" s="68" t="s">
+        <v>43</v>
+      </c>
+      <c r="T59" s="68"/>
+      <c r="U59" s="68"/>
+      <c r="V59" s="68"/>
+      <c r="W59" s="116"/>
+      <c r="X59" s="107"/>
+      <c r="Y59" s="107"/>
+      <c r="Z59" s="107"/>
+      <c r="AA59" s="107"/>
+      <c r="AB59" s="107"/>
+      <c r="AC59" s="107"/>
+      <c r="AD59" s="107"/>
+      <c r="AE59" s="107"/>
+      <c r="AF59" s="107"/>
+      <c r="AG59" s="107"/>
+      <c r="AH59" s="107"/>
+      <c r="AI59" s="107"/>
       <c r="AJ59" s="8"/>
     </row>
     <row r="60" spans="2:36" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B60" s="18"/>
-      <c r="C60" s="39" t="s">
+      <c r="C60" s="69" t="s">
+        <v>46</v>
+      </c>
+      <c r="D60" s="69"/>
+      <c r="E60" s="69"/>
+      <c r="F60" s="69"/>
+      <c r="G60" s="69"/>
+      <c r="H60" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="D60" s="39"/>
-      <c r="E60" s="39"/>
-      <c r="F60" s="39"/>
-      <c r="G60" s="39"/>
-      <c r="H60" s="39" t="s">
+      <c r="I60" s="69"/>
+      <c r="J60" s="69"/>
+      <c r="K60" s="69"/>
+      <c r="L60" s="69"/>
+      <c r="M60" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="I60" s="39"/>
-      <c r="J60" s="39"/>
-      <c r="K60" s="39"/>
-      <c r="L60" s="39"/>
-      <c r="M60" s="40" t="s">
+      <c r="N60" s="85"/>
+      <c r="O60" s="85"/>
+      <c r="P60" s="85"/>
+      <c r="Q60" s="85"/>
+      <c r="R60" s="86"/>
+      <c r="S60" s="69" t="s">
         <v>49</v>
       </c>
-      <c r="N60" s="41"/>
-      <c r="O60" s="41"/>
-      <c r="P60" s="41"/>
-      <c r="Q60" s="41"/>
-      <c r="R60" s="42"/>
-      <c r="S60" s="39" t="s">
-        <v>50</v>
-      </c>
-      <c r="T60" s="39"/>
-      <c r="U60" s="39"/>
-      <c r="V60" s="39"/>
-      <c r="W60" s="40"/>
-      <c r="X60" s="49"/>
-      <c r="Y60" s="49"/>
-      <c r="Z60" s="49"/>
-      <c r="AA60" s="49"/>
-      <c r="AB60" s="49"/>
-      <c r="AC60" s="49"/>
-      <c r="AD60" s="49"/>
-      <c r="AE60" s="49"/>
-      <c r="AF60" s="49"/>
-      <c r="AG60" s="49"/>
-      <c r="AH60" s="49"/>
-      <c r="AI60" s="49"/>
+      <c r="T60" s="69"/>
+      <c r="U60" s="69"/>
+      <c r="V60" s="69"/>
+      <c r="W60" s="84"/>
+      <c r="X60" s="107"/>
+      <c r="Y60" s="107"/>
+      <c r="Z60" s="107"/>
+      <c r="AA60" s="107"/>
+      <c r="AB60" s="107"/>
+      <c r="AC60" s="107"/>
+      <c r="AD60" s="107"/>
+      <c r="AE60" s="107"/>
+      <c r="AF60" s="107"/>
+      <c r="AG60" s="107"/>
+      <c r="AH60" s="107"/>
+      <c r="AI60" s="107"/>
       <c r="AJ60" s="8"/>
     </row>
     <row r="61" spans="2:36" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -3826,88 +3821,17 @@
       <c r="AJ61" s="26"/>
     </row>
     <row r="62" spans="2:36" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="AE62" s="43" t="s">
-        <v>51</v>
-      </c>
-      <c r="AF62" s="43"/>
-      <c r="AG62" s="43"/>
-      <c r="AH62" s="43"/>
-      <c r="AI62" s="43"/>
-      <c r="AJ62" s="43"/>
+      <c r="AE62" s="108" t="s">
+        <v>50</v>
+      </c>
+      <c r="AF62" s="108"/>
+      <c r="AG62" s="108"/>
+      <c r="AH62" s="108"/>
+      <c r="AI62" s="108"/>
+      <c r="AJ62" s="108"/>
     </row>
   </sheetData>
   <mergeCells count="85">
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="S8:Y8"/>
-    <mergeCell ref="B2:G5"/>
-    <mergeCell ref="H2:AJ5"/>
-    <mergeCell ref="B6:AJ6"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="S7:Y7"/>
-    <mergeCell ref="B9:G9"/>
-    <mergeCell ref="S9:Y9"/>
-    <mergeCell ref="B10:G10"/>
-    <mergeCell ref="S10:Y10"/>
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="S11:Y11"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="S12:Y12"/>
-    <mergeCell ref="AA12:AI17"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="B14:G14"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="B17:G17"/>
-    <mergeCell ref="B18:AJ18"/>
-    <mergeCell ref="Q19:V19"/>
-    <mergeCell ref="C21:C25"/>
-    <mergeCell ref="D21:K23"/>
-    <mergeCell ref="L21:Q23"/>
-    <mergeCell ref="R21:W23"/>
-    <mergeCell ref="X21:AC23"/>
-    <mergeCell ref="AD21:AI24"/>
-    <mergeCell ref="D24:K25"/>
-    <mergeCell ref="L24:Q25"/>
-    <mergeCell ref="R24:W25"/>
-    <mergeCell ref="X24:AC25"/>
-    <mergeCell ref="AD25:AI25"/>
-    <mergeCell ref="D26:K26"/>
-    <mergeCell ref="L26:Q26"/>
-    <mergeCell ref="R26:W26"/>
-    <mergeCell ref="X26:AC26"/>
-    <mergeCell ref="R27:W27"/>
-    <mergeCell ref="X27:AC27"/>
-    <mergeCell ref="D28:K28"/>
-    <mergeCell ref="L28:Q28"/>
-    <mergeCell ref="R28:W28"/>
-    <mergeCell ref="X28:AC28"/>
-    <mergeCell ref="D27:K27"/>
-    <mergeCell ref="L27:Q27"/>
-    <mergeCell ref="D29:K29"/>
-    <mergeCell ref="L29:Q29"/>
-    <mergeCell ref="R29:W29"/>
-    <mergeCell ref="X29:AC29"/>
-    <mergeCell ref="D30:K30"/>
-    <mergeCell ref="L30:Q30"/>
-    <mergeCell ref="R30:W30"/>
-    <mergeCell ref="X30:AC30"/>
-    <mergeCell ref="D31:K31"/>
-    <mergeCell ref="L31:Q31"/>
-    <mergeCell ref="R31:W31"/>
-    <mergeCell ref="X31:AC31"/>
-    <mergeCell ref="D32:K32"/>
-    <mergeCell ref="L32:Q32"/>
-    <mergeCell ref="R32:W32"/>
-    <mergeCell ref="X32:AC32"/>
-    <mergeCell ref="C33:AI41"/>
-    <mergeCell ref="C43:G43"/>
-    <mergeCell ref="H52:AD52"/>
-    <mergeCell ref="H53:AD53"/>
-    <mergeCell ref="C54:G54"/>
-    <mergeCell ref="H54:L54"/>
-    <mergeCell ref="M54:R54"/>
-    <mergeCell ref="S54:W54"/>
-    <mergeCell ref="X54:AI54"/>
     <mergeCell ref="H60:L60"/>
     <mergeCell ref="M60:R60"/>
     <mergeCell ref="S60:W60"/>
@@ -3922,6 +3846,77 @@
     <mergeCell ref="M59:R59"/>
     <mergeCell ref="S59:W59"/>
     <mergeCell ref="C60:G60"/>
+    <mergeCell ref="C33:AI41"/>
+    <mergeCell ref="C43:G43"/>
+    <mergeCell ref="H52:AD52"/>
+    <mergeCell ref="H53:AD53"/>
+    <mergeCell ref="C54:G54"/>
+    <mergeCell ref="H54:L54"/>
+    <mergeCell ref="M54:R54"/>
+    <mergeCell ref="S54:W54"/>
+    <mergeCell ref="X54:AI54"/>
+    <mergeCell ref="D31:K31"/>
+    <mergeCell ref="L31:Q31"/>
+    <mergeCell ref="R31:W31"/>
+    <mergeCell ref="X31:AC31"/>
+    <mergeCell ref="D32:K32"/>
+    <mergeCell ref="L32:Q32"/>
+    <mergeCell ref="R32:W32"/>
+    <mergeCell ref="X32:AC32"/>
+    <mergeCell ref="D29:K29"/>
+    <mergeCell ref="L29:Q29"/>
+    <mergeCell ref="R29:W29"/>
+    <mergeCell ref="X29:AC29"/>
+    <mergeCell ref="D30:K30"/>
+    <mergeCell ref="L30:Q30"/>
+    <mergeCell ref="R30:W30"/>
+    <mergeCell ref="X30:AC30"/>
+    <mergeCell ref="D28:K28"/>
+    <mergeCell ref="L28:Q28"/>
+    <mergeCell ref="R28:W28"/>
+    <mergeCell ref="X28:AC28"/>
+    <mergeCell ref="D27:K27"/>
+    <mergeCell ref="L27:Q27"/>
+    <mergeCell ref="D26:K26"/>
+    <mergeCell ref="L26:Q26"/>
+    <mergeCell ref="R26:W26"/>
+    <mergeCell ref="X26:AC26"/>
+    <mergeCell ref="R27:W27"/>
+    <mergeCell ref="X27:AC27"/>
+    <mergeCell ref="B18:AJ18"/>
+    <mergeCell ref="Q19:V19"/>
+    <mergeCell ref="C21:C25"/>
+    <mergeCell ref="D21:K23"/>
+    <mergeCell ref="L21:Q23"/>
+    <mergeCell ref="R21:W23"/>
+    <mergeCell ref="X21:AC23"/>
+    <mergeCell ref="AD21:AI24"/>
+    <mergeCell ref="D24:K25"/>
+    <mergeCell ref="L24:Q25"/>
+    <mergeCell ref="R24:W25"/>
+    <mergeCell ref="X24:AC25"/>
+    <mergeCell ref="AD25:AI25"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="S12:Y12"/>
+    <mergeCell ref="AA12:AI17"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="S9:Y9"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="S10:Y10"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="S11:Y11"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="S8:Y8"/>
+    <mergeCell ref="B2:G5"/>
+    <mergeCell ref="H2:AJ5"/>
+    <mergeCell ref="B6:AJ6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="S7:Y7"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0.2" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
feat: add HTML preview functionality for calibration certificates and update related templates
</commit_message>
<xml_diff>
--- a/public/assets/templates/template_kalibrasi_jangka_sorong_sertifikat.xlsx
+++ b/public/assets/templates/template_kalibrasi_jangka_sorong_sertifikat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BFF64DD-04FB-4C0A-A4A6-5DCC678912B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4BA745E-84ED-4E09-91F1-39D865AE2749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{12CE2AE1-1EA9-4BA9-947C-BB59CA2A4E03}"/>
   </bookViews>
@@ -667,7 +667,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -808,6 +808,24 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -841,23 +859,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -931,77 +934,71 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1360,15 +1357,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>184150</xdr:rowOff>
+      <xdr:colOff>62784</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>64833</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>184150</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>63499</xdr:rowOff>
+      <xdr:colOff>138626</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>178874</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1384,7 +1381,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -1398,8 +1395,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="704850" y="368300"/>
-          <a:ext cx="1409700" cy="603250"/>
+          <a:off x="308735" y="498601"/>
+          <a:ext cx="1305595" cy="355519"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1770,137 +1767,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3784DB8E-6CFA-4599-A8D3-4AF7E4F83F0D}">
   <dimension ref="B1:AM62"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="3.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="36" width="3.7265625" style="1" customWidth="1"/>
-    <col min="37" max="257" width="9" style="1"/>
-    <col min="258" max="292" width="3.7265625" style="1" customWidth="1"/>
-    <col min="293" max="513" width="9" style="1"/>
-    <col min="514" max="548" width="3.7265625" style="1" customWidth="1"/>
-    <col min="549" max="769" width="9" style="1"/>
-    <col min="770" max="804" width="3.7265625" style="1" customWidth="1"/>
-    <col min="805" max="1025" width="9" style="1"/>
-    <col min="1026" max="1060" width="3.7265625" style="1" customWidth="1"/>
-    <col min="1061" max="1281" width="9" style="1"/>
-    <col min="1282" max="1316" width="3.7265625" style="1" customWidth="1"/>
-    <col min="1317" max="1537" width="9" style="1"/>
-    <col min="1538" max="1572" width="3.7265625" style="1" customWidth="1"/>
-    <col min="1573" max="1793" width="9" style="1"/>
-    <col min="1794" max="1828" width="3.7265625" style="1" customWidth="1"/>
-    <col min="1829" max="2049" width="9" style="1"/>
-    <col min="2050" max="2084" width="3.7265625" style="1" customWidth="1"/>
-    <col min="2085" max="2305" width="9" style="1"/>
-    <col min="2306" max="2340" width="3.7265625" style="1" customWidth="1"/>
-    <col min="2341" max="2561" width="9" style="1"/>
-    <col min="2562" max="2596" width="3.7265625" style="1" customWidth="1"/>
-    <col min="2597" max="2817" width="9" style="1"/>
-    <col min="2818" max="2852" width="3.7265625" style="1" customWidth="1"/>
-    <col min="2853" max="3073" width="9" style="1"/>
-    <col min="3074" max="3108" width="3.7265625" style="1" customWidth="1"/>
-    <col min="3109" max="3329" width="9" style="1"/>
-    <col min="3330" max="3364" width="3.7265625" style="1" customWidth="1"/>
-    <col min="3365" max="3585" width="9" style="1"/>
-    <col min="3586" max="3620" width="3.7265625" style="1" customWidth="1"/>
-    <col min="3621" max="3841" width="9" style="1"/>
-    <col min="3842" max="3876" width="3.7265625" style="1" customWidth="1"/>
-    <col min="3877" max="4097" width="9" style="1"/>
-    <col min="4098" max="4132" width="3.7265625" style="1" customWidth="1"/>
-    <col min="4133" max="4353" width="9" style="1"/>
-    <col min="4354" max="4388" width="3.7265625" style="1" customWidth="1"/>
-    <col min="4389" max="4609" width="9" style="1"/>
-    <col min="4610" max="4644" width="3.7265625" style="1" customWidth="1"/>
-    <col min="4645" max="4865" width="9" style="1"/>
-    <col min="4866" max="4900" width="3.7265625" style="1" customWidth="1"/>
-    <col min="4901" max="5121" width="9" style="1"/>
-    <col min="5122" max="5156" width="3.7265625" style="1" customWidth="1"/>
-    <col min="5157" max="5377" width="9" style="1"/>
-    <col min="5378" max="5412" width="3.7265625" style="1" customWidth="1"/>
-    <col min="5413" max="5633" width="9" style="1"/>
-    <col min="5634" max="5668" width="3.7265625" style="1" customWidth="1"/>
-    <col min="5669" max="5889" width="9" style="1"/>
-    <col min="5890" max="5924" width="3.7265625" style="1" customWidth="1"/>
-    <col min="5925" max="6145" width="9" style="1"/>
-    <col min="6146" max="6180" width="3.7265625" style="1" customWidth="1"/>
-    <col min="6181" max="6401" width="9" style="1"/>
-    <col min="6402" max="6436" width="3.7265625" style="1" customWidth="1"/>
-    <col min="6437" max="6657" width="9" style="1"/>
-    <col min="6658" max="6692" width="3.7265625" style="1" customWidth="1"/>
-    <col min="6693" max="6913" width="9" style="1"/>
-    <col min="6914" max="6948" width="3.7265625" style="1" customWidth="1"/>
-    <col min="6949" max="7169" width="9" style="1"/>
-    <col min="7170" max="7204" width="3.7265625" style="1" customWidth="1"/>
-    <col min="7205" max="7425" width="9" style="1"/>
-    <col min="7426" max="7460" width="3.7265625" style="1" customWidth="1"/>
-    <col min="7461" max="7681" width="9" style="1"/>
-    <col min="7682" max="7716" width="3.7265625" style="1" customWidth="1"/>
-    <col min="7717" max="7937" width="9" style="1"/>
-    <col min="7938" max="7972" width="3.7265625" style="1" customWidth="1"/>
-    <col min="7973" max="8193" width="9" style="1"/>
-    <col min="8194" max="8228" width="3.7265625" style="1" customWidth="1"/>
-    <col min="8229" max="8449" width="9" style="1"/>
-    <col min="8450" max="8484" width="3.7265625" style="1" customWidth="1"/>
-    <col min="8485" max="8705" width="9" style="1"/>
-    <col min="8706" max="8740" width="3.7265625" style="1" customWidth="1"/>
-    <col min="8741" max="8961" width="9" style="1"/>
-    <col min="8962" max="8996" width="3.7265625" style="1" customWidth="1"/>
-    <col min="8997" max="9217" width="9" style="1"/>
-    <col min="9218" max="9252" width="3.7265625" style="1" customWidth="1"/>
-    <col min="9253" max="9473" width="9" style="1"/>
-    <col min="9474" max="9508" width="3.7265625" style="1" customWidth="1"/>
-    <col min="9509" max="9729" width="9" style="1"/>
-    <col min="9730" max="9764" width="3.7265625" style="1" customWidth="1"/>
-    <col min="9765" max="9985" width="9" style="1"/>
-    <col min="9986" max="10020" width="3.7265625" style="1" customWidth="1"/>
-    <col min="10021" max="10241" width="9" style="1"/>
-    <col min="10242" max="10276" width="3.7265625" style="1" customWidth="1"/>
-    <col min="10277" max="10497" width="9" style="1"/>
-    <col min="10498" max="10532" width="3.7265625" style="1" customWidth="1"/>
-    <col min="10533" max="10753" width="9" style="1"/>
-    <col min="10754" max="10788" width="3.7265625" style="1" customWidth="1"/>
-    <col min="10789" max="11009" width="9" style="1"/>
-    <col min="11010" max="11044" width="3.7265625" style="1" customWidth="1"/>
-    <col min="11045" max="11265" width="9" style="1"/>
-    <col min="11266" max="11300" width="3.7265625" style="1" customWidth="1"/>
-    <col min="11301" max="11521" width="9" style="1"/>
-    <col min="11522" max="11556" width="3.7265625" style="1" customWidth="1"/>
-    <col min="11557" max="11777" width="9" style="1"/>
-    <col min="11778" max="11812" width="3.7265625" style="1" customWidth="1"/>
-    <col min="11813" max="12033" width="9" style="1"/>
-    <col min="12034" max="12068" width="3.7265625" style="1" customWidth="1"/>
-    <col min="12069" max="12289" width="9" style="1"/>
-    <col min="12290" max="12324" width="3.7265625" style="1" customWidth="1"/>
-    <col min="12325" max="12545" width="9" style="1"/>
-    <col min="12546" max="12580" width="3.7265625" style="1" customWidth="1"/>
-    <col min="12581" max="12801" width="9" style="1"/>
-    <col min="12802" max="12836" width="3.7265625" style="1" customWidth="1"/>
-    <col min="12837" max="13057" width="9" style="1"/>
-    <col min="13058" max="13092" width="3.7265625" style="1" customWidth="1"/>
-    <col min="13093" max="13313" width="9" style="1"/>
-    <col min="13314" max="13348" width="3.7265625" style="1" customWidth="1"/>
-    <col min="13349" max="13569" width="9" style="1"/>
-    <col min="13570" max="13604" width="3.7265625" style="1" customWidth="1"/>
-    <col min="13605" max="13825" width="9" style="1"/>
-    <col min="13826" max="13860" width="3.7265625" style="1" customWidth="1"/>
-    <col min="13861" max="14081" width="9" style="1"/>
-    <col min="14082" max="14116" width="3.7265625" style="1" customWidth="1"/>
-    <col min="14117" max="14337" width="9" style="1"/>
-    <col min="14338" max="14372" width="3.7265625" style="1" customWidth="1"/>
-    <col min="14373" max="14593" width="9" style="1"/>
-    <col min="14594" max="14628" width="3.7265625" style="1" customWidth="1"/>
-    <col min="14629" max="14849" width="9" style="1"/>
-    <col min="14850" max="14884" width="3.7265625" style="1" customWidth="1"/>
-    <col min="14885" max="15105" width="9" style="1"/>
-    <col min="15106" max="15140" width="3.7265625" style="1" customWidth="1"/>
-    <col min="15141" max="15361" width="9" style="1"/>
-    <col min="15362" max="15396" width="3.7265625" style="1" customWidth="1"/>
-    <col min="15397" max="15617" width="9" style="1"/>
-    <col min="15618" max="15652" width="3.7265625" style="1" customWidth="1"/>
-    <col min="15653" max="15873" width="9" style="1"/>
-    <col min="15874" max="15908" width="3.7265625" style="1" customWidth="1"/>
-    <col min="15909" max="16129" width="9" style="1"/>
-    <col min="16130" max="16164" width="3.7265625" style="1" customWidth="1"/>
-    <col min="16165" max="16384" width="9" style="1"/>
+    <col min="1" max="16384" width="3.54296875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:39" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -2092,14 +1961,14 @@
       <c r="AJ6" s="112"/>
     </row>
     <row r="7" spans="2:39" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="92" t="s">
+      <c r="B7" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="93"/>
-      <c r="D7" s="93"/>
-      <c r="E7" s="93"/>
-      <c r="F7" s="93"/>
-      <c r="G7" s="93"/>
+      <c r="C7" s="69"/>
+      <c r="D7" s="69"/>
+      <c r="E7" s="69"/>
+      <c r="F7" s="69"/>
+      <c r="G7" s="69"/>
       <c r="H7" s="4" t="s">
         <v>2</v>
       </c>
@@ -2112,15 +1981,15 @@
       <c r="O7" s="113"/>
       <c r="P7" s="113"/>
       <c r="Q7" s="113"/>
-      <c r="S7" s="94" t="s">
+      <c r="S7" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="T7" s="94"/>
-      <c r="U7" s="94"/>
-      <c r="V7" s="94"/>
-      <c r="W7" s="94"/>
-      <c r="X7" s="94"/>
-      <c r="Y7" s="94"/>
+      <c r="T7" s="69"/>
+      <c r="U7" s="69"/>
+      <c r="V7" s="69"/>
+      <c r="W7" s="69"/>
+      <c r="X7" s="69"/>
+      <c r="Y7" s="69"/>
       <c r="Z7" s="5" t="s">
         <v>2</v>
       </c>
@@ -2136,260 +2005,260 @@
       <c r="AJ7" s="7"/>
     </row>
     <row r="8" spans="2:39" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="92" t="s">
+      <c r="B8" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="93"/>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
+      <c r="C8" s="69"/>
+      <c r="D8" s="69"/>
+      <c r="E8" s="69"/>
+      <c r="F8" s="69"/>
+      <c r="G8" s="69"/>
       <c r="H8" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I8" s="114"/>
-      <c r="J8" s="114"/>
-      <c r="K8" s="114"/>
-      <c r="L8" s="114"/>
-      <c r="M8" s="114"/>
-      <c r="N8" s="114"/>
-      <c r="O8" s="114"/>
-      <c r="P8" s="114"/>
-      <c r="Q8" s="114"/>
-      <c r="S8" s="94" t="s">
+      <c r="I8" s="95"/>
+      <c r="J8" s="95"/>
+      <c r="K8" s="95"/>
+      <c r="L8" s="95"/>
+      <c r="M8" s="95"/>
+      <c r="N8" s="95"/>
+      <c r="O8" s="95"/>
+      <c r="P8" s="95"/>
+      <c r="Q8" s="95"/>
+      <c r="S8" s="69" t="s">
         <v>5</v>
       </c>
-      <c r="T8" s="94"/>
-      <c r="U8" s="94"/>
-      <c r="V8" s="94"/>
-      <c r="W8" s="94"/>
-      <c r="X8" s="94"/>
-      <c r="Y8" s="94"/>
+      <c r="T8" s="69"/>
+      <c r="U8" s="69"/>
+      <c r="V8" s="69"/>
+      <c r="W8" s="69"/>
+      <c r="X8" s="69"/>
+      <c r="Y8" s="69"/>
       <c r="Z8" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="AA8" s="114"/>
-      <c r="AB8" s="114"/>
-      <c r="AC8" s="114"/>
-      <c r="AD8" s="114"/>
-      <c r="AE8" s="114"/>
-      <c r="AF8" s="114"/>
-      <c r="AG8" s="114"/>
-      <c r="AH8" s="114"/>
-      <c r="AI8" s="114"/>
+      <c r="AA8" s="95"/>
+      <c r="AB8" s="95"/>
+      <c r="AC8" s="95"/>
+      <c r="AD8" s="95"/>
+      <c r="AE8" s="95"/>
+      <c r="AF8" s="95"/>
+      <c r="AG8" s="95"/>
+      <c r="AH8" s="95"/>
+      <c r="AI8" s="95"/>
       <c r="AJ8" s="7"/>
     </row>
     <row r="9" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B9" s="92" t="s">
+      <c r="B9" s="93" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="93"/>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
+      <c r="C9" s="69"/>
+      <c r="D9" s="69"/>
+      <c r="E9" s="69"/>
+      <c r="F9" s="69"/>
+      <c r="G9" s="69"/>
       <c r="H9" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I9" s="114"/>
-      <c r="J9" s="114"/>
-      <c r="K9" s="114"/>
-      <c r="L9" s="114"/>
-      <c r="M9" s="114"/>
-      <c r="N9" s="114"/>
-      <c r="O9" s="114"/>
-      <c r="P9" s="114"/>
-      <c r="Q9" s="114"/>
-      <c r="S9" s="93" t="s">
+      <c r="I9" s="95"/>
+      <c r="J9" s="95"/>
+      <c r="K9" s="95"/>
+      <c r="L9" s="95"/>
+      <c r="M9" s="95"/>
+      <c r="N9" s="95"/>
+      <c r="O9" s="95"/>
+      <c r="P9" s="95"/>
+      <c r="Q9" s="95"/>
+      <c r="S9" s="69" t="s">
         <v>7</v>
       </c>
-      <c r="T9" s="93"/>
-      <c r="U9" s="93"/>
-      <c r="V9" s="93"/>
-      <c r="W9" s="93"/>
-      <c r="X9" s="93"/>
-      <c r="Y9" s="93"/>
+      <c r="T9" s="69"/>
+      <c r="U9" s="69"/>
+      <c r="V9" s="69"/>
+      <c r="W9" s="69"/>
+      <c r="X9" s="69"/>
+      <c r="Y9" s="69"/>
       <c r="Z9" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="AA9" s="114"/>
-      <c r="AB9" s="114"/>
-      <c r="AC9" s="114"/>
-      <c r="AD9" s="114"/>
-      <c r="AE9" s="114"/>
-      <c r="AF9" s="114"/>
-      <c r="AG9" s="114"/>
-      <c r="AH9" s="114"/>
-      <c r="AI9" s="114"/>
+      <c r="AA9" s="95"/>
+      <c r="AB9" s="95"/>
+      <c r="AC9" s="95"/>
+      <c r="AD9" s="95"/>
+      <c r="AE9" s="95"/>
+      <c r="AF9" s="95"/>
+      <c r="AG9" s="95"/>
+      <c r="AH9" s="95"/>
+      <c r="AI9" s="95"/>
       <c r="AJ9" s="8"/>
       <c r="AK9" s="9"/>
       <c r="AL9" s="9"/>
       <c r="AM9" s="9"/>
     </row>
     <row r="10" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B10" s="96" t="s">
+      <c r="B10" s="114" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="97"/>
-      <c r="D10" s="97"/>
-      <c r="E10" s="97"/>
-      <c r="F10" s="97"/>
-      <c r="G10" s="97"/>
+      <c r="C10" s="115"/>
+      <c r="D10" s="115"/>
+      <c r="E10" s="115"/>
+      <c r="F10" s="115"/>
+      <c r="G10" s="115"/>
       <c r="H10" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I10" s="114"/>
-      <c r="J10" s="114"/>
-      <c r="K10" s="114"/>
-      <c r="L10" s="114"/>
-      <c r="M10" s="114"/>
-      <c r="N10" s="114"/>
-      <c r="O10" s="114"/>
-      <c r="P10" s="114"/>
-      <c r="Q10" s="114"/>
-      <c r="S10" s="94" t="s">
+      <c r="I10" s="95"/>
+      <c r="J10" s="95"/>
+      <c r="K10" s="95"/>
+      <c r="L10" s="95"/>
+      <c r="M10" s="95"/>
+      <c r="N10" s="95"/>
+      <c r="O10" s="95"/>
+      <c r="P10" s="95"/>
+      <c r="Q10" s="95"/>
+      <c r="S10" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="T10" s="94"/>
-      <c r="U10" s="94"/>
-      <c r="V10" s="94"/>
-      <c r="W10" s="94"/>
-      <c r="X10" s="94"/>
-      <c r="Y10" s="94"/>
+      <c r="T10" s="69"/>
+      <c r="U10" s="69"/>
+      <c r="V10" s="69"/>
+      <c r="W10" s="69"/>
+      <c r="X10" s="69"/>
+      <c r="Y10" s="69"/>
       <c r="Z10" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="AA10" s="116"/>
-      <c r="AB10" s="116"/>
-      <c r="AC10" s="116"/>
-      <c r="AD10" s="116"/>
-      <c r="AE10" s="116"/>
-      <c r="AF10" s="116"/>
-      <c r="AG10" s="116"/>
-      <c r="AH10" s="116"/>
-      <c r="AI10" s="116"/>
+      <c r="AA10" s="97"/>
+      <c r="AB10" s="97"/>
+      <c r="AC10" s="97"/>
+      <c r="AD10" s="97"/>
+      <c r="AE10" s="97"/>
+      <c r="AF10" s="97"/>
+      <c r="AG10" s="97"/>
+      <c r="AH10" s="97"/>
+      <c r="AI10" s="97"/>
       <c r="AJ10" s="8"/>
       <c r="AK10" s="9"/>
       <c r="AL10" s="9"/>
       <c r="AM10" s="9"/>
     </row>
     <row r="11" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B11" s="92" t="s">
+      <c r="B11" s="93" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="93"/>
-      <c r="D11" s="93"/>
-      <c r="E11" s="93"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="93"/>
+      <c r="C11" s="69"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="69"/>
       <c r="H11" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I11" s="114"/>
-      <c r="J11" s="114"/>
-      <c r="K11" s="114"/>
-      <c r="L11" s="114"/>
-      <c r="M11" s="114"/>
-      <c r="N11" s="114"/>
-      <c r="O11" s="114"/>
-      <c r="P11" s="114"/>
-      <c r="Q11" s="114"/>
-      <c r="S11" s="94" t="s">
+      <c r="I11" s="95"/>
+      <c r="J11" s="95"/>
+      <c r="K11" s="95"/>
+      <c r="L11" s="95"/>
+      <c r="M11" s="95"/>
+      <c r="N11" s="95"/>
+      <c r="O11" s="95"/>
+      <c r="P11" s="95"/>
+      <c r="Q11" s="95"/>
+      <c r="S11" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="T11" s="94"/>
-      <c r="U11" s="94"/>
-      <c r="V11" s="94"/>
-      <c r="W11" s="94"/>
-      <c r="X11" s="94"/>
-      <c r="Y11" s="94"/>
+      <c r="T11" s="69"/>
+      <c r="U11" s="69"/>
+      <c r="V11" s="69"/>
+      <c r="W11" s="69"/>
+      <c r="X11" s="69"/>
+      <c r="Y11" s="69"/>
       <c r="Z11" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="AA11" s="116"/>
-      <c r="AB11" s="116"/>
-      <c r="AC11" s="116"/>
-      <c r="AD11" s="116"/>
-      <c r="AE11" s="116"/>
-      <c r="AF11" s="116"/>
-      <c r="AG11" s="116"/>
-      <c r="AH11" s="116"/>
-      <c r="AI11" s="116"/>
+      <c r="AA11" s="97"/>
+      <c r="AB11" s="97"/>
+      <c r="AC11" s="97"/>
+      <c r="AD11" s="97"/>
+      <c r="AE11" s="97"/>
+      <c r="AF11" s="97"/>
+      <c r="AG11" s="97"/>
+      <c r="AH11" s="97"/>
+      <c r="AI11" s="97"/>
       <c r="AJ11" s="8"/>
       <c r="AK11" s="9"/>
       <c r="AL11" s="9"/>
       <c r="AM11" s="9"/>
     </row>
     <row r="12" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B12" s="92" t="s">
+      <c r="B12" s="93" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="93"/>
-      <c r="D12" s="93"/>
-      <c r="E12" s="93"/>
-      <c r="F12" s="93"/>
-      <c r="G12" s="93"/>
+      <c r="C12" s="69"/>
+      <c r="D12" s="69"/>
+      <c r="E12" s="69"/>
+      <c r="F12" s="69"/>
+      <c r="G12" s="69"/>
       <c r="H12" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I12" s="114"/>
-      <c r="J12" s="114"/>
-      <c r="K12" s="114"/>
-      <c r="L12" s="114"/>
-      <c r="M12" s="114"/>
-      <c r="N12" s="114"/>
-      <c r="O12" s="114"/>
-      <c r="P12" s="114"/>
-      <c r="Q12" s="114"/>
-      <c r="S12" s="94" t="s">
+      <c r="I12" s="95"/>
+      <c r="J12" s="95"/>
+      <c r="K12" s="95"/>
+      <c r="L12" s="95"/>
+      <c r="M12" s="95"/>
+      <c r="N12" s="95"/>
+      <c r="O12" s="95"/>
+      <c r="P12" s="95"/>
+      <c r="Q12" s="95"/>
+      <c r="S12" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="T12" s="94"/>
-      <c r="U12" s="94"/>
-      <c r="V12" s="94"/>
-      <c r="W12" s="94"/>
-      <c r="X12" s="94"/>
-      <c r="Y12" s="94"/>
+      <c r="T12" s="69"/>
+      <c r="U12" s="69"/>
+      <c r="V12" s="69"/>
+      <c r="W12" s="69"/>
+      <c r="X12" s="69"/>
+      <c r="Y12" s="69"/>
       <c r="Z12" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="AA12" s="95" t="s">
+      <c r="AA12" s="94" t="s">
         <v>50</v>
       </c>
-      <c r="AB12" s="95"/>
-      <c r="AC12" s="95"/>
-      <c r="AD12" s="95"/>
-      <c r="AE12" s="95"/>
-      <c r="AF12" s="95"/>
-      <c r="AG12" s="95"/>
-      <c r="AH12" s="95"/>
-      <c r="AI12" s="95"/>
+      <c r="AB12" s="94"/>
+      <c r="AC12" s="94"/>
+      <c r="AD12" s="94"/>
+      <c r="AE12" s="94"/>
+      <c r="AF12" s="94"/>
+      <c r="AG12" s="94"/>
+      <c r="AH12" s="94"/>
+      <c r="AI12" s="94"/>
       <c r="AJ12" s="8"/>
       <c r="AK12" s="9"/>
       <c r="AL12" s="9"/>
       <c r="AM12" s="9"/>
     </row>
     <row r="13" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B13" s="92" t="s">
+      <c r="B13" s="93" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="93"/>
-      <c r="D13" s="93"/>
-      <c r="E13" s="93"/>
-      <c r="F13" s="93"/>
-      <c r="G13" s="93"/>
+      <c r="C13" s="69"/>
+      <c r="D13" s="69"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="69"/>
       <c r="H13" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I13" s="114"/>
-      <c r="J13" s="114"/>
-      <c r="K13" s="114"/>
-      <c r="L13" s="114"/>
-      <c r="M13" s="114"/>
-      <c r="N13" s="114"/>
-      <c r="O13" s="114"/>
-      <c r="P13" s="114"/>
-      <c r="Q13" s="114"/>
+      <c r="I13" s="95"/>
+      <c r="J13" s="95"/>
+      <c r="K13" s="95"/>
+      <c r="L13" s="95"/>
+      <c r="M13" s="95"/>
+      <c r="N13" s="95"/>
+      <c r="O13" s="95"/>
+      <c r="P13" s="95"/>
+      <c r="Q13" s="95"/>
       <c r="S13" s="6"/>
       <c r="T13" s="6"/>
       <c r="U13" s="6"/>
@@ -2398,187 +2267,187 @@
       <c r="X13" s="6"/>
       <c r="Y13" s="6"/>
       <c r="Z13" s="10"/>
-      <c r="AA13" s="95"/>
-      <c r="AB13" s="95"/>
-      <c r="AC13" s="95"/>
-      <c r="AD13" s="95"/>
-      <c r="AE13" s="95"/>
-      <c r="AF13" s="95"/>
-      <c r="AG13" s="95"/>
-      <c r="AH13" s="95"/>
-      <c r="AI13" s="95"/>
+      <c r="AA13" s="94"/>
+      <c r="AB13" s="94"/>
+      <c r="AC13" s="94"/>
+      <c r="AD13" s="94"/>
+      <c r="AE13" s="94"/>
+      <c r="AF13" s="94"/>
+      <c r="AG13" s="94"/>
+      <c r="AH13" s="94"/>
+      <c r="AI13" s="94"/>
       <c r="AJ13" s="8"/>
       <c r="AK13" s="9"/>
       <c r="AL13" s="9"/>
       <c r="AM13" s="9"/>
     </row>
     <row r="14" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B14" s="92" t="s">
+      <c r="B14" s="93" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="93"/>
-      <c r="D14" s="93"/>
-      <c r="E14" s="93"/>
-      <c r="F14" s="93"/>
-      <c r="G14" s="93"/>
+      <c r="C14" s="69"/>
+      <c r="D14" s="69"/>
+      <c r="E14" s="69"/>
+      <c r="F14" s="69"/>
+      <c r="G14" s="69"/>
       <c r="H14" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I14" s="114"/>
-      <c r="J14" s="114"/>
-      <c r="K14" s="114"/>
-      <c r="L14" s="114"/>
-      <c r="M14" s="114"/>
-      <c r="N14" s="114"/>
-      <c r="O14" s="114"/>
-      <c r="P14" s="114"/>
-      <c r="Q14" s="114"/>
-      <c r="AA14" s="95"/>
-      <c r="AB14" s="95"/>
-      <c r="AC14" s="95"/>
-      <c r="AD14" s="95"/>
-      <c r="AE14" s="95"/>
-      <c r="AF14" s="95"/>
-      <c r="AG14" s="95"/>
-      <c r="AH14" s="95"/>
-      <c r="AI14" s="95"/>
+      <c r="I14" s="95"/>
+      <c r="J14" s="95"/>
+      <c r="K14" s="95"/>
+      <c r="L14" s="95"/>
+      <c r="M14" s="95"/>
+      <c r="N14" s="95"/>
+      <c r="O14" s="95"/>
+      <c r="P14" s="95"/>
+      <c r="Q14" s="95"/>
+      <c r="AA14" s="94"/>
+      <c r="AB14" s="94"/>
+      <c r="AC14" s="94"/>
+      <c r="AD14" s="94"/>
+      <c r="AE14" s="94"/>
+      <c r="AF14" s="94"/>
+      <c r="AG14" s="94"/>
+      <c r="AH14" s="94"/>
+      <c r="AI14" s="94"/>
       <c r="AJ14" s="8"/>
       <c r="AK14" s="11"/>
       <c r="AL14" s="11"/>
       <c r="AM14" s="11"/>
     </row>
     <row r="15" spans="2:39" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B15" s="92" t="s">
+      <c r="B15" s="93" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="93"/>
-      <c r="D15" s="93"/>
-      <c r="E15" s="93"/>
-      <c r="F15" s="93"/>
-      <c r="G15" s="93"/>
+      <c r="C15" s="69"/>
+      <c r="D15" s="69"/>
+      <c r="E15" s="69"/>
+      <c r="F15" s="69"/>
+      <c r="G15" s="69"/>
       <c r="H15" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I15" s="114"/>
-      <c r="J15" s="114"/>
-      <c r="K15" s="114"/>
-      <c r="L15" s="114"/>
-      <c r="M15" s="114"/>
-      <c r="N15" s="114"/>
-      <c r="O15" s="114"/>
-      <c r="P15" s="114"/>
-      <c r="Q15" s="114"/>
-      <c r="AA15" s="95"/>
-      <c r="AB15" s="95"/>
-      <c r="AC15" s="95"/>
-      <c r="AD15" s="95"/>
-      <c r="AE15" s="95"/>
-      <c r="AF15" s="95"/>
-      <c r="AG15" s="95"/>
-      <c r="AH15" s="95"/>
-      <c r="AI15" s="95"/>
+      <c r="I15" s="95"/>
+      <c r="J15" s="95"/>
+      <c r="K15" s="95"/>
+      <c r="L15" s="95"/>
+      <c r="M15" s="95"/>
+      <c r="N15" s="95"/>
+      <c r="O15" s="95"/>
+      <c r="P15" s="95"/>
+      <c r="Q15" s="95"/>
+      <c r="AA15" s="94"/>
+      <c r="AB15" s="94"/>
+      <c r="AC15" s="94"/>
+      <c r="AD15" s="94"/>
+      <c r="AE15" s="94"/>
+      <c r="AF15" s="94"/>
+      <c r="AG15" s="94"/>
+      <c r="AH15" s="94"/>
+      <c r="AI15" s="94"/>
       <c r="AJ15" s="7"/>
     </row>
     <row r="16" spans="2:39" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="92" t="s">
+      <c r="B16" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="93"/>
-      <c r="D16" s="93"/>
-      <c r="E16" s="93"/>
-      <c r="F16" s="93"/>
-      <c r="G16" s="93"/>
+      <c r="C16" s="69"/>
+      <c r="D16" s="69"/>
+      <c r="E16" s="69"/>
+      <c r="F16" s="69"/>
+      <c r="G16" s="69"/>
       <c r="H16" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I16" s="114"/>
-      <c r="J16" s="114"/>
-      <c r="K16" s="114"/>
-      <c r="L16" s="114"/>
-      <c r="M16" s="114"/>
-      <c r="N16" s="114"/>
-      <c r="O16" s="114"/>
-      <c r="P16" s="114"/>
-      <c r="Q16" s="114"/>
-      <c r="AA16" s="95"/>
-      <c r="AB16" s="95"/>
-      <c r="AC16" s="95"/>
-      <c r="AD16" s="95"/>
-      <c r="AE16" s="95"/>
-      <c r="AF16" s="95"/>
-      <c r="AG16" s="95"/>
-      <c r="AH16" s="95"/>
-      <c r="AI16" s="95"/>
+      <c r="I16" s="95"/>
+      <c r="J16" s="95"/>
+      <c r="K16" s="95"/>
+      <c r="L16" s="95"/>
+      <c r="M16" s="95"/>
+      <c r="N16" s="95"/>
+      <c r="O16" s="95"/>
+      <c r="P16" s="95"/>
+      <c r="Q16" s="95"/>
+      <c r="AA16" s="94"/>
+      <c r="AB16" s="94"/>
+      <c r="AC16" s="94"/>
+      <c r="AD16" s="94"/>
+      <c r="AE16" s="94"/>
+      <c r="AF16" s="94"/>
+      <c r="AG16" s="94"/>
+      <c r="AH16" s="94"/>
+      <c r="AI16" s="94"/>
       <c r="AJ16" s="7"/>
     </row>
     <row r="17" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B17" s="92" t="s">
+      <c r="B17" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="93"/>
-      <c r="D17" s="93"/>
-      <c r="E17" s="93"/>
-      <c r="F17" s="93"/>
-      <c r="G17" s="93"/>
+      <c r="C17" s="69"/>
+      <c r="D17" s="69"/>
+      <c r="E17" s="69"/>
+      <c r="F17" s="69"/>
+      <c r="G17" s="69"/>
       <c r="H17" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I17" s="115"/>
-      <c r="J17" s="115"/>
-      <c r="K17" s="115"/>
-      <c r="L17" s="115"/>
-      <c r="M17" s="115"/>
-      <c r="N17" s="115"/>
-      <c r="O17" s="115"/>
-      <c r="P17" s="115"/>
-      <c r="Q17" s="115"/>
-      <c r="AA17" s="95"/>
-      <c r="AB17" s="95"/>
-      <c r="AC17" s="95"/>
-      <c r="AD17" s="95"/>
-      <c r="AE17" s="95"/>
-      <c r="AF17" s="95"/>
-      <c r="AG17" s="95"/>
-      <c r="AH17" s="95"/>
-      <c r="AI17" s="95"/>
+      <c r="I17" s="96"/>
+      <c r="J17" s="96"/>
+      <c r="K17" s="96"/>
+      <c r="L17" s="96"/>
+      <c r="M17" s="96"/>
+      <c r="N17" s="96"/>
+      <c r="O17" s="96"/>
+      <c r="P17" s="96"/>
+      <c r="Q17" s="96"/>
+      <c r="AA17" s="94"/>
+      <c r="AB17" s="94"/>
+      <c r="AC17" s="94"/>
+      <c r="AD17" s="94"/>
+      <c r="AE17" s="94"/>
+      <c r="AF17" s="94"/>
+      <c r="AG17" s="94"/>
+      <c r="AH17" s="94"/>
+      <c r="AI17" s="94"/>
       <c r="AJ17" s="7"/>
     </row>
     <row r="18" spans="2:36" ht="3" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="75"/>
-      <c r="C18" s="76"/>
-      <c r="D18" s="76"/>
-      <c r="E18" s="76"/>
-      <c r="F18" s="76"/>
-      <c r="G18" s="76"/>
-      <c r="H18" s="76"/>
-      <c r="I18" s="76"/>
-      <c r="J18" s="76"/>
-      <c r="K18" s="76"/>
-      <c r="L18" s="76"/>
-      <c r="M18" s="76"/>
-      <c r="N18" s="76"/>
-      <c r="O18" s="76"/>
-      <c r="P18" s="76"/>
-      <c r="Q18" s="76"/>
-      <c r="R18" s="76"/>
-      <c r="S18" s="76"/>
-      <c r="T18" s="76"/>
-      <c r="U18" s="76"/>
-      <c r="V18" s="76"/>
-      <c r="W18" s="76"/>
-      <c r="X18" s="76"/>
-      <c r="Y18" s="76"/>
-      <c r="Z18" s="76"/>
-      <c r="AA18" s="76"/>
-      <c r="AB18" s="76"/>
-      <c r="AC18" s="76"/>
-      <c r="AD18" s="76"/>
-      <c r="AE18" s="76"/>
-      <c r="AF18" s="76"/>
-      <c r="AG18" s="76"/>
-      <c r="AH18" s="76"/>
-      <c r="AI18" s="76"/>
-      <c r="AJ18" s="77"/>
+      <c r="B18" s="76"/>
+      <c r="C18" s="77"/>
+      <c r="D18" s="77"/>
+      <c r="E18" s="77"/>
+      <c r="F18" s="77"/>
+      <c r="G18" s="77"/>
+      <c r="H18" s="77"/>
+      <c r="I18" s="77"/>
+      <c r="J18" s="77"/>
+      <c r="K18" s="77"/>
+      <c r="L18" s="77"/>
+      <c r="M18" s="77"/>
+      <c r="N18" s="77"/>
+      <c r="O18" s="77"/>
+      <c r="P18" s="77"/>
+      <c r="Q18" s="77"/>
+      <c r="R18" s="77"/>
+      <c r="S18" s="77"/>
+      <c r="T18" s="77"/>
+      <c r="U18" s="77"/>
+      <c r="V18" s="77"/>
+      <c r="W18" s="77"/>
+      <c r="X18" s="77"/>
+      <c r="Y18" s="77"/>
+      <c r="Z18" s="77"/>
+      <c r="AA18" s="77"/>
+      <c r="AB18" s="77"/>
+      <c r="AC18" s="77"/>
+      <c r="AD18" s="77"/>
+      <c r="AE18" s="77"/>
+      <c r="AF18" s="77"/>
+      <c r="AG18" s="77"/>
+      <c r="AH18" s="77"/>
+      <c r="AI18" s="77"/>
+      <c r="AJ18" s="78"/>
     </row>
     <row r="19" spans="2:36" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B19" s="2"/>
@@ -2596,14 +2465,14 @@
       <c r="N19" s="3"/>
       <c r="O19" s="3"/>
       <c r="P19" s="12"/>
-      <c r="Q19" s="78" t="s">
+      <c r="Q19" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="R19" s="79"/>
-      <c r="S19" s="79"/>
-      <c r="T19" s="79"/>
-      <c r="U19" s="79"/>
-      <c r="V19" s="79"/>
+      <c r="R19" s="80"/>
+      <c r="S19" s="80"/>
+      <c r="T19" s="80"/>
+      <c r="U19" s="80"/>
+      <c r="V19" s="80"/>
       <c r="W19" s="12"/>
       <c r="X19" s="3"/>
       <c r="Y19" s="3"/>
@@ -2625,170 +2494,170 @@
     </row>
     <row r="21" spans="2:36" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="14"/>
-      <c r="C21" s="80" t="s">
+      <c r="C21" s="81" t="s">
         <v>21</v>
       </c>
-      <c r="D21" s="81" t="s">
+      <c r="D21" s="82" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="82"/>
-      <c r="F21" s="82"/>
-      <c r="G21" s="82"/>
-      <c r="H21" s="82"/>
-      <c r="I21" s="82"/>
-      <c r="J21" s="82"/>
-      <c r="K21" s="83"/>
-      <c r="L21" s="90" t="s">
+      <c r="E21" s="83"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="83"/>
+      <c r="H21" s="83"/>
+      <c r="I21" s="83"/>
+      <c r="J21" s="83"/>
+      <c r="K21" s="84"/>
+      <c r="L21" s="91" t="s">
         <v>23</v>
       </c>
-      <c r="M21" s="90"/>
-      <c r="N21" s="90"/>
-      <c r="O21" s="90"/>
-      <c r="P21" s="90"/>
-      <c r="Q21" s="90"/>
-      <c r="R21" s="90" t="s">
+      <c r="M21" s="91"/>
+      <c r="N21" s="91"/>
+      <c r="O21" s="91"/>
+      <c r="P21" s="91"/>
+      <c r="Q21" s="91"/>
+      <c r="R21" s="91" t="s">
         <v>24</v>
       </c>
-      <c r="S21" s="90"/>
-      <c r="T21" s="90"/>
-      <c r="U21" s="90"/>
-      <c r="V21" s="90"/>
-      <c r="W21" s="90"/>
-      <c r="X21" s="91" t="s">
+      <c r="S21" s="91"/>
+      <c r="T21" s="91"/>
+      <c r="U21" s="91"/>
+      <c r="V21" s="91"/>
+      <c r="W21" s="91"/>
+      <c r="X21" s="92" t="s">
         <v>25</v>
       </c>
-      <c r="Y21" s="91"/>
-      <c r="Z21" s="91"/>
-      <c r="AA21" s="91"/>
-      <c r="AB21" s="91"/>
-      <c r="AC21" s="91"/>
-      <c r="AD21" s="81" t="s">
+      <c r="Y21" s="92"/>
+      <c r="Z21" s="92"/>
+      <c r="AA21" s="92"/>
+      <c r="AB21" s="92"/>
+      <c r="AC21" s="92"/>
+      <c r="AD21" s="82" t="s">
         <v>26</v>
       </c>
-      <c r="AE21" s="82"/>
-      <c r="AF21" s="82"/>
-      <c r="AG21" s="82"/>
-      <c r="AH21" s="82"/>
-      <c r="AI21" s="83"/>
+      <c r="AE21" s="83"/>
+      <c r="AF21" s="83"/>
+      <c r="AG21" s="83"/>
+      <c r="AH21" s="83"/>
+      <c r="AI21" s="84"/>
       <c r="AJ21" s="7"/>
     </row>
     <row r="22" spans="2:36" ht="3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="14"/>
       <c r="C22" s="50"/>
-      <c r="D22" s="84"/>
-      <c r="E22" s="85"/>
-      <c r="F22" s="85"/>
-      <c r="G22" s="85"/>
-      <c r="H22" s="85"/>
-      <c r="I22" s="85"/>
-      <c r="J22" s="85"/>
-      <c r="K22" s="86"/>
-      <c r="L22" s="90"/>
-      <c r="M22" s="90"/>
-      <c r="N22" s="90"/>
-      <c r="O22" s="90"/>
-      <c r="P22" s="90"/>
-      <c r="Q22" s="90"/>
-      <c r="R22" s="90"/>
-      <c r="S22" s="90"/>
-      <c r="T22" s="90"/>
-      <c r="U22" s="90"/>
-      <c r="V22" s="90"/>
-      <c r="W22" s="90"/>
-      <c r="X22" s="91"/>
-      <c r="Y22" s="91"/>
-      <c r="Z22" s="91"/>
-      <c r="AA22" s="91"/>
-      <c r="AB22" s="91"/>
-      <c r="AC22" s="91"/>
-      <c r="AD22" s="84"/>
-      <c r="AE22" s="85"/>
-      <c r="AF22" s="85"/>
-      <c r="AG22" s="85"/>
-      <c r="AH22" s="85"/>
-      <c r="AI22" s="86"/>
+      <c r="D22" s="85"/>
+      <c r="E22" s="86"/>
+      <c r="F22" s="86"/>
+      <c r="G22" s="86"/>
+      <c r="H22" s="86"/>
+      <c r="I22" s="86"/>
+      <c r="J22" s="86"/>
+      <c r="K22" s="87"/>
+      <c r="L22" s="91"/>
+      <c r="M22" s="91"/>
+      <c r="N22" s="91"/>
+      <c r="O22" s="91"/>
+      <c r="P22" s="91"/>
+      <c r="Q22" s="91"/>
+      <c r="R22" s="91"/>
+      <c r="S22" s="91"/>
+      <c r="T22" s="91"/>
+      <c r="U22" s="91"/>
+      <c r="V22" s="91"/>
+      <c r="W22" s="91"/>
+      <c r="X22" s="92"/>
+      <c r="Y22" s="92"/>
+      <c r="Z22" s="92"/>
+      <c r="AA22" s="92"/>
+      <c r="AB22" s="92"/>
+      <c r="AC22" s="92"/>
+      <c r="AD22" s="85"/>
+      <c r="AE22" s="86"/>
+      <c r="AF22" s="86"/>
+      <c r="AG22" s="86"/>
+      <c r="AH22" s="86"/>
+      <c r="AI22" s="87"/>
       <c r="AJ22" s="7"/>
     </row>
     <row r="23" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="14"/>
       <c r="C23" s="50"/>
-      <c r="D23" s="87"/>
-      <c r="E23" s="88"/>
-      <c r="F23" s="88"/>
-      <c r="G23" s="88"/>
-      <c r="H23" s="88"/>
-      <c r="I23" s="88"/>
-      <c r="J23" s="88"/>
-      <c r="K23" s="89"/>
-      <c r="L23" s="90"/>
-      <c r="M23" s="90"/>
-      <c r="N23" s="90"/>
-      <c r="O23" s="90"/>
-      <c r="P23" s="90"/>
-      <c r="Q23" s="90"/>
-      <c r="R23" s="90"/>
-      <c r="S23" s="90"/>
-      <c r="T23" s="90"/>
-      <c r="U23" s="90"/>
-      <c r="V23" s="90"/>
-      <c r="W23" s="90"/>
-      <c r="X23" s="91"/>
-      <c r="Y23" s="91"/>
-      <c r="Z23" s="91"/>
-      <c r="AA23" s="91"/>
-      <c r="AB23" s="91"/>
-      <c r="AC23" s="91"/>
-      <c r="AD23" s="84"/>
-      <c r="AE23" s="85"/>
-      <c r="AF23" s="85"/>
-      <c r="AG23" s="85"/>
-      <c r="AH23" s="85"/>
-      <c r="AI23" s="86"/>
+      <c r="D23" s="88"/>
+      <c r="E23" s="89"/>
+      <c r="F23" s="89"/>
+      <c r="G23" s="89"/>
+      <c r="H23" s="89"/>
+      <c r="I23" s="89"/>
+      <c r="J23" s="89"/>
+      <c r="K23" s="90"/>
+      <c r="L23" s="91"/>
+      <c r="M23" s="91"/>
+      <c r="N23" s="91"/>
+      <c r="O23" s="91"/>
+      <c r="P23" s="91"/>
+      <c r="Q23" s="91"/>
+      <c r="R23" s="91"/>
+      <c r="S23" s="91"/>
+      <c r="T23" s="91"/>
+      <c r="U23" s="91"/>
+      <c r="V23" s="91"/>
+      <c r="W23" s="91"/>
+      <c r="X23" s="92"/>
+      <c r="Y23" s="92"/>
+      <c r="Z23" s="92"/>
+      <c r="AA23" s="92"/>
+      <c r="AB23" s="92"/>
+      <c r="AC23" s="92"/>
+      <c r="AD23" s="85"/>
+      <c r="AE23" s="86"/>
+      <c r="AF23" s="86"/>
+      <c r="AG23" s="86"/>
+      <c r="AH23" s="86"/>
+      <c r="AI23" s="87"/>
       <c r="AJ23" s="7"/>
     </row>
     <row r="24" spans="2:36" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="14"/>
       <c r="C24" s="50"/>
-      <c r="D24" s="63" t="s">
+      <c r="D24" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="E24" s="64"/>
-      <c r="F24" s="64"/>
-      <c r="G24" s="64"/>
-      <c r="H24" s="64"/>
-      <c r="I24" s="64"/>
-      <c r="J24" s="64"/>
-      <c r="K24" s="65"/>
-      <c r="L24" s="63" t="s">
+      <c r="E24" s="53"/>
+      <c r="F24" s="53"/>
+      <c r="G24" s="53"/>
+      <c r="H24" s="53"/>
+      <c r="I24" s="53"/>
+      <c r="J24" s="53"/>
+      <c r="K24" s="54"/>
+      <c r="L24" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="M24" s="64"/>
-      <c r="N24" s="64"/>
-      <c r="O24" s="64"/>
-      <c r="P24" s="64"/>
-      <c r="Q24" s="65"/>
-      <c r="R24" s="63" t="s">
+      <c r="M24" s="53"/>
+      <c r="N24" s="53"/>
+      <c r="O24" s="53"/>
+      <c r="P24" s="53"/>
+      <c r="Q24" s="54"/>
+      <c r="R24" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="S24" s="64"/>
-      <c r="T24" s="64"/>
-      <c r="U24" s="64"/>
-      <c r="V24" s="64"/>
-      <c r="W24" s="65"/>
-      <c r="X24" s="63" t="s">
+      <c r="S24" s="53"/>
+      <c r="T24" s="53"/>
+      <c r="U24" s="53"/>
+      <c r="V24" s="53"/>
+      <c r="W24" s="54"/>
+      <c r="X24" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="Y24" s="64"/>
-      <c r="Z24" s="64"/>
-      <c r="AA24" s="64"/>
-      <c r="AB24" s="64"/>
-      <c r="AC24" s="65"/>
-      <c r="AD24" s="84"/>
-      <c r="AE24" s="85"/>
-      <c r="AF24" s="85"/>
-      <c r="AG24" s="85"/>
-      <c r="AH24" s="85"/>
-      <c r="AI24" s="86"/>
+      <c r="Y24" s="53"/>
+      <c r="Z24" s="53"/>
+      <c r="AA24" s="53"/>
+      <c r="AB24" s="53"/>
+      <c r="AC24" s="54"/>
+      <c r="AD24" s="85"/>
+      <c r="AE24" s="86"/>
+      <c r="AF24" s="86"/>
+      <c r="AG24" s="86"/>
+      <c r="AH24" s="86"/>
+      <c r="AI24" s="87"/>
       <c r="AJ24" s="7"/>
     </row>
     <row r="25" spans="2:36" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -2835,32 +2704,32 @@
       <c r="C26" s="15">
         <v>1</v>
       </c>
-      <c r="D26" s="69"/>
-      <c r="E26" s="70"/>
-      <c r="F26" s="70"/>
-      <c r="G26" s="70"/>
-      <c r="H26" s="70"/>
-      <c r="I26" s="70"/>
-      <c r="J26" s="70"/>
-      <c r="K26" s="71"/>
-      <c r="L26" s="69"/>
-      <c r="M26" s="70"/>
-      <c r="N26" s="70"/>
-      <c r="O26" s="70"/>
-      <c r="P26" s="70"/>
-      <c r="Q26" s="71"/>
-      <c r="R26" s="69"/>
-      <c r="S26" s="70"/>
-      <c r="T26" s="70"/>
-      <c r="U26" s="70"/>
-      <c r="V26" s="70"/>
-      <c r="W26" s="71"/>
-      <c r="X26" s="72"/>
-      <c r="Y26" s="73"/>
-      <c r="Z26" s="73"/>
-      <c r="AA26" s="73"/>
-      <c r="AB26" s="73"/>
-      <c r="AC26" s="74"/>
+      <c r="D26" s="70"/>
+      <c r="E26" s="71"/>
+      <c r="F26" s="71"/>
+      <c r="G26" s="71"/>
+      <c r="H26" s="71"/>
+      <c r="I26" s="71"/>
+      <c r="J26" s="71"/>
+      <c r="K26" s="72"/>
+      <c r="L26" s="70"/>
+      <c r="M26" s="71"/>
+      <c r="N26" s="71"/>
+      <c r="O26" s="71"/>
+      <c r="P26" s="71"/>
+      <c r="Q26" s="72"/>
+      <c r="R26" s="70"/>
+      <c r="S26" s="71"/>
+      <c r="T26" s="71"/>
+      <c r="U26" s="71"/>
+      <c r="V26" s="71"/>
+      <c r="W26" s="72"/>
+      <c r="X26" s="73"/>
+      <c r="Y26" s="74"/>
+      <c r="Z26" s="74"/>
+      <c r="AA26" s="74"/>
+      <c r="AB26" s="74"/>
+      <c r="AC26" s="75"/>
       <c r="AD26" s="26"/>
       <c r="AE26" s="27"/>
       <c r="AF26" s="27"/>
@@ -2874,32 +2743,32 @@
       <c r="C27" s="15">
         <v>2</v>
       </c>
-      <c r="D27" s="69"/>
-      <c r="E27" s="70"/>
-      <c r="F27" s="70"/>
-      <c r="G27" s="70"/>
-      <c r="H27" s="70"/>
-      <c r="I27" s="70"/>
-      <c r="J27" s="70"/>
-      <c r="K27" s="71"/>
-      <c r="L27" s="69"/>
-      <c r="M27" s="70"/>
-      <c r="N27" s="70"/>
-      <c r="O27" s="70"/>
-      <c r="P27" s="70"/>
-      <c r="Q27" s="71"/>
-      <c r="R27" s="69"/>
-      <c r="S27" s="70"/>
-      <c r="T27" s="70"/>
-      <c r="U27" s="70"/>
-      <c r="V27" s="70"/>
-      <c r="W27" s="71"/>
-      <c r="X27" s="72"/>
-      <c r="Y27" s="73"/>
-      <c r="Z27" s="73"/>
-      <c r="AA27" s="73"/>
-      <c r="AB27" s="73"/>
-      <c r="AC27" s="74"/>
+      <c r="D27" s="70"/>
+      <c r="E27" s="71"/>
+      <c r="F27" s="71"/>
+      <c r="G27" s="71"/>
+      <c r="H27" s="71"/>
+      <c r="I27" s="71"/>
+      <c r="J27" s="71"/>
+      <c r="K27" s="72"/>
+      <c r="L27" s="70"/>
+      <c r="M27" s="71"/>
+      <c r="N27" s="71"/>
+      <c r="O27" s="71"/>
+      <c r="P27" s="71"/>
+      <c r="Q27" s="72"/>
+      <c r="R27" s="70"/>
+      <c r="S27" s="71"/>
+      <c r="T27" s="71"/>
+      <c r="U27" s="71"/>
+      <c r="V27" s="71"/>
+      <c r="W27" s="72"/>
+      <c r="X27" s="73"/>
+      <c r="Y27" s="74"/>
+      <c r="Z27" s="74"/>
+      <c r="AA27" s="74"/>
+      <c r="AB27" s="74"/>
+      <c r="AC27" s="75"/>
       <c r="AD27" s="26"/>
       <c r="AE27" s="27"/>
       <c r="AF27" s="27"/>
@@ -2913,32 +2782,32 @@
       <c r="C28" s="15">
         <v>3</v>
       </c>
-      <c r="D28" s="69"/>
-      <c r="E28" s="70"/>
-      <c r="F28" s="70"/>
-      <c r="G28" s="70"/>
-      <c r="H28" s="70"/>
-      <c r="I28" s="70"/>
-      <c r="J28" s="70"/>
-      <c r="K28" s="71"/>
-      <c r="L28" s="69"/>
-      <c r="M28" s="70"/>
-      <c r="N28" s="70"/>
-      <c r="O28" s="70"/>
-      <c r="P28" s="70"/>
-      <c r="Q28" s="71"/>
-      <c r="R28" s="69"/>
-      <c r="S28" s="70"/>
-      <c r="T28" s="70"/>
-      <c r="U28" s="70"/>
-      <c r="V28" s="70"/>
-      <c r="W28" s="71"/>
-      <c r="X28" s="72"/>
-      <c r="Y28" s="73"/>
-      <c r="Z28" s="73"/>
-      <c r="AA28" s="73"/>
-      <c r="AB28" s="73"/>
-      <c r="AC28" s="74"/>
+      <c r="D28" s="70"/>
+      <c r="E28" s="71"/>
+      <c r="F28" s="71"/>
+      <c r="G28" s="71"/>
+      <c r="H28" s="71"/>
+      <c r="I28" s="71"/>
+      <c r="J28" s="71"/>
+      <c r="K28" s="72"/>
+      <c r="L28" s="70"/>
+      <c r="M28" s="71"/>
+      <c r="N28" s="71"/>
+      <c r="O28" s="71"/>
+      <c r="P28" s="71"/>
+      <c r="Q28" s="72"/>
+      <c r="R28" s="70"/>
+      <c r="S28" s="71"/>
+      <c r="T28" s="71"/>
+      <c r="U28" s="71"/>
+      <c r="V28" s="71"/>
+      <c r="W28" s="72"/>
+      <c r="X28" s="73"/>
+      <c r="Y28" s="74"/>
+      <c r="Z28" s="74"/>
+      <c r="AA28" s="74"/>
+      <c r="AB28" s="74"/>
+      <c r="AC28" s="75"/>
       <c r="AD28" s="26"/>
       <c r="AE28" s="27"/>
       <c r="AF28" s="27"/>
@@ -2952,32 +2821,32 @@
       <c r="C29" s="15">
         <v>4</v>
       </c>
-      <c r="D29" s="69"/>
-      <c r="E29" s="70"/>
-      <c r="F29" s="70"/>
-      <c r="G29" s="70"/>
-      <c r="H29" s="70"/>
-      <c r="I29" s="70"/>
-      <c r="J29" s="70"/>
-      <c r="K29" s="71"/>
-      <c r="L29" s="69"/>
-      <c r="M29" s="70"/>
-      <c r="N29" s="70"/>
-      <c r="O29" s="70"/>
-      <c r="P29" s="70"/>
-      <c r="Q29" s="71"/>
-      <c r="R29" s="69"/>
-      <c r="S29" s="70"/>
-      <c r="T29" s="70"/>
-      <c r="U29" s="70"/>
-      <c r="V29" s="70"/>
-      <c r="W29" s="71"/>
-      <c r="X29" s="72"/>
-      <c r="Y29" s="73"/>
-      <c r="Z29" s="73"/>
-      <c r="AA29" s="73"/>
-      <c r="AB29" s="73"/>
-      <c r="AC29" s="74"/>
+      <c r="D29" s="70"/>
+      <c r="E29" s="71"/>
+      <c r="F29" s="71"/>
+      <c r="G29" s="71"/>
+      <c r="H29" s="71"/>
+      <c r="I29" s="71"/>
+      <c r="J29" s="71"/>
+      <c r="K29" s="72"/>
+      <c r="L29" s="70"/>
+      <c r="M29" s="71"/>
+      <c r="N29" s="71"/>
+      <c r="O29" s="71"/>
+      <c r="P29" s="71"/>
+      <c r="Q29" s="72"/>
+      <c r="R29" s="70"/>
+      <c r="S29" s="71"/>
+      <c r="T29" s="71"/>
+      <c r="U29" s="71"/>
+      <c r="V29" s="71"/>
+      <c r="W29" s="72"/>
+      <c r="X29" s="73"/>
+      <c r="Y29" s="74"/>
+      <c r="Z29" s="74"/>
+      <c r="AA29" s="74"/>
+      <c r="AB29" s="74"/>
+      <c r="AC29" s="75"/>
       <c r="AD29" s="26"/>
       <c r="AE29" s="27"/>
       <c r="AF29" s="27"/>
@@ -2991,32 +2860,32 @@
       <c r="C30" s="15">
         <v>5</v>
       </c>
-      <c r="D30" s="69"/>
-      <c r="E30" s="70"/>
-      <c r="F30" s="70"/>
-      <c r="G30" s="70"/>
-      <c r="H30" s="70"/>
-      <c r="I30" s="70"/>
-      <c r="J30" s="70"/>
-      <c r="K30" s="71"/>
-      <c r="L30" s="69"/>
-      <c r="M30" s="70"/>
-      <c r="N30" s="70"/>
-      <c r="O30" s="70"/>
-      <c r="P30" s="70"/>
-      <c r="Q30" s="71"/>
-      <c r="R30" s="69"/>
-      <c r="S30" s="70"/>
-      <c r="T30" s="70"/>
-      <c r="U30" s="70"/>
-      <c r="V30" s="70"/>
-      <c r="W30" s="71"/>
-      <c r="X30" s="72"/>
-      <c r="Y30" s="73"/>
-      <c r="Z30" s="73"/>
-      <c r="AA30" s="73"/>
-      <c r="AB30" s="73"/>
-      <c r="AC30" s="74"/>
+      <c r="D30" s="70"/>
+      <c r="E30" s="71"/>
+      <c r="F30" s="71"/>
+      <c r="G30" s="71"/>
+      <c r="H30" s="71"/>
+      <c r="I30" s="71"/>
+      <c r="J30" s="71"/>
+      <c r="K30" s="72"/>
+      <c r="L30" s="70"/>
+      <c r="M30" s="71"/>
+      <c r="N30" s="71"/>
+      <c r="O30" s="71"/>
+      <c r="P30" s="71"/>
+      <c r="Q30" s="72"/>
+      <c r="R30" s="70"/>
+      <c r="S30" s="71"/>
+      <c r="T30" s="71"/>
+      <c r="U30" s="71"/>
+      <c r="V30" s="71"/>
+      <c r="W30" s="72"/>
+      <c r="X30" s="73"/>
+      <c r="Y30" s="74"/>
+      <c r="Z30" s="74"/>
+      <c r="AA30" s="74"/>
+      <c r="AB30" s="74"/>
+      <c r="AC30" s="75"/>
       <c r="AD30" s="23"/>
       <c r="AE30" s="24"/>
       <c r="AF30" s="24"/>
@@ -3030,32 +2899,32 @@
       <c r="C31" s="15">
         <v>6</v>
       </c>
-      <c r="D31" s="63"/>
-      <c r="E31" s="64"/>
-      <c r="F31" s="64"/>
-      <c r="G31" s="64"/>
-      <c r="H31" s="64"/>
-      <c r="I31" s="64"/>
-      <c r="J31" s="64"/>
-      <c r="K31" s="65"/>
-      <c r="L31" s="66"/>
-      <c r="M31" s="67"/>
-      <c r="N31" s="67"/>
-      <c r="O31" s="67"/>
-      <c r="P31" s="67"/>
-      <c r="Q31" s="68"/>
-      <c r="R31" s="66"/>
-      <c r="S31" s="67"/>
-      <c r="T31" s="67"/>
-      <c r="U31" s="67"/>
-      <c r="V31" s="67"/>
-      <c r="W31" s="68"/>
-      <c r="X31" s="66"/>
-      <c r="Y31" s="67"/>
-      <c r="Z31" s="67"/>
-      <c r="AA31" s="67"/>
-      <c r="AB31" s="67"/>
-      <c r="AC31" s="68"/>
+      <c r="D31" s="52"/>
+      <c r="E31" s="53"/>
+      <c r="F31" s="53"/>
+      <c r="G31" s="53"/>
+      <c r="H31" s="53"/>
+      <c r="I31" s="53"/>
+      <c r="J31" s="53"/>
+      <c r="K31" s="54"/>
+      <c r="L31" s="55"/>
+      <c r="M31" s="56"/>
+      <c r="N31" s="56"/>
+      <c r="O31" s="56"/>
+      <c r="P31" s="56"/>
+      <c r="Q31" s="57"/>
+      <c r="R31" s="55"/>
+      <c r="S31" s="56"/>
+      <c r="T31" s="56"/>
+      <c r="U31" s="56"/>
+      <c r="V31" s="56"/>
+      <c r="W31" s="57"/>
+      <c r="X31" s="55"/>
+      <c r="Y31" s="56"/>
+      <c r="Z31" s="56"/>
+      <c r="AA31" s="56"/>
+      <c r="AB31" s="56"/>
+      <c r="AC31" s="57"/>
       <c r="AD31" s="29"/>
       <c r="AE31" s="30"/>
       <c r="AF31" s="30"/>
@@ -3069,32 +2938,32 @@
       <c r="C32" s="15">
         <v>7</v>
       </c>
-      <c r="D32" s="63"/>
-      <c r="E32" s="64"/>
-      <c r="F32" s="64"/>
-      <c r="G32" s="64"/>
-      <c r="H32" s="64"/>
-      <c r="I32" s="64"/>
-      <c r="J32" s="64"/>
-      <c r="K32" s="65"/>
-      <c r="L32" s="66"/>
-      <c r="M32" s="67"/>
-      <c r="N32" s="67"/>
-      <c r="O32" s="67"/>
-      <c r="P32" s="67"/>
-      <c r="Q32" s="68"/>
-      <c r="R32" s="66"/>
-      <c r="S32" s="67"/>
-      <c r="T32" s="67"/>
-      <c r="U32" s="67"/>
-      <c r="V32" s="67"/>
-      <c r="W32" s="68"/>
-      <c r="X32" s="66"/>
-      <c r="Y32" s="67"/>
-      <c r="Z32" s="67"/>
-      <c r="AA32" s="67"/>
-      <c r="AB32" s="67"/>
-      <c r="AC32" s="68"/>
+      <c r="D32" s="52"/>
+      <c r="E32" s="53"/>
+      <c r="F32" s="53"/>
+      <c r="G32" s="53"/>
+      <c r="H32" s="53"/>
+      <c r="I32" s="53"/>
+      <c r="J32" s="53"/>
+      <c r="K32" s="54"/>
+      <c r="L32" s="55"/>
+      <c r="M32" s="56"/>
+      <c r="N32" s="56"/>
+      <c r="O32" s="56"/>
+      <c r="P32" s="56"/>
+      <c r="Q32" s="57"/>
+      <c r="R32" s="55"/>
+      <c r="S32" s="56"/>
+      <c r="T32" s="56"/>
+      <c r="U32" s="56"/>
+      <c r="V32" s="56"/>
+      <c r="W32" s="57"/>
+      <c r="X32" s="55"/>
+      <c r="Y32" s="56"/>
+      <c r="Z32" s="56"/>
+      <c r="AA32" s="56"/>
+      <c r="AB32" s="56"/>
+      <c r="AC32" s="57"/>
       <c r="AD32" s="32"/>
       <c r="AE32" s="33"/>
       <c r="AF32" s="33"/>
@@ -3105,337 +2974,337 @@
     </row>
     <row r="33" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="14"/>
-      <c r="C33" s="52" t="s">
+      <c r="C33" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="D33" s="52"/>
-      <c r="E33" s="52"/>
-      <c r="F33" s="52"/>
-      <c r="G33" s="52"/>
-      <c r="H33" s="52"/>
-      <c r="I33" s="52"/>
-      <c r="J33" s="52"/>
-      <c r="K33" s="52"/>
-      <c r="L33" s="52"/>
-      <c r="M33" s="52"/>
-      <c r="N33" s="52"/>
-      <c r="O33" s="52"/>
-      <c r="P33" s="52"/>
-      <c r="Q33" s="52"/>
-      <c r="R33" s="52"/>
-      <c r="S33" s="52"/>
-      <c r="T33" s="52"/>
-      <c r="U33" s="52"/>
-      <c r="V33" s="52"/>
-      <c r="W33" s="52"/>
-      <c r="X33" s="52"/>
-      <c r="Y33" s="52"/>
-      <c r="Z33" s="52"/>
-      <c r="AA33" s="52"/>
-      <c r="AB33" s="52"/>
-      <c r="AC33" s="52"/>
-      <c r="AD33" s="52"/>
-      <c r="AE33" s="52"/>
-      <c r="AF33" s="52"/>
-      <c r="AG33" s="52"/>
-      <c r="AH33" s="52"/>
-      <c r="AI33" s="52"/>
+      <c r="D33" s="58"/>
+      <c r="E33" s="58"/>
+      <c r="F33" s="58"/>
+      <c r="G33" s="58"/>
+      <c r="H33" s="58"/>
+      <c r="I33" s="58"/>
+      <c r="J33" s="58"/>
+      <c r="K33" s="58"/>
+      <c r="L33" s="58"/>
+      <c r="M33" s="58"/>
+      <c r="N33" s="58"/>
+      <c r="O33" s="58"/>
+      <c r="P33" s="58"/>
+      <c r="Q33" s="58"/>
+      <c r="R33" s="58"/>
+      <c r="S33" s="58"/>
+      <c r="T33" s="58"/>
+      <c r="U33" s="58"/>
+      <c r="V33" s="58"/>
+      <c r="W33" s="58"/>
+      <c r="X33" s="58"/>
+      <c r="Y33" s="58"/>
+      <c r="Z33" s="58"/>
+      <c r="AA33" s="58"/>
+      <c r="AB33" s="58"/>
+      <c r="AC33" s="58"/>
+      <c r="AD33" s="58"/>
+      <c r="AE33" s="58"/>
+      <c r="AF33" s="58"/>
+      <c r="AG33" s="58"/>
+      <c r="AH33" s="58"/>
+      <c r="AI33" s="58"/>
       <c r="AJ33" s="7"/>
     </row>
     <row r="34" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="14"/>
-      <c r="C34" s="52"/>
-      <c r="D34" s="52"/>
-      <c r="E34" s="52"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="52"/>
-      <c r="H34" s="52"/>
-      <c r="I34" s="52"/>
-      <c r="J34" s="52"/>
-      <c r="K34" s="52"/>
-      <c r="L34" s="52"/>
-      <c r="M34" s="52"/>
-      <c r="N34" s="52"/>
-      <c r="O34" s="52"/>
-      <c r="P34" s="52"/>
-      <c r="Q34" s="52"/>
-      <c r="R34" s="52"/>
-      <c r="S34" s="52"/>
-      <c r="T34" s="52"/>
-      <c r="U34" s="52"/>
-      <c r="V34" s="52"/>
-      <c r="W34" s="52"/>
-      <c r="X34" s="52"/>
-      <c r="Y34" s="52"/>
-      <c r="Z34" s="52"/>
-      <c r="AA34" s="52"/>
-      <c r="AB34" s="52"/>
-      <c r="AC34" s="52"/>
-      <c r="AD34" s="52"/>
-      <c r="AE34" s="52"/>
-      <c r="AF34" s="52"/>
-      <c r="AG34" s="52"/>
-      <c r="AH34" s="52"/>
-      <c r="AI34" s="52"/>
+      <c r="C34" s="58"/>
+      <c r="D34" s="58"/>
+      <c r="E34" s="58"/>
+      <c r="F34" s="58"/>
+      <c r="G34" s="58"/>
+      <c r="H34" s="58"/>
+      <c r="I34" s="58"/>
+      <c r="J34" s="58"/>
+      <c r="K34" s="58"/>
+      <c r="L34" s="58"/>
+      <c r="M34" s="58"/>
+      <c r="N34" s="58"/>
+      <c r="O34" s="58"/>
+      <c r="P34" s="58"/>
+      <c r="Q34" s="58"/>
+      <c r="R34" s="58"/>
+      <c r="S34" s="58"/>
+      <c r="T34" s="58"/>
+      <c r="U34" s="58"/>
+      <c r="V34" s="58"/>
+      <c r="W34" s="58"/>
+      <c r="X34" s="58"/>
+      <c r="Y34" s="58"/>
+      <c r="Z34" s="58"/>
+      <c r="AA34" s="58"/>
+      <c r="AB34" s="58"/>
+      <c r="AC34" s="58"/>
+      <c r="AD34" s="58"/>
+      <c r="AE34" s="58"/>
+      <c r="AF34" s="58"/>
+      <c r="AG34" s="58"/>
+      <c r="AH34" s="58"/>
+      <c r="AI34" s="58"/>
       <c r="AJ34" s="7"/>
     </row>
     <row r="35" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="14"/>
-      <c r="C35" s="52"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="52"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="52"/>
-      <c r="H35" s="52"/>
-      <c r="I35" s="52"/>
-      <c r="J35" s="52"/>
-      <c r="K35" s="52"/>
-      <c r="L35" s="52"/>
-      <c r="M35" s="52"/>
-      <c r="N35" s="52"/>
-      <c r="O35" s="52"/>
-      <c r="P35" s="52"/>
-      <c r="Q35" s="52"/>
-      <c r="R35" s="52"/>
-      <c r="S35" s="52"/>
-      <c r="T35" s="52"/>
-      <c r="U35" s="52"/>
-      <c r="V35" s="52"/>
-      <c r="W35" s="52"/>
-      <c r="X35" s="52"/>
-      <c r="Y35" s="52"/>
-      <c r="Z35" s="52"/>
-      <c r="AA35" s="52"/>
-      <c r="AB35" s="52"/>
-      <c r="AC35" s="52"/>
-      <c r="AD35" s="52"/>
-      <c r="AE35" s="52"/>
-      <c r="AF35" s="52"/>
-      <c r="AG35" s="52"/>
-      <c r="AH35" s="52"/>
-      <c r="AI35" s="52"/>
+      <c r="C35" s="58"/>
+      <c r="D35" s="58"/>
+      <c r="E35" s="58"/>
+      <c r="F35" s="58"/>
+      <c r="G35" s="58"/>
+      <c r="H35" s="58"/>
+      <c r="I35" s="58"/>
+      <c r="J35" s="58"/>
+      <c r="K35" s="58"/>
+      <c r="L35" s="58"/>
+      <c r="M35" s="58"/>
+      <c r="N35" s="58"/>
+      <c r="O35" s="58"/>
+      <c r="P35" s="58"/>
+      <c r="Q35" s="58"/>
+      <c r="R35" s="58"/>
+      <c r="S35" s="58"/>
+      <c r="T35" s="58"/>
+      <c r="U35" s="58"/>
+      <c r="V35" s="58"/>
+      <c r="W35" s="58"/>
+      <c r="X35" s="58"/>
+      <c r="Y35" s="58"/>
+      <c r="Z35" s="58"/>
+      <c r="AA35" s="58"/>
+      <c r="AB35" s="58"/>
+      <c r="AC35" s="58"/>
+      <c r="AD35" s="58"/>
+      <c r="AE35" s="58"/>
+      <c r="AF35" s="58"/>
+      <c r="AG35" s="58"/>
+      <c r="AH35" s="58"/>
+      <c r="AI35" s="58"/>
       <c r="AJ35" s="7"/>
     </row>
     <row r="36" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="14"/>
-      <c r="C36" s="52"/>
-      <c r="D36" s="52"/>
-      <c r="E36" s="52"/>
-      <c r="F36" s="52"/>
-      <c r="G36" s="52"/>
-      <c r="H36" s="52"/>
-      <c r="I36" s="52"/>
-      <c r="J36" s="52"/>
-      <c r="K36" s="52"/>
-      <c r="L36" s="52"/>
-      <c r="M36" s="52"/>
-      <c r="N36" s="52"/>
-      <c r="O36" s="52"/>
-      <c r="P36" s="52"/>
-      <c r="Q36" s="52"/>
-      <c r="R36" s="52"/>
-      <c r="S36" s="52"/>
-      <c r="T36" s="52"/>
-      <c r="U36" s="52"/>
-      <c r="V36" s="52"/>
-      <c r="W36" s="52"/>
-      <c r="X36" s="52"/>
-      <c r="Y36" s="52"/>
-      <c r="Z36" s="52"/>
-      <c r="AA36" s="52"/>
-      <c r="AB36" s="52"/>
-      <c r="AC36" s="52"/>
-      <c r="AD36" s="52"/>
-      <c r="AE36" s="52"/>
-      <c r="AF36" s="52"/>
-      <c r="AG36" s="52"/>
-      <c r="AH36" s="52"/>
-      <c r="AI36" s="52"/>
+      <c r="C36" s="58"/>
+      <c r="D36" s="58"/>
+      <c r="E36" s="58"/>
+      <c r="F36" s="58"/>
+      <c r="G36" s="58"/>
+      <c r="H36" s="58"/>
+      <c r="I36" s="58"/>
+      <c r="J36" s="58"/>
+      <c r="K36" s="58"/>
+      <c r="L36" s="58"/>
+      <c r="M36" s="58"/>
+      <c r="N36" s="58"/>
+      <c r="O36" s="58"/>
+      <c r="P36" s="58"/>
+      <c r="Q36" s="58"/>
+      <c r="R36" s="58"/>
+      <c r="S36" s="58"/>
+      <c r="T36" s="58"/>
+      <c r="U36" s="58"/>
+      <c r="V36" s="58"/>
+      <c r="W36" s="58"/>
+      <c r="X36" s="58"/>
+      <c r="Y36" s="58"/>
+      <c r="Z36" s="58"/>
+      <c r="AA36" s="58"/>
+      <c r="AB36" s="58"/>
+      <c r="AC36" s="58"/>
+      <c r="AD36" s="58"/>
+      <c r="AE36" s="58"/>
+      <c r="AF36" s="58"/>
+      <c r="AG36" s="58"/>
+      <c r="AH36" s="58"/>
+      <c r="AI36" s="58"/>
       <c r="AJ36" s="7"/>
     </row>
     <row r="37" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="14"/>
-      <c r="C37" s="52"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="52"/>
-      <c r="F37" s="52"/>
-      <c r="G37" s="52"/>
-      <c r="H37" s="52"/>
-      <c r="I37" s="52"/>
-      <c r="J37" s="52"/>
-      <c r="K37" s="52"/>
-      <c r="L37" s="52"/>
-      <c r="M37" s="52"/>
-      <c r="N37" s="52"/>
-      <c r="O37" s="52"/>
-      <c r="P37" s="52"/>
-      <c r="Q37" s="52"/>
-      <c r="R37" s="52"/>
-      <c r="S37" s="52"/>
-      <c r="T37" s="52"/>
-      <c r="U37" s="52"/>
-      <c r="V37" s="52"/>
-      <c r="W37" s="52"/>
-      <c r="X37" s="52"/>
-      <c r="Y37" s="52"/>
-      <c r="Z37" s="52"/>
-      <c r="AA37" s="52"/>
-      <c r="AB37" s="52"/>
-      <c r="AC37" s="52"/>
-      <c r="AD37" s="52"/>
-      <c r="AE37" s="52"/>
-      <c r="AF37" s="52"/>
-      <c r="AG37" s="52"/>
-      <c r="AH37" s="52"/>
-      <c r="AI37" s="52"/>
+      <c r="C37" s="58"/>
+      <c r="D37" s="58"/>
+      <c r="E37" s="58"/>
+      <c r="F37" s="58"/>
+      <c r="G37" s="58"/>
+      <c r="H37" s="58"/>
+      <c r="I37" s="58"/>
+      <c r="J37" s="58"/>
+      <c r="K37" s="58"/>
+      <c r="L37" s="58"/>
+      <c r="M37" s="58"/>
+      <c r="N37" s="58"/>
+      <c r="O37" s="58"/>
+      <c r="P37" s="58"/>
+      <c r="Q37" s="58"/>
+      <c r="R37" s="58"/>
+      <c r="S37" s="58"/>
+      <c r="T37" s="58"/>
+      <c r="U37" s="58"/>
+      <c r="V37" s="58"/>
+      <c r="W37" s="58"/>
+      <c r="X37" s="58"/>
+      <c r="Y37" s="58"/>
+      <c r="Z37" s="58"/>
+      <c r="AA37" s="58"/>
+      <c r="AB37" s="58"/>
+      <c r="AC37" s="58"/>
+      <c r="AD37" s="58"/>
+      <c r="AE37" s="58"/>
+      <c r="AF37" s="58"/>
+      <c r="AG37" s="58"/>
+      <c r="AH37" s="58"/>
+      <c r="AI37" s="58"/>
       <c r="AJ37" s="7"/>
     </row>
     <row r="38" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="14"/>
-      <c r="C38" s="52"/>
-      <c r="D38" s="52"/>
-      <c r="E38" s="52"/>
-      <c r="F38" s="52"/>
-      <c r="G38" s="52"/>
-      <c r="H38" s="52"/>
-      <c r="I38" s="52"/>
-      <c r="J38" s="52"/>
-      <c r="K38" s="52"/>
-      <c r="L38" s="52"/>
-      <c r="M38" s="52"/>
-      <c r="N38" s="52"/>
-      <c r="O38" s="52"/>
-      <c r="P38" s="52"/>
-      <c r="Q38" s="52"/>
-      <c r="R38" s="52"/>
-      <c r="S38" s="52"/>
-      <c r="T38" s="52"/>
-      <c r="U38" s="52"/>
-      <c r="V38" s="52"/>
-      <c r="W38" s="52"/>
-      <c r="X38" s="52"/>
-      <c r="Y38" s="52"/>
-      <c r="Z38" s="52"/>
-      <c r="AA38" s="52"/>
-      <c r="AB38" s="52"/>
-      <c r="AC38" s="52"/>
-      <c r="AD38" s="52"/>
-      <c r="AE38" s="52"/>
-      <c r="AF38" s="52"/>
-      <c r="AG38" s="52"/>
-      <c r="AH38" s="52"/>
-      <c r="AI38" s="52"/>
+      <c r="C38" s="58"/>
+      <c r="D38" s="58"/>
+      <c r="E38" s="58"/>
+      <c r="F38" s="58"/>
+      <c r="G38" s="58"/>
+      <c r="H38" s="58"/>
+      <c r="I38" s="58"/>
+      <c r="J38" s="58"/>
+      <c r="K38" s="58"/>
+      <c r="L38" s="58"/>
+      <c r="M38" s="58"/>
+      <c r="N38" s="58"/>
+      <c r="O38" s="58"/>
+      <c r="P38" s="58"/>
+      <c r="Q38" s="58"/>
+      <c r="R38" s="58"/>
+      <c r="S38" s="58"/>
+      <c r="T38" s="58"/>
+      <c r="U38" s="58"/>
+      <c r="V38" s="58"/>
+      <c r="W38" s="58"/>
+      <c r="X38" s="58"/>
+      <c r="Y38" s="58"/>
+      <c r="Z38" s="58"/>
+      <c r="AA38" s="58"/>
+      <c r="AB38" s="58"/>
+      <c r="AC38" s="58"/>
+      <c r="AD38" s="58"/>
+      <c r="AE38" s="58"/>
+      <c r="AF38" s="58"/>
+      <c r="AG38" s="58"/>
+      <c r="AH38" s="58"/>
+      <c r="AI38" s="58"/>
       <c r="AJ38" s="7"/>
     </row>
     <row r="39" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="14"/>
-      <c r="C39" s="52"/>
-      <c r="D39" s="52"/>
-      <c r="E39" s="52"/>
-      <c r="F39" s="52"/>
-      <c r="G39" s="52"/>
-      <c r="H39" s="52"/>
-      <c r="I39" s="52"/>
-      <c r="J39" s="52"/>
-      <c r="K39" s="52"/>
-      <c r="L39" s="52"/>
-      <c r="M39" s="52"/>
-      <c r="N39" s="52"/>
-      <c r="O39" s="52"/>
-      <c r="P39" s="52"/>
-      <c r="Q39" s="52"/>
-      <c r="R39" s="52"/>
-      <c r="S39" s="52"/>
-      <c r="T39" s="52"/>
-      <c r="U39" s="52"/>
-      <c r="V39" s="52"/>
-      <c r="W39" s="52"/>
-      <c r="X39" s="52"/>
-      <c r="Y39" s="52"/>
-      <c r="Z39" s="52"/>
-      <c r="AA39" s="52"/>
-      <c r="AB39" s="52"/>
-      <c r="AC39" s="52"/>
-      <c r="AD39" s="52"/>
-      <c r="AE39" s="52"/>
-      <c r="AF39" s="52"/>
-      <c r="AG39" s="52"/>
-      <c r="AH39" s="52"/>
-      <c r="AI39" s="52"/>
+      <c r="C39" s="58"/>
+      <c r="D39" s="58"/>
+      <c r="E39" s="58"/>
+      <c r="F39" s="58"/>
+      <c r="G39" s="58"/>
+      <c r="H39" s="58"/>
+      <c r="I39" s="58"/>
+      <c r="J39" s="58"/>
+      <c r="K39" s="58"/>
+      <c r="L39" s="58"/>
+      <c r="M39" s="58"/>
+      <c r="N39" s="58"/>
+      <c r="O39" s="58"/>
+      <c r="P39" s="58"/>
+      <c r="Q39" s="58"/>
+      <c r="R39" s="58"/>
+      <c r="S39" s="58"/>
+      <c r="T39" s="58"/>
+      <c r="U39" s="58"/>
+      <c r="V39" s="58"/>
+      <c r="W39" s="58"/>
+      <c r="X39" s="58"/>
+      <c r="Y39" s="58"/>
+      <c r="Z39" s="58"/>
+      <c r="AA39" s="58"/>
+      <c r="AB39" s="58"/>
+      <c r="AC39" s="58"/>
+      <c r="AD39" s="58"/>
+      <c r="AE39" s="58"/>
+      <c r="AF39" s="58"/>
+      <c r="AG39" s="58"/>
+      <c r="AH39" s="58"/>
+      <c r="AI39" s="58"/>
       <c r="AJ39" s="7"/>
     </row>
     <row r="40" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="14"/>
-      <c r="C40" s="52"/>
-      <c r="D40" s="52"/>
-      <c r="E40" s="52"/>
-      <c r="F40" s="52"/>
-      <c r="G40" s="52"/>
-      <c r="H40" s="52"/>
-      <c r="I40" s="52"/>
-      <c r="J40" s="52"/>
-      <c r="K40" s="52"/>
-      <c r="L40" s="52"/>
-      <c r="M40" s="52"/>
-      <c r="N40" s="52"/>
-      <c r="O40" s="52"/>
-      <c r="P40" s="52"/>
-      <c r="Q40" s="52"/>
-      <c r="R40" s="52"/>
-      <c r="S40" s="52"/>
-      <c r="T40" s="52"/>
-      <c r="U40" s="52"/>
-      <c r="V40" s="52"/>
-      <c r="W40" s="52"/>
-      <c r="X40" s="52"/>
-      <c r="Y40" s="52"/>
-      <c r="Z40" s="52"/>
-      <c r="AA40" s="52"/>
-      <c r="AB40" s="52"/>
-      <c r="AC40" s="52"/>
-      <c r="AD40" s="52"/>
-      <c r="AE40" s="52"/>
-      <c r="AF40" s="52"/>
-      <c r="AG40" s="52"/>
-      <c r="AH40" s="52"/>
-      <c r="AI40" s="52"/>
+      <c r="C40" s="58"/>
+      <c r="D40" s="58"/>
+      <c r="E40" s="58"/>
+      <c r="F40" s="58"/>
+      <c r="G40" s="58"/>
+      <c r="H40" s="58"/>
+      <c r="I40" s="58"/>
+      <c r="J40" s="58"/>
+      <c r="K40" s="58"/>
+      <c r="L40" s="58"/>
+      <c r="M40" s="58"/>
+      <c r="N40" s="58"/>
+      <c r="O40" s="58"/>
+      <c r="P40" s="58"/>
+      <c r="Q40" s="58"/>
+      <c r="R40" s="58"/>
+      <c r="S40" s="58"/>
+      <c r="T40" s="58"/>
+      <c r="U40" s="58"/>
+      <c r="V40" s="58"/>
+      <c r="W40" s="58"/>
+      <c r="X40" s="58"/>
+      <c r="Y40" s="58"/>
+      <c r="Z40" s="58"/>
+      <c r="AA40" s="58"/>
+      <c r="AB40" s="58"/>
+      <c r="AC40" s="58"/>
+      <c r="AD40" s="58"/>
+      <c r="AE40" s="58"/>
+      <c r="AF40" s="58"/>
+      <c r="AG40" s="58"/>
+      <c r="AH40" s="58"/>
+      <c r="AI40" s="58"/>
       <c r="AJ40" s="7"/>
     </row>
     <row r="41" spans="2:36" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="14"/>
-      <c r="C41" s="52"/>
-      <c r="D41" s="52"/>
-      <c r="E41" s="52"/>
-      <c r="F41" s="52"/>
-      <c r="G41" s="52"/>
-      <c r="H41" s="52"/>
-      <c r="I41" s="52"/>
-      <c r="J41" s="52"/>
-      <c r="K41" s="52"/>
-      <c r="L41" s="52"/>
-      <c r="M41" s="52"/>
-      <c r="N41" s="52"/>
-      <c r="O41" s="52"/>
-      <c r="P41" s="52"/>
-      <c r="Q41" s="52"/>
-      <c r="R41" s="52"/>
-      <c r="S41" s="52"/>
-      <c r="T41" s="52"/>
-      <c r="U41" s="52"/>
-      <c r="V41" s="52"/>
-      <c r="W41" s="52"/>
-      <c r="X41" s="52"/>
-      <c r="Y41" s="52"/>
-      <c r="Z41" s="52"/>
-      <c r="AA41" s="52"/>
-      <c r="AB41" s="52"/>
-      <c r="AC41" s="52"/>
-      <c r="AD41" s="52"/>
-      <c r="AE41" s="52"/>
-      <c r="AF41" s="52"/>
-      <c r="AG41" s="52"/>
-      <c r="AH41" s="52"/>
-      <c r="AI41" s="52"/>
+      <c r="C41" s="58"/>
+      <c r="D41" s="58"/>
+      <c r="E41" s="58"/>
+      <c r="F41" s="58"/>
+      <c r="G41" s="58"/>
+      <c r="H41" s="58"/>
+      <c r="I41" s="58"/>
+      <c r="J41" s="58"/>
+      <c r="K41" s="58"/>
+      <c r="L41" s="58"/>
+      <c r="M41" s="58"/>
+      <c r="N41" s="58"/>
+      <c r="O41" s="58"/>
+      <c r="P41" s="58"/>
+      <c r="Q41" s="58"/>
+      <c r="R41" s="58"/>
+      <c r="S41" s="58"/>
+      <c r="T41" s="58"/>
+      <c r="U41" s="58"/>
+      <c r="V41" s="58"/>
+      <c r="W41" s="58"/>
+      <c r="X41" s="58"/>
+      <c r="Y41" s="58"/>
+      <c r="Z41" s="58"/>
+      <c r="AA41" s="58"/>
+      <c r="AB41" s="58"/>
+      <c r="AC41" s="58"/>
+      <c r="AD41" s="58"/>
+      <c r="AE41" s="58"/>
+      <c r="AF41" s="58"/>
+      <c r="AG41" s="58"/>
+      <c r="AH41" s="58"/>
+      <c r="AI41" s="58"/>
       <c r="AJ41" s="7"/>
     </row>
     <row r="42" spans="2:36" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -3475,218 +3344,218 @@
     </row>
     <row r="43" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B43" s="14"/>
-      <c r="C43" s="53" t="s">
+      <c r="C43" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="D43" s="53"/>
-      <c r="E43" s="53"/>
-      <c r="F43" s="53"/>
-      <c r="G43" s="53"/>
+      <c r="D43" s="59"/>
+      <c r="E43" s="59"/>
+      <c r="F43" s="59"/>
+      <c r="G43" s="59"/>
       <c r="AJ43" s="7"/>
     </row>
     <row r="44" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B44" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C44" s="93" t="s">
+      <c r="C44" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="D44" s="93"/>
-      <c r="E44" s="93"/>
-      <c r="F44" s="93"/>
-      <c r="G44" s="93"/>
-      <c r="H44" s="93"/>
-      <c r="I44" s="93"/>
-      <c r="J44" s="93"/>
-      <c r="K44" s="93"/>
-      <c r="L44" s="93"/>
-      <c r="M44" s="93"/>
-      <c r="N44" s="93"/>
-      <c r="O44" s="93"/>
-      <c r="P44" s="93"/>
-      <c r="Q44" s="93"/>
-      <c r="R44" s="93"/>
-      <c r="S44" s="93"/>
-      <c r="T44" s="93"/>
-      <c r="U44" s="93"/>
-      <c r="V44" s="93"/>
-      <c r="W44" s="93"/>
-      <c r="X44" s="93"/>
-      <c r="Y44" s="93"/>
-      <c r="Z44" s="93"/>
-      <c r="AA44" s="93"/>
-      <c r="AB44" s="93"/>
-      <c r="AC44" s="93"/>
-      <c r="AD44" s="93"/>
-      <c r="AE44" s="93"/>
-      <c r="AF44" s="93"/>
-      <c r="AG44" s="93"/>
-      <c r="AH44" s="93"/>
-      <c r="AI44" s="93"/>
+      <c r="D44" s="69"/>
+      <c r="E44" s="69"/>
+      <c r="F44" s="69"/>
+      <c r="G44" s="69"/>
+      <c r="H44" s="69"/>
+      <c r="I44" s="69"/>
+      <c r="J44" s="69"/>
+      <c r="K44" s="69"/>
+      <c r="L44" s="69"/>
+      <c r="M44" s="69"/>
+      <c r="N44" s="69"/>
+      <c r="O44" s="69"/>
+      <c r="P44" s="69"/>
+      <c r="Q44" s="69"/>
+      <c r="R44" s="69"/>
+      <c r="S44" s="69"/>
+      <c r="T44" s="69"/>
+      <c r="U44" s="69"/>
+      <c r="V44" s="69"/>
+      <c r="W44" s="69"/>
+      <c r="X44" s="69"/>
+      <c r="Y44" s="69"/>
+      <c r="Z44" s="69"/>
+      <c r="AA44" s="69"/>
+      <c r="AB44" s="69"/>
+      <c r="AC44" s="69"/>
+      <c r="AD44" s="69"/>
+      <c r="AE44" s="69"/>
+      <c r="AF44" s="69"/>
+      <c r="AG44" s="69"/>
+      <c r="AH44" s="69"/>
+      <c r="AI44" s="69"/>
       <c r="AJ44" s="7"/>
     </row>
     <row r="45" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B45" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C45" s="93" t="s">
+      <c r="C45" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="D45" s="93"/>
-      <c r="E45" s="93"/>
-      <c r="F45" s="93"/>
-      <c r="G45" s="93"/>
-      <c r="H45" s="93"/>
-      <c r="I45" s="93"/>
-      <c r="J45" s="93"/>
-      <c r="K45" s="93"/>
-      <c r="L45" s="93"/>
-      <c r="M45" s="93"/>
-      <c r="N45" s="93"/>
-      <c r="O45" s="93"/>
-      <c r="P45" s="93"/>
-      <c r="Q45" s="93"/>
-      <c r="R45" s="93"/>
-      <c r="S45" s="93"/>
-      <c r="T45" s="93"/>
-      <c r="U45" s="93"/>
-      <c r="V45" s="93"/>
-      <c r="W45" s="93"/>
-      <c r="X45" s="93"/>
-      <c r="Y45" s="93"/>
-      <c r="Z45" s="93"/>
-      <c r="AA45" s="93"/>
-      <c r="AB45" s="93"/>
-      <c r="AC45" s="93"/>
-      <c r="AD45" s="93"/>
-      <c r="AE45" s="93"/>
-      <c r="AF45" s="93"/>
-      <c r="AG45" s="93"/>
-      <c r="AH45" s="93"/>
-      <c r="AI45" s="93"/>
+      <c r="D45" s="69"/>
+      <c r="E45" s="69"/>
+      <c r="F45" s="69"/>
+      <c r="G45" s="69"/>
+      <c r="H45" s="69"/>
+      <c r="I45" s="69"/>
+      <c r="J45" s="69"/>
+      <c r="K45" s="69"/>
+      <c r="L45" s="69"/>
+      <c r="M45" s="69"/>
+      <c r="N45" s="69"/>
+      <c r="O45" s="69"/>
+      <c r="P45" s="69"/>
+      <c r="Q45" s="69"/>
+      <c r="R45" s="69"/>
+      <c r="S45" s="69"/>
+      <c r="T45" s="69"/>
+      <c r="U45" s="69"/>
+      <c r="V45" s="69"/>
+      <c r="W45" s="69"/>
+      <c r="X45" s="69"/>
+      <c r="Y45" s="69"/>
+      <c r="Z45" s="69"/>
+      <c r="AA45" s="69"/>
+      <c r="AB45" s="69"/>
+      <c r="AC45" s="69"/>
+      <c r="AD45" s="69"/>
+      <c r="AE45" s="69"/>
+      <c r="AF45" s="69"/>
+      <c r="AG45" s="69"/>
+      <c r="AH45" s="69"/>
+      <c r="AI45" s="69"/>
       <c r="AJ45" s="7"/>
     </row>
     <row r="46" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B46" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C46" s="93" t="s">
+      <c r="C46" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="D46" s="93"/>
-      <c r="E46" s="93"/>
-      <c r="F46" s="93"/>
-      <c r="G46" s="93"/>
-      <c r="H46" s="93"/>
-      <c r="I46" s="93"/>
-      <c r="J46" s="93"/>
-      <c r="K46" s="93"/>
-      <c r="L46" s="93"/>
-      <c r="M46" s="93"/>
-      <c r="N46" s="93"/>
-      <c r="O46" s="93"/>
-      <c r="P46" s="93"/>
-      <c r="Q46" s="93"/>
-      <c r="R46" s="93"/>
-      <c r="S46" s="93"/>
-      <c r="T46" s="93"/>
-      <c r="U46" s="93"/>
-      <c r="V46" s="93"/>
-      <c r="W46" s="93"/>
-      <c r="X46" s="93"/>
-      <c r="Y46" s="93"/>
-      <c r="Z46" s="93"/>
-      <c r="AA46" s="93"/>
-      <c r="AB46" s="93"/>
-      <c r="AC46" s="93"/>
-      <c r="AD46" s="93"/>
-      <c r="AE46" s="93"/>
-      <c r="AF46" s="93"/>
-      <c r="AG46" s="93"/>
-      <c r="AH46" s="93"/>
-      <c r="AI46" s="93"/>
+      <c r="D46" s="69"/>
+      <c r="E46" s="69"/>
+      <c r="F46" s="69"/>
+      <c r="G46" s="69"/>
+      <c r="H46" s="69"/>
+      <c r="I46" s="69"/>
+      <c r="J46" s="69"/>
+      <c r="K46" s="69"/>
+      <c r="L46" s="69"/>
+      <c r="M46" s="69"/>
+      <c r="N46" s="69"/>
+      <c r="O46" s="69"/>
+      <c r="P46" s="69"/>
+      <c r="Q46" s="69"/>
+      <c r="R46" s="69"/>
+      <c r="S46" s="69"/>
+      <c r="T46" s="69"/>
+      <c r="U46" s="69"/>
+      <c r="V46" s="69"/>
+      <c r="W46" s="69"/>
+      <c r="X46" s="69"/>
+      <c r="Y46" s="69"/>
+      <c r="Z46" s="69"/>
+      <c r="AA46" s="69"/>
+      <c r="AB46" s="69"/>
+      <c r="AC46" s="69"/>
+      <c r="AD46" s="69"/>
+      <c r="AE46" s="69"/>
+      <c r="AF46" s="69"/>
+      <c r="AG46" s="69"/>
+      <c r="AH46" s="69"/>
+      <c r="AI46" s="69"/>
       <c r="AJ46" s="7"/>
     </row>
     <row r="47" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B47" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C47" s="93" t="s">
+      <c r="C47" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="D47" s="93"/>
-      <c r="E47" s="93"/>
-      <c r="F47" s="93"/>
-      <c r="G47" s="93"/>
-      <c r="H47" s="93"/>
-      <c r="I47" s="93"/>
-      <c r="J47" s="93"/>
-      <c r="K47" s="93"/>
-      <c r="L47" s="93"/>
-      <c r="M47" s="93"/>
-      <c r="N47" s="93"/>
-      <c r="O47" s="93"/>
-      <c r="P47" s="93"/>
-      <c r="Q47" s="93"/>
-      <c r="R47" s="93"/>
-      <c r="S47" s="93"/>
-      <c r="T47" s="93"/>
-      <c r="U47" s="93"/>
-      <c r="V47" s="93"/>
-      <c r="W47" s="93"/>
-      <c r="X47" s="93"/>
-      <c r="Y47" s="93"/>
-      <c r="Z47" s="93"/>
-      <c r="AA47" s="93"/>
-      <c r="AB47" s="93"/>
-      <c r="AC47" s="93"/>
-      <c r="AD47" s="93"/>
-      <c r="AE47" s="93"/>
-      <c r="AF47" s="93"/>
-      <c r="AG47" s="93"/>
-      <c r="AH47" s="93"/>
-      <c r="AI47" s="93"/>
+      <c r="D47" s="69"/>
+      <c r="E47" s="69"/>
+      <c r="F47" s="69"/>
+      <c r="G47" s="69"/>
+      <c r="H47" s="69"/>
+      <c r="I47" s="69"/>
+      <c r="J47" s="69"/>
+      <c r="K47" s="69"/>
+      <c r="L47" s="69"/>
+      <c r="M47" s="69"/>
+      <c r="N47" s="69"/>
+      <c r="O47" s="69"/>
+      <c r="P47" s="69"/>
+      <c r="Q47" s="69"/>
+      <c r="R47" s="69"/>
+      <c r="S47" s="69"/>
+      <c r="T47" s="69"/>
+      <c r="U47" s="69"/>
+      <c r="V47" s="69"/>
+      <c r="W47" s="69"/>
+      <c r="X47" s="69"/>
+      <c r="Y47" s="69"/>
+      <c r="Z47" s="69"/>
+      <c r="AA47" s="69"/>
+      <c r="AB47" s="69"/>
+      <c r="AC47" s="69"/>
+      <c r="AD47" s="69"/>
+      <c r="AE47" s="69"/>
+      <c r="AF47" s="69"/>
+      <c r="AG47" s="69"/>
+      <c r="AH47" s="69"/>
+      <c r="AI47" s="69"/>
       <c r="AJ47" s="7"/>
     </row>
     <row r="48" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B48" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="93" t="s">
+      <c r="C48" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="D48" s="93"/>
-      <c r="E48" s="93"/>
-      <c r="F48" s="93"/>
-      <c r="G48" s="93"/>
-      <c r="H48" s="93"/>
-      <c r="I48" s="93"/>
-      <c r="J48" s="93"/>
-      <c r="K48" s="93"/>
-      <c r="L48" s="93"/>
-      <c r="M48" s="93"/>
-      <c r="N48" s="93"/>
-      <c r="O48" s="93"/>
-      <c r="P48" s="93"/>
-      <c r="Q48" s="93"/>
-      <c r="R48" s="93"/>
-      <c r="S48" s="93"/>
-      <c r="T48" s="93"/>
-      <c r="U48" s="93"/>
-      <c r="V48" s="93"/>
-      <c r="W48" s="93"/>
-      <c r="X48" s="93"/>
-      <c r="Y48" s="93"/>
-      <c r="Z48" s="93"/>
-      <c r="AA48" s="93"/>
-      <c r="AB48" s="93"/>
-      <c r="AC48" s="93"/>
-      <c r="AD48" s="93"/>
-      <c r="AE48" s="93"/>
-      <c r="AF48" s="93"/>
-      <c r="AG48" s="93"/>
-      <c r="AH48" s="93"/>
-      <c r="AI48" s="93"/>
+      <c r="D48" s="69"/>
+      <c r="E48" s="69"/>
+      <c r="F48" s="69"/>
+      <c r="G48" s="69"/>
+      <c r="H48" s="69"/>
+      <c r="I48" s="69"/>
+      <c r="J48" s="69"/>
+      <c r="K48" s="69"/>
+      <c r="L48" s="69"/>
+      <c r="M48" s="69"/>
+      <c r="N48" s="69"/>
+      <c r="O48" s="69"/>
+      <c r="P48" s="69"/>
+      <c r="Q48" s="69"/>
+      <c r="R48" s="69"/>
+      <c r="S48" s="69"/>
+      <c r="T48" s="69"/>
+      <c r="U48" s="69"/>
+      <c r="V48" s="69"/>
+      <c r="W48" s="69"/>
+      <c r="X48" s="69"/>
+      <c r="Y48" s="69"/>
+      <c r="Z48" s="69"/>
+      <c r="AA48" s="69"/>
+      <c r="AB48" s="69"/>
+      <c r="AC48" s="69"/>
+      <c r="AD48" s="69"/>
+      <c r="AE48" s="69"/>
+      <c r="AF48" s="69"/>
+      <c r="AG48" s="69"/>
+      <c r="AH48" s="69"/>
+      <c r="AI48" s="69"/>
       <c r="AJ48" s="7"/>
     </row>
     <row r="49" spans="2:36" ht="7" customHeight="1" x14ac:dyDescent="0.35">
@@ -3704,94 +3573,94 @@
     </row>
     <row r="52" spans="2:36" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B52" s="14"/>
-      <c r="H52" s="54" t="s">
+      <c r="H52" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="I52" s="55"/>
-      <c r="J52" s="55"/>
-      <c r="K52" s="55"/>
-      <c r="L52" s="55"/>
-      <c r="M52" s="55"/>
-      <c r="N52" s="55"/>
-      <c r="O52" s="55"/>
-      <c r="P52" s="55"/>
-      <c r="Q52" s="55"/>
-      <c r="R52" s="55"/>
-      <c r="S52" s="55"/>
-      <c r="T52" s="55"/>
-      <c r="U52" s="55"/>
-      <c r="V52" s="55"/>
-      <c r="W52" s="55"/>
-      <c r="X52" s="55"/>
-      <c r="Y52" s="55"/>
-      <c r="Z52" s="55"/>
-      <c r="AA52" s="55"/>
-      <c r="AB52" s="55"/>
-      <c r="AC52" s="55"/>
-      <c r="AD52" s="55"/>
+      <c r="I52" s="61"/>
+      <c r="J52" s="61"/>
+      <c r="K52" s="61"/>
+      <c r="L52" s="61"/>
+      <c r="M52" s="61"/>
+      <c r="N52" s="61"/>
+      <c r="O52" s="61"/>
+      <c r="P52" s="61"/>
+      <c r="Q52" s="61"/>
+      <c r="R52" s="61"/>
+      <c r="S52" s="61"/>
+      <c r="T52" s="61"/>
+      <c r="U52" s="61"/>
+      <c r="V52" s="61"/>
+      <c r="W52" s="61"/>
+      <c r="X52" s="61"/>
+      <c r="Y52" s="61"/>
+      <c r="Z52" s="61"/>
+      <c r="AA52" s="61"/>
+      <c r="AB52" s="61"/>
+      <c r="AC52" s="61"/>
+      <c r="AD52" s="61"/>
       <c r="AJ52" s="7"/>
     </row>
     <row r="53" spans="2:36" x14ac:dyDescent="0.35">
       <c r="B53" s="14"/>
-      <c r="H53" s="56" t="s">
+      <c r="H53" s="62" t="s">
         <v>36</v>
       </c>
-      <c r="I53" s="56"/>
-      <c r="J53" s="56"/>
-      <c r="K53" s="56"/>
-      <c r="L53" s="56"/>
-      <c r="M53" s="56"/>
-      <c r="N53" s="56"/>
-      <c r="O53" s="56"/>
-      <c r="P53" s="56"/>
-      <c r="Q53" s="56"/>
-      <c r="R53" s="56"/>
-      <c r="S53" s="56"/>
-      <c r="T53" s="56"/>
-      <c r="U53" s="56"/>
-      <c r="V53" s="56"/>
-      <c r="W53" s="56"/>
-      <c r="X53" s="56"/>
-      <c r="Y53" s="56"/>
-      <c r="Z53" s="56"/>
-      <c r="AA53" s="56"/>
-      <c r="AB53" s="56"/>
-      <c r="AC53" s="56"/>
-      <c r="AD53" s="56"/>
+      <c r="I53" s="62"/>
+      <c r="J53" s="62"/>
+      <c r="K53" s="62"/>
+      <c r="L53" s="62"/>
+      <c r="M53" s="62"/>
+      <c r="N53" s="62"/>
+      <c r="O53" s="62"/>
+      <c r="P53" s="62"/>
+      <c r="Q53" s="62"/>
+      <c r="R53" s="62"/>
+      <c r="S53" s="62"/>
+      <c r="T53" s="62"/>
+      <c r="U53" s="62"/>
+      <c r="V53" s="62"/>
+      <c r="W53" s="62"/>
+      <c r="X53" s="62"/>
+      <c r="Y53" s="62"/>
+      <c r="Z53" s="62"/>
+      <c r="AA53" s="62"/>
+      <c r="AB53" s="62"/>
+      <c r="AC53" s="62"/>
+      <c r="AD53" s="62"/>
       <c r="AJ53" s="7"/>
     </row>
     <row r="54" spans="2:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B54" s="14"/>
-      <c r="C54" s="57" t="s">
+      <c r="C54" s="63" t="s">
         <v>37</v>
       </c>
-      <c r="D54" s="57"/>
-      <c r="E54" s="57"/>
-      <c r="F54" s="57"/>
-      <c r="G54" s="57"/>
-      <c r="H54" s="58" t="s">
+      <c r="D54" s="63"/>
+      <c r="E54" s="63"/>
+      <c r="F54" s="63"/>
+      <c r="G54" s="63"/>
+      <c r="H54" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="I54" s="58"/>
-      <c r="J54" s="58"/>
-      <c r="K54" s="58"/>
-      <c r="L54" s="58"/>
-      <c r="M54" s="59" t="s">
+      <c r="I54" s="64"/>
+      <c r="J54" s="64"/>
+      <c r="K54" s="64"/>
+      <c r="L54" s="64"/>
+      <c r="M54" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="N54" s="60"/>
-      <c r="O54" s="60"/>
-      <c r="P54" s="60"/>
-      <c r="Q54" s="60"/>
-      <c r="R54" s="61"/>
-      <c r="S54" s="58" t="s">
+      <c r="N54" s="66"/>
+      <c r="O54" s="66"/>
+      <c r="P54" s="66"/>
+      <c r="Q54" s="66"/>
+      <c r="R54" s="67"/>
+      <c r="S54" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="T54" s="58"/>
-      <c r="U54" s="58"/>
-      <c r="V54" s="58"/>
-      <c r="W54" s="58"/>
-      <c r="X54" s="62"/>
+      <c r="T54" s="64"/>
+      <c r="U54" s="64"/>
+      <c r="V54" s="64"/>
+      <c r="W54" s="64"/>
+      <c r="X54" s="68"/>
       <c r="Y54" s="45"/>
       <c r="Z54" s="45"/>
       <c r="AA54" s="45"/>

</xml_diff>